<commit_message>
refactor(roadmap): loai bo cac hang muc Done va Pending, cap nhat 29 US Active Q4 2026
</commit_message>
<xml_diff>
--- a/thuyttdoc/Roadmap_Website_CMS_Q4_2026.xlsx
+++ b/thuyttdoc/Roadmap_Website_CMS_Q4_2026.xlsx
@@ -52,13 +52,13 @@
     <font>
       <name val="Times New Roman"/>
       <b val="1"/>
-      <color rgb="004338CA"/>
+      <color rgb="000F766E"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Times New Roman"/>
       <b val="1"/>
-      <color rgb="000F766E"/>
+      <color rgb="004338CA"/>
       <sz val="11"/>
     </font>
     <font>
@@ -101,8 +101,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EEF2FF"/>
-        <bgColor rgb="00EEF2FF"/>
+        <fgColor rgb="00CCFBF1"/>
+        <bgColor rgb="00CCFBF1"/>
       </patternFill>
     </fill>
     <fill>
@@ -113,8 +113,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CCFBF1"/>
-        <bgColor rgb="00CCFBF1"/>
+        <fgColor rgb="00EEF2FF"/>
+        <bgColor rgb="00EEF2FF"/>
       </patternFill>
     </fill>
     <fill>
@@ -586,7 +586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J39"/>
+  <dimension ref="A1:J33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -604,14 +604,14 @@
     <row r="1" ht="40" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>PRODUCT ROADMAP — FPT TELECOM | WEBSITE FPT.VN &amp; CMS (QUÝ 4/2026)</t>
+          <t>PRODUCT ROADMAP — FPT TELECOM | WEBSITE FPT.VN &amp; CMS (QUÝ 4/2026 - ACTIVE SCOPE)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mục tiêu: Hoàn thiện nền tảng CMS Core, Tối ưu luồng Mua kèm &amp; Giỏ hàng, Triển khai chiến dịch Campaign NHA/LDP &amp; Dự phòng vận hành linh hoạt (15-20%)</t>
+          <t>Phạm vi thực thi: 29 User Stories Active (Đã loại bỏ các mục Done &amp; Pending) | Quỹ dự phòng vận hành linh hoạt 15 - 20%</t>
         </is>
       </c>
     </row>
@@ -670,17 +670,17 @@
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>US-08</t>
+          <t>US-MENU</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>[CMS]</t>
+          <t>[Web, CMS]</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Nội dung hiển thị Gói bán</t>
+          <t>MENU</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
@@ -690,7 +690,7 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Sprint 19 (01/10 - 15/10)</t>
+          <t>Sprint 20 (16/10 - 31/10)</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -700,17 +700,17 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>DEV In Progress</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>LongNH156</t>
+          <t>ThuyTT104 / SonLN11</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>85%</t>
+          <t>60%</t>
         </is>
       </c>
       <c r="J4" s="6" t="inlineStr">
@@ -722,17 +722,17 @@
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>US-09</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
+          <t>US-12</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>[CMS]</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Cấu hình hiển thị checkout</t>
+          <t>Quản lý trang</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
@@ -747,7 +747,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -774,17 +774,17 @@
     <row r="6" ht="24" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>US-10</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
+          <t>US-13</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>[CMS]</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Phương thức Thanh toán</t>
+          <t>Quản lý section</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -826,17 +826,17 @@
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>US-MENU</t>
+          <t>US-14</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>[Web, CMS]</t>
+          <t>[CMS]</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>MENU</t>
+          <t>Quản lý Block</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
@@ -846,27 +846,27 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Sprint 20 (16/10 - 31/10)</t>
+          <t>Sprint 19 (01/10 - 15/10)</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>DEV In Progress</t>
+          <t>UAT</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>ThuyTT104 / SonLN11</t>
+          <t>LongNH156</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>60%</t>
+          <t>85%</t>
         </is>
       </c>
       <c r="J7" s="6" t="inlineStr">
@@ -878,17 +878,17 @@
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>US-07</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
+          <t>US-15</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>[CMS]</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Quản lý bài viết của tác giả (Quản lý tin tức)</t>
+          <t>Quản lý menu</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Chưa tiếp nhận</t>
+          <t>UAT</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -918,29 +918,29 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>85%</t>
         </is>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>Content / SEO</t>
+          <t>Core Product</t>
         </is>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>US-11</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
+          <t>US-07</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>[CMS]</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Quản lý Badge/Tag</t>
+          <t>Quản lý bài viết của tác giả (Quản lý tin tức)</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -950,7 +950,7 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Sprint 19 (01/10 - 15/10)</t>
+          <t>Sprint 20 (16/10 - 31/10)</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -960,7 +960,7 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -970,247 +970,247 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>85%</t>
+          <t>15%</t>
         </is>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>Core Product</t>
+          <t>Content / SEO</t>
         </is>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>US-12</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>[CMS]</t>
+          <t>US-REPORT2</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>[Web]</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Quản lý trang</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>Tháng 10</t>
+          <t>Report: Ghi nhận thông tin báo cáo phase 2 - quy hoạch bộ báo cáo chuẩn cho ĐKOL</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>Tháng 11</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Sprint 19 (01/10 - 15/10)</t>
+          <t>Sprint 21 (01/11 - 15/11)</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>DEV In Progress</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>LongNH156</t>
+          <t>ThuyTT104</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>85%</t>
+          <t>55%</t>
         </is>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>Core Product</t>
+          <t>Analytics / Partner</t>
         </is>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>US-13</t>
+          <t>US-QC</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>[CMS]</t>
+          <t>[CMS, Web]</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Quản lý section</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>Tháng 10</t>
+          <t>Quản lý quảng cáo</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>Tháng 11</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Sprint 19 (01/10 - 15/10)</t>
+          <t>Sprint 21 (01/11 - 15/11)</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>Đang phân tích/Document</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>LongNH156</t>
+          <t>SonLN11</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>85%</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>Core Product</t>
+          <t>Marketing</t>
         </is>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>US-14</t>
+          <t>US-LDPLOCAL</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>[CMS]</t>
+          <t>[Web, CMS]</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Quản lý Block</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>Tháng 10</t>
+          <t>CMS config LDP local - QT tạo LDP Local - SEO - Schame</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>Tháng 11</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Sprint 19 (01/10 - 15/10)</t>
+          <t>Sprint 21 (01/11 - 15/11)</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>Đang phân tích/Document</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>LongNH156</t>
+          <t>SonLN11</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>85%</t>
+          <t>35%</t>
         </is>
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>Core Product</t>
+          <t>SEO / Growth</t>
         </is>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>US-15</t>
+          <t>US-BREADCRUMBS</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>[CMS]</t>
+          <t>[CMS, Web]</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Quản lý menu</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>Tháng 10</t>
+          <t>Quản lý Breadcrums trên trang/ landing Page</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>Tháng 11</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Sprint 20 (16/10 - 31/10)</t>
+          <t>Sprint 22 (16/11 - 30/11)</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>Đang phân tích/Document</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>LongNH156</t>
+          <t>SonLN11</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>85%</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>Core Product</t>
+          <t>SEO / Navigation</t>
         </is>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>US-16</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>[CMS]</t>
+          <t>US-CHARM</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>[Web]</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Quản lý banner</t>
-        </is>
-      </c>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t>Tháng 10</t>
+          <t>Luồng bán kèm PK (charm) trên website fpt.vn</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>Tháng 11</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Sprint 20 (16/10 - 31/10)</t>
+          <t>Sprint 21 (01/11 - 15/11)</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -1220,49 +1220,49 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>Đã tiếp nhận yêu cầu</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>LongNH156</t>
+          <t>ThuyTT104</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>85%</t>
+          <t>40%</t>
         </is>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Commerce Feature</t>
         </is>
       </c>
     </row>
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>US-17</t>
+          <t>US-18</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>[CMS]</t>
+          <t>[CMS, Web]</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Quản lý popup</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>Tháng 10</t>
+          <t>Quản lý FAQ</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>Tháng 11</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Sprint 20 (16/10 - 31/10)</t>
+          <t>Sprint 22 (16/11 - 30/11)</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -1272,39 +1272,39 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>Đang phân tích/Document</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>LongNH156</t>
+          <t>SonLN11</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>85%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Content / Support</t>
         </is>
       </c>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>US-REPORT2</t>
-        </is>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>[Web]</t>
+          <t>US-URL</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>[CMS, Web]</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Report: Ghi nhận thông tin báo cáo phase 2 - quy hoạch bộ báo cáo chuẩn cho ĐKOL</t>
+          <t>Quản lý URL</t>
         </is>
       </c>
       <c r="D16" s="10" t="inlineStr">
@@ -1314,49 +1314,49 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Sprint 21 (01/11 - 15/11)</t>
+          <t>Sprint 22 (16/11 - 30/11)</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>DEV In Progress</t>
+          <t>Đang phân tích/Document</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>ThuyTT104</t>
+          <t>SonLN11</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>55%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>Analytics / Partner</t>
+          <t>SEO / Infra</t>
         </is>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>US-QC</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="inlineStr">
+          <t>US-SECTIONLIB</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>[CMS, Web]</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Quản lý quảng cáo</t>
+          <t>Xây dựng thư viện section mở rộng cho tạo LDP kéo thả</t>
         </is>
       </c>
       <c r="D17" s="10" t="inlineStr">
@@ -1366,12 +1366,12 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Sprint 21 (01/11 - 15/11)</t>
+          <t>Sprint 22 (16/11 - 30/11)</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -1386,29 +1386,29 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>LDP Builder</t>
         </is>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>US-LDPLOCAL</t>
-        </is>
-      </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>[Web, CMS]</t>
+          <t>US-GIFT</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>[Web]</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>CMS config LDP local - QT tạo LDP Local - SEO - Schame</t>
+          <t>Luồng quà tặng (Mũ bảo hiểm) trên website</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
@@ -1423,44 +1423,44 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>Đang phân tích/Document</t>
+          <t>Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>SonLN11</t>
+          <t>ThuyTT104</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>35%</t>
+          <t>10%</t>
         </is>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>SEO / Growth</t>
+          <t>Commerce Feature</t>
         </is>
       </c>
     </row>
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>US-BREADCRUMBS</t>
-        </is>
-      </c>
-      <c r="B19" s="8" t="inlineStr">
-        <is>
-          <t>[CMS, Web]</t>
+          <t>US-28</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>[Web]</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Quản lý Breadcrums trên trang/ landing Page</t>
+          <t>[FMI Phase 4 | NBA] Phối hợp tích hợp Trigger Popup &amp; Web Push trên fptvn.vn</t>
         </is>
       </c>
       <c r="D19" s="10" t="inlineStr">
@@ -1475,34 +1475,34 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P4</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>Đang phân tích/Document</t>
+          <t>Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>SonLN11</t>
+          <t>ThuyTT104</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>10%</t>
         </is>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>SEO / Navigation</t>
+          <t>Personalization</t>
         </is>
       </c>
     </row>
     <row r="20" ht="24" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>US-CHARM</t>
+          <t>US-47</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
@@ -1512,27 +1512,27 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Luồng bán kèm PK (charm) trên website fpt.vn</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="inlineStr">
-        <is>
-          <t>Tháng 11</t>
+          <t>Luồng giỏ hàng trên kênh</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>Tháng 12</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Sprint 21 (01/11 - 15/11)</t>
+          <t>Sprint 23 (01/12 - 15/12)</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>Đã tiếp nhận yêu cầu</t>
+          <t>Đang phân tích/Document</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1542,39 +1542,39 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>40%</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>Commerce Feature</t>
+          <t>Core Commerce</t>
         </is>
       </c>
     </row>
     <row r="21" ht="24" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>US-18</t>
-        </is>
-      </c>
-      <c r="B21" s="8" t="inlineStr">
+          <t>US-NEWS</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>[CMS, Web]</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Quản lý FAQ</t>
-        </is>
-      </c>
-      <c r="D21" s="10" t="inlineStr">
-        <is>
-          <t>Tháng 11</t>
+          <t>Quản lý tin tức</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>Tháng 12</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Sprint 22 (16/11 - 30/11)</t>
+          <t>Sprint 23 (01/12 - 15/12)</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -1584,49 +1584,49 @@
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>Đang phân tích/Document</t>
+          <t>Đã tiếp nhận yêu cầu</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>SonLN11</t>
+          <t>LongNH156</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
-          <t>Content / Support</t>
+          <t>Content / SEO</t>
         </is>
       </c>
     </row>
     <row r="22" ht="24" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>US-URL</t>
+          <t>US-AUTHOR</t>
         </is>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>[CMS, Web]</t>
+          <t>[CMS]</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Quản lý URL</t>
-        </is>
-      </c>
-      <c r="D22" s="10" t="inlineStr">
-        <is>
-          <t>Tháng 11</t>
+          <t>Quản lý Profile Tác giả</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>Tháng 12</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Sprint 22 (16/11 - 30/11)</t>
+          <t>Sprint 23 (01/12 - 15/12)</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -1636,49 +1636,49 @@
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>Đang phân tích/Document</t>
+          <t>Đã tiếp nhận yêu cầu</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>SonLN11</t>
+          <t>LongNH156</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
-          <t>SEO / Infra</t>
+          <t>Content / SEO</t>
         </is>
       </c>
     </row>
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>US-SECTIONLIB</t>
-        </is>
-      </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>[CMS, Web]</t>
+          <t>US-38</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>[Web, CMS]</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Xây dựng thư viện section mở rộng cho tạo LDP kéo thả</t>
-        </is>
-      </c>
-      <c r="D23" s="10" t="inlineStr">
-        <is>
-          <t>Tháng 11</t>
+          <t>Trang LDP CSCA</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>Tháng 12</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Sprint 22 (16/11 - 30/11)</t>
+          <t>Sprint 24 (16/12 - 31/12)</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -1688,7 +1688,7 @@
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>Đang phân tích/Document</t>
+          <t>Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
@@ -1698,44 +1698,44 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
-          <t>LDP Builder</t>
+          <t>Campaign LDP</t>
         </is>
       </c>
     </row>
     <row r="24" ht="24" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>US-GIFT</t>
-        </is>
-      </c>
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>[Web]</t>
+          <t>US-39</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>[Web, CMS]</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Luồng quà tặng (Mũ bảo hiểm) trên website</t>
-        </is>
-      </c>
-      <c r="D24" s="10" t="inlineStr">
-        <is>
-          <t>Tháng 11</t>
+          <t>Trang LDP Fcitizen</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>Tháng 12</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Sprint 21 (01/11 - 15/11)</t>
+          <t>Sprint 24 (16/12 - 31/12)</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -1745,49 +1745,49 @@
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>ThuyTT104</t>
+          <t>SonLN11</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>10%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
-          <t>Commerce Feature</t>
+          <t>Campaign LDP</t>
         </is>
       </c>
     </row>
     <row r="25" ht="24" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>US-28</t>
-        </is>
-      </c>
-      <c r="B25" s="9" t="inlineStr">
-        <is>
-          <t>[Web]</t>
+          <t>US-40</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>[Web, CMS]</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>[FMI Phase 4 | NBA] Phối hợp tích hợp Trigger Popup &amp; Web Push trên fptvn.vn</t>
-        </is>
-      </c>
-      <c r="D25" s="10" t="inlineStr">
-        <is>
-          <t>Tháng 11</t>
+          <t>Trang LDP NHA</t>
+        </is>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>Tháng 12</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Sprint 22 (16/11 - 30/11)</t>
+          <t>Sprint 24 (16/12 - 31/12)</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>P4</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -1797,34 +1797,34 @@
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>ThuyTT104</t>
+          <t>SonLN11</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>10%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
-          <t>Personalization</t>
+          <t>Campaign LDP</t>
         </is>
       </c>
     </row>
     <row r="26" ht="24" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>US-47</t>
-        </is>
-      </c>
-      <c r="B26" s="9" t="inlineStr">
-        <is>
-          <t>[Web]</t>
+          <t>US-41</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>[Web, CMS]</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Luồng giỏ hàng trên kênh</t>
+          <t>Trang LDP NHA lịch thi đấu</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -1834,49 +1834,49 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Sprint 23 (01/12 - 15/12)</t>
+          <t>Sprint 24 (16/12 - 31/12)</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>Đang phân tích/Document</t>
+          <t>Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>ThuyTT104</t>
+          <t>SonLN11</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>Core Commerce</t>
+          <t>Campaign LDP</t>
         </is>
       </c>
     </row>
     <row r="27" ht="24" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>US-NEWS</t>
-        </is>
-      </c>
-      <c r="B27" s="8" t="inlineStr">
-        <is>
-          <t>[CMS, Web]</t>
+          <t>US-42</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>[Web, CMS]</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Quản lý tin tức</t>
+          <t>Trang LDP NHA bảng xếp hạng</t>
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr">
@@ -1886,7 +1886,7 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Sprint 23 (01/12 - 15/12)</t>
+          <t>Sprint 24 (16/12 - 31/12)</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
@@ -1896,39 +1896,39 @@
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>Đã tiếp nhận yêu cầu</t>
+          <t>Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>LongNH156</t>
+          <t>SonLN11</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
-          <t>Content / SEO</t>
+          <t>Campaign LDP</t>
         </is>
       </c>
     </row>
     <row r="28" ht="24" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>US-AUTHOR</t>
+          <t>US-43</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>[CMS]</t>
+          <t>[Web, CMS]</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Quản lý Profile Tác giả</t>
+          <t>Trang LDP NHA -SA</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -1938,7 +1938,7 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Sprint 23 (01/12 - 15/12)</t>
+          <t>Sprint 24 (16/12 - 31/12)</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
@@ -1948,39 +1948,39 @@
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>Đã tiếp nhận yêu cầu</t>
+          <t>Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>LongNH156</t>
+          <t>SonLN11</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>Content / SEO</t>
+          <t>Campaign LDP</t>
         </is>
       </c>
     </row>
     <row r="29" ht="24" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>US-38</t>
-        </is>
-      </c>
-      <c r="B29" s="8" t="inlineStr">
+          <t>US-26</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>[Web, CMS]</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Trang LDP CSCA</t>
+          <t>Các link chạy ads team Performance chạy ads - quy hoạch về CMS mới</t>
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr">
@@ -1990,49 +1990,49 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Sprint 24 (16/12 - 31/12)</t>
+          <t>Sprint 23 (01/12 - 15/12)</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>Chưa tiếp nhận</t>
+          <t>Đang phân tích/Document</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>SonLN11</t>
+          <t>LongNH156 / SonLN11</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
-          <t>Campaign LDP</t>
+          <t>Marketing Ops</t>
         </is>
       </c>
     </row>
     <row r="30" ht="24" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>US-39</t>
-        </is>
-      </c>
-      <c r="B30" s="8" t="inlineStr">
-        <is>
-          <t>[Web, CMS]</t>
+          <t>US-48</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>[Web]</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Trang LDP Fcitizen</t>
+          <t>Rule ưu tiên Apply Voucher / Rule loại trừ Voucher / Cấu hình trang chi tiết Voucher</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -2042,12 +2042,12 @@
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>Sprint 24 (16/12 - 31/12)</t>
+          <t>Sprint 23 (01/12 - 15/12)</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -2057,34 +2057,34 @@
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>SonLN11</t>
+          <t>ThuyTT104</t>
         </is>
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>10%</t>
         </is>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>Campaign LDP</t>
+          <t>Promotion Engine</t>
         </is>
       </c>
     </row>
     <row r="31" ht="24" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>US-40</t>
-        </is>
-      </c>
-      <c r="B31" s="8" t="inlineStr">
-        <is>
-          <t>[Web, CMS]</t>
+          <t>US-27</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>[CMS, Web]</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Trang LDP NHA</t>
+          <t>Bổ sung trang "Combo Internet Camera"</t>
         </is>
       </c>
       <c r="D31" s="11" t="inlineStr">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P4</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
@@ -2119,421 +2119,109 @@
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
-          <t>Campaign LDP</t>
+          <t>Product Page</t>
         </is>
       </c>
     </row>
     <row r="32" ht="24" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>US-41</t>
-        </is>
-      </c>
-      <c r="B32" s="8" t="inlineStr">
+          <t>US-19</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>[CMS, Web]</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Suggest gói</t>
+        </is>
+      </c>
+      <c r="D32" s="11" t="inlineStr">
+        <is>
+          <t>Tháng 12</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>Sprint 24 (16/12 - 31/12)</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>Chưa tiếp nhận</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>SonLN11</t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="J32" s="6" t="inlineStr">
+        <is>
+          <t>Interactive Tool</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="24" customHeight="1">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>OPS-BUFFER</t>
+        </is>
+      </c>
+      <c r="B33" s="12" t="inlineStr">
         <is>
           <t>[Web, CMS]</t>
         </is>
       </c>
-      <c r="C32" s="6" t="inlineStr">
-        <is>
-          <t>Trang LDP NHA lịch thi đấu</t>
-        </is>
-      </c>
-      <c r="D32" s="11" t="inlineStr">
-        <is>
-          <t>Tháng 12</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>Sprint 24 (16/12 - 31/12)</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="G32" s="4" t="inlineStr">
-        <is>
-          <t>Chưa tiếp nhận</t>
-        </is>
-      </c>
-      <c r="H32" s="4" t="inlineStr">
-        <is>
-          <t>SonLN11</t>
-        </is>
-      </c>
-      <c r="I32" s="4" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="J32" s="6" t="inlineStr">
-        <is>
-          <t>Campaign LDP</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="24" customHeight="1">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>US-42</t>
-        </is>
-      </c>
-      <c r="B33" s="8" t="inlineStr">
-        <is>
-          <t>[Web, CMS]</t>
-        </is>
-      </c>
-      <c r="C33" s="6" t="inlineStr">
-        <is>
-          <t>Trang LDP NHA bảng xếp hạng</t>
-        </is>
-      </c>
-      <c r="D33" s="11" t="inlineStr">
-        <is>
-          <t>Tháng 12</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>Sprint 24 (16/12 - 31/12)</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="G33" s="4" t="inlineStr">
-        <is>
-          <t>Chưa tiếp nhận</t>
-        </is>
-      </c>
-      <c r="H33" s="4" t="inlineStr">
-        <is>
-          <t>SonLN11</t>
-        </is>
-      </c>
-      <c r="I33" s="4" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="J33" s="6" t="inlineStr">
-        <is>
-          <t>Campaign LDP</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="24" customHeight="1">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>US-43</t>
-        </is>
-      </c>
-      <c r="B34" s="8" t="inlineStr">
-        <is>
-          <t>[Web, CMS]</t>
-        </is>
-      </c>
-      <c r="C34" s="6" t="inlineStr">
-        <is>
-          <t>Trang LDP NHA -SA</t>
-        </is>
-      </c>
-      <c r="D34" s="11" t="inlineStr">
-        <is>
-          <t>Tháng 12</t>
-        </is>
-      </c>
-      <c r="E34" s="4" t="inlineStr">
-        <is>
-          <t>Sprint 24 (16/12 - 31/12)</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="G34" s="4" t="inlineStr">
-        <is>
-          <t>Chưa tiếp nhận</t>
-        </is>
-      </c>
-      <c r="H34" s="4" t="inlineStr">
-        <is>
-          <t>SonLN11</t>
-        </is>
-      </c>
-      <c r="I34" s="4" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="J34" s="6" t="inlineStr">
-        <is>
-          <t>Campaign LDP</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="24" customHeight="1">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>US-26</t>
-        </is>
-      </c>
-      <c r="B35" s="8" t="inlineStr">
-        <is>
-          <t>[Web, CMS]</t>
-        </is>
-      </c>
-      <c r="C35" s="6" t="inlineStr">
-        <is>
-          <t>Các link chạy ads team Performance chạy ads - quy hoạch về CMS mới</t>
-        </is>
-      </c>
-      <c r="D35" s="11" t="inlineStr">
-        <is>
-          <t>Tháng 12</t>
-        </is>
-      </c>
-      <c r="E35" s="4" t="inlineStr">
-        <is>
-          <t>Sprint 23 (01/12 - 15/12)</t>
-        </is>
-      </c>
-      <c r="F35" s="4" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="G35" s="4" t="inlineStr">
-        <is>
-          <t>Đang phân tích/Document</t>
-        </is>
-      </c>
-      <c r="H35" s="4" t="inlineStr">
-        <is>
-          <t>LongNH156 / SonLN11</t>
-        </is>
-      </c>
-      <c r="I35" s="4" t="inlineStr">
-        <is>
-          <t>20%</t>
-        </is>
-      </c>
-      <c r="J35" s="6" t="inlineStr">
-        <is>
-          <t>Marketing Ops</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="24" customHeight="1">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>US-48</t>
-        </is>
-      </c>
-      <c r="B36" s="9" t="inlineStr">
-        <is>
-          <t>[Web]</t>
-        </is>
-      </c>
-      <c r="C36" s="6" t="inlineStr">
-        <is>
-          <t>Rule ưu tiên Apply Voucher / Rule loại trừ Voucher / Cấu hình trang chi tiết Voucher</t>
-        </is>
-      </c>
-      <c r="D36" s="11" t="inlineStr">
-        <is>
-          <t>Tháng 12</t>
-        </is>
-      </c>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t>Sprint 23 (01/12 - 15/12)</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="G36" s="4" t="inlineStr">
-        <is>
-          <t>Chưa tiếp nhận</t>
-        </is>
-      </c>
-      <c r="H36" s="4" t="inlineStr">
-        <is>
-          <t>ThuyTT104</t>
-        </is>
-      </c>
-      <c r="I36" s="4" t="inlineStr">
-        <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="J36" s="6" t="inlineStr">
-        <is>
-          <t>Promotion Engine</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="24" customHeight="1">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>US-27</t>
-        </is>
-      </c>
-      <c r="B37" s="8" t="inlineStr">
-        <is>
-          <t>[CMS, Web]</t>
-        </is>
-      </c>
-      <c r="C37" s="6" t="inlineStr">
-        <is>
-          <t>Bổ sung trang "Combo Internet Camera"</t>
-        </is>
-      </c>
-      <c r="D37" s="11" t="inlineStr">
-        <is>
-          <t>Tháng 12</t>
-        </is>
-      </c>
-      <c r="E37" s="4" t="inlineStr">
-        <is>
-          <t>Sprint 24 (16/12 - 31/12)</t>
-        </is>
-      </c>
-      <c r="F37" s="4" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
-      <c r="G37" s="4" t="inlineStr">
-        <is>
-          <t>Chưa tiếp nhận</t>
-        </is>
-      </c>
-      <c r="H37" s="4" t="inlineStr">
-        <is>
-          <t>SonLN11</t>
-        </is>
-      </c>
-      <c r="I37" s="4" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="J37" s="6" t="inlineStr">
-        <is>
-          <t>Product Page</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="24" customHeight="1">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>US-19</t>
-        </is>
-      </c>
-      <c r="B38" s="8" t="inlineStr">
-        <is>
-          <t>[CMS, Web]</t>
-        </is>
-      </c>
-      <c r="C38" s="6" t="inlineStr">
-        <is>
-          <t>Suggest gói</t>
-        </is>
-      </c>
-      <c r="D38" s="11" t="inlineStr">
-        <is>
-          <t>Tháng 12</t>
-        </is>
-      </c>
-      <c r="E38" s="4" t="inlineStr">
-        <is>
-          <t>Sprint 24 (16/12 - 31/12)</t>
-        </is>
-      </c>
-      <c r="F38" s="4" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
-      <c r="G38" s="4" t="inlineStr">
-        <is>
-          <t>Chưa tiếp nhận</t>
-        </is>
-      </c>
-      <c r="H38" s="4" t="inlineStr">
-        <is>
-          <t>SonLN11</t>
-        </is>
-      </c>
-      <c r="I38" s="4" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="J38" s="6" t="inlineStr">
-        <is>
-          <t>Interactive Tool</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="24" customHeight="1">
-      <c r="A39" s="12" t="inlineStr">
-        <is>
-          <t>OPS-BUFFER</t>
-        </is>
-      </c>
-      <c r="B39" s="12" t="inlineStr">
-        <is>
-          <t>[Web, CMS]</t>
-        </is>
-      </c>
-      <c r="C39" s="13" t="inlineStr">
+      <c r="C33" s="13" t="inlineStr">
         <is>
           <t>[VẬN HÀNH &amp; DỰ PHÒNG] Quỹ năng lực linh hoạt xử lý yêu cầu phát sinh (15-20% Sprint Capacity)</t>
         </is>
       </c>
-      <c r="D39" s="12" t="inlineStr">
+      <c r="D33" s="12" t="inlineStr">
         <is>
           <t>Xuyên suốt Q4/2026</t>
         </is>
       </c>
-      <c r="E39" s="12" t="inlineStr">
+      <c r="E33" s="12" t="inlineStr">
         <is>
           <t>Sprints 19 - 24</t>
         </is>
       </c>
-      <c r="F39" s="12" t="inlineStr">
+      <c r="F33" s="12" t="inlineStr">
         <is>
           <t>P1 - Linh hoạt</t>
         </is>
       </c>
-      <c r="G39" s="12" t="inlineStr">
+      <c r="G33" s="12" t="inlineStr">
         <is>
           <t>Đang vận hành</t>
         </is>
       </c>
-      <c r="H39" s="12" t="inlineStr">
+      <c r="H33" s="12" t="inlineStr">
         <is>
           <t>All Team (BA/Dev/QC)</t>
         </is>
       </c>
-      <c r="I39" s="12" t="inlineStr">
+      <c r="I33" s="12" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
-      <c r="J39" s="13" t="inlineStr">
+      <c r="J33" s="13" t="inlineStr">
         <is>
           <t>Operations Buffer</t>
         </is>
@@ -2554,7 +2242,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2570,7 +2258,7 @@
     <row r="1" ht="35" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CHI TIẾT BACKLOG QUÝ 4/2026 — ACCEPTANCE CRITERIA &amp; MÔ TẢ NGHIỆP VỤ</t>
+          <t>CHI TIẾT 29 USER STORIES ACTIVE QUÝ 4/2026 (ĐÃ LOẠI BỎ DONE &amp; PENDING)</t>
         </is>
       </c>
     </row>
@@ -2619,17 +2307,17 @@
     <row r="3" ht="36" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>US-08</t>
+          <t>US-MENU</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>[CMS]</t>
+          <t>[Web, CMS]</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Nội dung hiển thị Gói bán</t>
+          <t>MENU</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
@@ -2644,24 +2332,24 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>DEV In Progress</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>LongNH156</t>
+          <t>ThuyTT104 / SonLN11</t>
         </is>
       </c>
       <c r="H3" s="15" t="inlineStr">
         <is>
-          <t>Sync Core Data tự động; Khóa Read-only Core; Cho phép Enrich tên hiển thị, thứ tự, bullet point ưu đãi, Badge, Toggle hiển thị.</t>
+          <t>Quy hoạch và đồng bộ luồng cấu hình Menu đa cấp trên CMS và hiển thị trải nghiệm Responsive trên Website fpt.vn.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="36" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>US-09</t>
+          <t>US-12</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -2671,7 +2359,7 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Cấu hình hiển thị checkout</t>
+          <t>Quản lý trang</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -2681,7 +2369,7 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -2696,14 +2384,14 @@
       </c>
       <c r="H4" s="15" t="inlineStr">
         <is>
-          <t>Cấu hình Form checkout động (Toggle On/Off, Required/Optional, Drag &amp; Drop), Validation Regex, Gán Add-ons &amp; Quà tặng 0đ.</t>
+          <t>Module quản trị cấu trúc trang tổng thể, tạo trang mới, cấu hình SEO meta, quản lý trạng thái xuất bản.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="36" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>US-10</t>
+          <t>US-13</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -2713,7 +2401,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Phương thức Thanh toán</t>
+          <t>Quản lý section</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -2723,7 +2411,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -2738,24 +2426,24 @@
       </c>
       <c r="H5" s="15" t="inlineStr">
         <is>
-          <t>Quản lý danh sách cổng (FPT Pay, VNPay, MoMo, ATM/Visa, COD), tích hợp Kill-Switch ngắt khẩn cấp cổng thanh toán lỗi.</t>
+          <t>Tạo và cấu hình các Section nội dung linh hoạt trên CMS phục vụ dựng trang nhanh.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>US-MENU</t>
+          <t>US-14</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>[Web, CMS]</t>
+          <t>[CMS]</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>MENU</t>
+          <t>Quản lý Block</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -2765,29 +2453,29 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>DEV In Progress</t>
+          <t>UAT</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>ThuyTT104 / SonLN11</t>
+          <t>LongNH156</t>
         </is>
       </c>
       <c r="H6" s="15" t="inlineStr">
         <is>
-          <t>Quy hoạch và đồng bộ luồng cấu hình Menu đa cấp trên CMS và hiển thị trải nghiệm Responsive trên Website fpt.vn.</t>
+          <t>Quản lý các khối thành phần (Block) tái sử dụng cho nhiều layout trang khác nhau.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>US-07</t>
+          <t>US-15</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -2797,7 +2485,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Quản lý bài viết của tác giả (Quản lý tin tức)</t>
+          <t>Quản lý menu</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -2812,7 +2500,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Chưa tiếp nhận</t>
+          <t>UAT</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -2822,14 +2510,14 @@
       </c>
       <c r="H7" s="15" t="inlineStr">
         <is>
-          <t>Tạo mới, chỉnh sửa thông tin tác giả và gán tác giả viết bài khi soạn thảo tin tức trên CMS.</t>
+          <t>Quản trị danh mục menu điều hướng, thứ tự cấp bậc cha-con, liên kết trang trên CMS.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="36" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>US-11</t>
+          <t>US-07</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -2839,7 +2527,7 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Quản lý Badge/Tag</t>
+          <t>Quản lý bài viết của tác giả (Quản lý tin tức)</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -2854,7 +2542,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -2864,197 +2552,197 @@
       </c>
       <c r="H8" s="15" t="inlineStr">
         <is>
-          <t>Thư viện Badge/Tag truyền thông (Hot, Mới, Bán chạy, Flash sale), cấu hình gán linh hoạt vào sản phẩm/gói dịch vụ.</t>
+          <t>Tạo mới, chỉnh sửa thông tin tác giả và gán tác giả viết bài khi soạn thảo tin tức trên CMS.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="36" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>US-12</t>
+          <t>US-REPORT2</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>[CMS]</t>
+          <t>[Web]</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Quản lý trang</t>
+          <t>Report: Ghi nhận thông tin báo cáo phase 2 - quy hoạch bộ báo cáo chuẩn cho ĐKOL</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Tháng 10</t>
+          <t>Tháng 11</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>DEV In Progress</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>LongNH156</t>
+          <t>ThuyTT104</t>
         </is>
       </c>
       <c r="H9" s="15" t="inlineStr">
         <is>
-          <t>Module quản trị cấu trúc trang tổng thể, tạo trang mới, cấu hình SEO meta, quản lý trạng thái xuất bản.</t>
+          <t>Chuẩn hóa bộ báo cáo tracking chuyển đổi, lượt xem, đơn hàng dành riêng cho kênh đối tác ĐKOL.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="36" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>US-13</t>
+          <t>US-QC</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>[CMS]</t>
+          <t>[CMS, Web]</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Quản lý section</t>
+          <t>Quản lý quảng cáo</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Tháng 10</t>
+          <t>Tháng 11</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>Đang phân tích/Document</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>LongNH156</t>
+          <t>SonLN11</t>
         </is>
       </c>
       <c r="H10" s="15" t="inlineStr">
         <is>
-          <t>Tạo và cấu hình các Section nội dung linh hoạt trên CMS phục vụ dựng trang nhanh.</t>
+          <t>Cấu hình các vị trí quảng cáo đối tác, banner tài trợ, banner chiến dịch trên website.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="36" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>US-14</t>
+          <t>US-LDPLOCAL</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>[CMS]</t>
+          <t>[Web, CMS]</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Quản lý Block</t>
+          <t>CMS config LDP local - QT tạo LDP Local - SEO - Schame</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Tháng 10</t>
+          <t>Tháng 11</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>Đang phân tích/Document</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>LongNH156</t>
+          <t>SonLN11</t>
         </is>
       </c>
       <c r="H11" s="15" t="inlineStr">
         <is>
-          <t>Quản lý các khối thành phần (Block) tái sử dụng cho nhiều layout trang khác nhau.</t>
+          <t>Tạo trang LDP theo vùng miền/tỉnh thành, tự động gắn Schema JSON-LD và tối ưu hóa SEO local.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="36" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>US-15</t>
+          <t>US-BREADCRUMBS</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>[CMS]</t>
+          <t>[CMS, Web]</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Quản lý menu</t>
+          <t>Quản lý Breadcrums trên trang/ landing Page</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Tháng 10</t>
+          <t>Tháng 11</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>Đang phân tích/Document</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>LongNH156</t>
+          <t>SonLN11</t>
         </is>
       </c>
       <c r="H12" s="15" t="inlineStr">
         <is>
-          <t>Quản trị danh mục menu điều hướng, thứ tự cấp bậc cha-con, liên kết trang trên CMS.</t>
+          <t>Cấu hình thanh điều hướng Breadcrumb động theo cấu trúc cây thư mục, tối ưu UX và SEO structured data.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="36" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>US-16</t>
+          <t>US-CHARM</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>[CMS]</t>
+          <t>[Web]</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Quản lý banner</t>
+          <t>Luồng bán kèm PK (charm) trên website fpt.vn</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Tháng 10</t>
+          <t>Tháng 11</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -3064,39 +2752,39 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>Đã tiếp nhận yêu cầu</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>LongNH156</t>
+          <t>ThuyTT104</t>
         </is>
       </c>
       <c r="H13" s="15" t="inlineStr">
         <is>
-          <t>Quản trị banner theo từng vị trí (Header, Hero, Body), hẹn giờ hiển thị, tracking click.</t>
+          <t>Xây dựng luồng mua kèm Charm phụ kiện Camera Play 4 (ưu đãi 0đ hoặc phụ thu, Best-deal, quota 1:1).</t>
         </is>
       </c>
     </row>
     <row r="14" ht="36" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>US-17</t>
+          <t>US-18</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>[CMS]</t>
+          <t>[CMS, Web]</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Quản lý popup</t>
+          <t>Quản lý FAQ</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Tháng 10</t>
+          <t>Tháng 11</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -3106,34 +2794,34 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>Đang phân tích/Document</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>LongNH156</t>
+          <t>SonLN11</t>
         </is>
       </c>
       <c r="H14" s="15" t="inlineStr">
         <is>
-          <t>Cấu hình hiển thị Popup truyền thông, điều kiện trigger theo trang, tần suất hiển thị cho KH.</t>
+          <t>Quản trị danh mục câu hỏi thường gặp theo chủ đề sản phẩm/dịch vụ, hỗ trợ tìm kiếm và hiển thị FAQ schema.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="36" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>US-REPORT2</t>
+          <t>US-URL</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>[Web]</t>
+          <t>[CMS, Web]</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Report: Ghi nhận thông tin báo cáo phase 2 - quy hoạch bộ báo cáo chuẩn cho ĐKOL</t>
+          <t>Quản lý URL</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -3143,29 +2831,29 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>DEV In Progress</t>
+          <t>Đang phân tích/Document</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>ThuyTT104</t>
+          <t>SonLN11</t>
         </is>
       </c>
       <c r="H15" s="15" t="inlineStr">
         <is>
-          <t>Chuẩn hóa bộ báo cáo tracking chuyển đổi, lượt xem, đơn hàng dành riêng cho kênh đối tác ĐKOL.</t>
+          <t>Quy hoạch cấu trúc URL thân thiện (Friendly URL), cấu hình 301 Redirect và kiểm soát duplicate URL.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="36" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>US-QC</t>
+          <t>US-SECTIONLIB</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -3175,7 +2863,7 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Quản lý quảng cáo</t>
+          <t>Xây dựng thư viện section mở rộng cho tạo LDP kéo thả</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -3185,7 +2873,7 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
@@ -3200,24 +2888,24 @@
       </c>
       <c r="H16" s="15" t="inlineStr">
         <is>
-          <t>Cấu hình các vị trí quảng cáo đối tác, banner tài trợ, banner chiến dịch trên website.</t>
+          <t>Bổ sung kho Section component mẫu (Pricing table, Hero form, Feedback, Video review) để kéo thả LDP.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="36" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>US-LDPLOCAL</t>
+          <t>US-GIFT</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>[Web, CMS]</t>
+          <t>[Web]</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>CMS config LDP local - QT tạo LDP Local - SEO - Schame</t>
+          <t>Luồng quà tặng (Mũ bảo hiểm) trên website</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -3227,39 +2915,39 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Đang phân tích/Document</t>
+          <t>Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>SonLN11</t>
+          <t>ThuyTT104</t>
         </is>
       </c>
       <c r="H17" s="15" t="inlineStr">
         <is>
-          <t>Tạo trang LDP theo vùng miền/tỉnh thành, tự động gắn Schema JSON-LD và tối ưu hóa SEO local.</t>
+          <t>Tích hợp luồng quà tặng hiện vật theo chương trình kích cầu đăng ký Internet/Camera toàn trình.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="36" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>US-BREADCRUMBS</t>
+          <t>US-28</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>[CMS, Web]</t>
+          <t>[Web]</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Quản lý Breadcrums trên trang/ landing Page</t>
+          <t>[FMI Phase 4 | NBA] Phối hợp tích hợp Trigger Popup &amp; Web Push trên fptvn.vn</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -3269,29 +2957,29 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P4</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Đang phân tích/Document</t>
+          <t>Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>SonLN11</t>
+          <t>ThuyTT104</t>
         </is>
       </c>
       <c r="H18" s="15" t="inlineStr">
         <is>
-          <t>Cấu hình thanh điều hướng Breadcrumb động theo cấu trúc cây thư mục, tối ưu UX và SEO structured data.</t>
+          <t>Kết nối API hệ thống Next Best Action (NBA) để kích hoạt popup ngữ cảnh và thông báo Web Push.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="36" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>US-CHARM</t>
+          <t>US-47</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -3301,22 +2989,22 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Luồng bán kèm PK (charm) trên website fpt.vn</t>
+          <t>Luồng giỏ hàng trên kênh</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Tháng 11</t>
+          <t>Tháng 12</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Đã tiếp nhận yêu cầu</t>
+          <t>Đang phân tích/Document</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -3326,14 +3014,14 @@
       </c>
       <c r="H19" s="15" t="inlineStr">
         <is>
-          <t>Xây dựng luồng mua kèm Charm phụ kiện Camera Play 4 (ưu đãi 0đ hoặc phụ thu, Best-deal, quota 1:1).</t>
+          <t>Xây dựng Cart toàn trình: giỏ hàng đa sản phẩm, gộp đơn dịch vụ + thiết bị, tính toán khuyến mãi real-time.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="36" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>US-18</t>
+          <t>US-NEWS</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -3343,12 +3031,12 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Quản lý FAQ</t>
+          <t>Quản lý tin tức</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Tháng 11</t>
+          <t>Tháng 12</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
@@ -3358,39 +3046,39 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Đang phân tích/Document</t>
+          <t>Đã tiếp nhận yêu cầu</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>SonLN11</t>
+          <t>LongNH156</t>
         </is>
       </c>
       <c r="H20" s="15" t="inlineStr">
         <is>
-          <t>Quản trị danh mục câu hỏi thường gặp theo chủ đề sản phẩm/dịch vụ, hỗ trợ tìm kiếm và hiển thị FAQ schema.</t>
+          <t>Hệ thống tin tức hoàn chỉnh: danh mục tin, bài viết chuyên sâu, tin khuyến mãi, gắn tag sản phẩm.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="36" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>US-URL</t>
+          <t>US-AUTHOR</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>[CMS, Web]</t>
+          <t>[CMS]</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Quản lý URL</t>
+          <t>Quản lý Profile Tác giả</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Tháng 11</t>
+          <t>Tháng 12</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
@@ -3400,39 +3088,39 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Đang phân tích/Document</t>
+          <t>Đã tiếp nhận yêu cầu</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>SonLN11</t>
+          <t>LongNH156</t>
         </is>
       </c>
       <c r="H21" s="15" t="inlineStr">
         <is>
-          <t>Quy hoạch cấu trúc URL thân thiện (Friendly URL), cấu hình 301 Redirect và kiểm soát duplicate URL.</t>
+          <t>Quản lý trang hồ sơ chuyên gia / tác giả tin tức (E-E-A-T chuẩn Google), liên kết mạng xã hội và bài viết.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="36" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>US-SECTIONLIB</t>
+          <t>US-38</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>[CMS, Web]</t>
+          <t>[Web, CMS]</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Xây dựng thư viện section mở rộng cho tạo LDP kéo thả</t>
+          <t>Trang LDP CSCA</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Tháng 11</t>
+          <t>Tháng 12</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
@@ -3442,7 +3130,7 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Đang phân tích/Document</t>
+          <t>Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -3452,34 +3140,34 @@
       </c>
       <c r="H22" s="15" t="inlineStr">
         <is>
-          <t>Bổ sung kho Section component mẫu (Pricing table, Hero form, Feedback, Video review) để kéo thả LDP.</t>
+          <t>Landing Page dành riêng cho dịch vụ Chữ ký số &amp; An toàn thông tin doanh nghiệp (CSCA).</t>
         </is>
       </c>
     </row>
     <row r="23" ht="36" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>US-GIFT</t>
+          <t>US-39</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>[Web]</t>
+          <t>[Web, CMS]</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Luồng quà tặng (Mũ bảo hiểm) trên website</t>
+          <t>Trang LDP Fcitizen</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Tháng 11</t>
+          <t>Tháng 12</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -3489,39 +3177,39 @@
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>ThuyTT104</t>
+          <t>SonLN11</t>
         </is>
       </c>
       <c r="H23" s="15" t="inlineStr">
         <is>
-          <t>Tích hợp luồng quà tặng hiện vật theo chương trình kích cầu đăng ký Internet/Camera toàn trình.</t>
+          <t>Landing Page chương trình ưu đãi công dân số FPT Citizen.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="36" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>US-28</t>
+          <t>US-40</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>[Web]</t>
+          <t>[Web, CMS]</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>[FMI Phase 4 | NBA] Phối hợp tích hợp Trigger Popup &amp; Web Push trên fptvn.vn</t>
+          <t>Trang LDP NHA</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Tháng 11</t>
+          <t>Tháng 12</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>P4</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
@@ -3531,29 +3219,29 @@
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>ThuyTT104</t>
+          <t>SonLN11</t>
         </is>
       </c>
       <c r="H24" s="15" t="inlineStr">
         <is>
-          <t>Kết nối API hệ thống Next Best Action (NBA) để kích hoạt popup ngữ cảnh và thông báo Web Push.</t>
+          <t>Landing Page chiến dịch Bản quyền Ngoại Hạng Anh (NHA) trên hệ thống FPT Play.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="36" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>US-47</t>
+          <t>US-41</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>[Web]</t>
+          <t>[Web, CMS]</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Luồng giỏ hàng trên kênh</t>
+          <t>Trang LDP NHA lịch thi đấu</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
@@ -3563,39 +3251,39 @@
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Đang phân tích/Document</t>
+          <t>Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>ThuyTT104</t>
+          <t>SonLN11</t>
         </is>
       </c>
       <c r="H25" s="15" t="inlineStr">
         <is>
-          <t>Xây dựng Cart toàn trình: giỏ hàng đa sản phẩm, gộp đơn dịch vụ + thiết bị, tính toán khuyến mãi real-time.</t>
+          <t>Sub-page Lịch thi đấu giải Ngoại Hạng Anh cập nhật liên tục kèm nút đăng ký gói FPT Play.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="36" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>US-NEWS</t>
+          <t>US-42</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>[CMS, Web]</t>
+          <t>[Web, CMS]</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Quản lý tin tức</t>
+          <t>Trang LDP NHA bảng xếp hạng</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -3610,34 +3298,34 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>Đã tiếp nhận yêu cầu</t>
+          <t>Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>LongNH156</t>
+          <t>SonLN11</t>
         </is>
       </c>
       <c r="H26" s="15" t="inlineStr">
         <is>
-          <t>Hệ thống tin tức hoàn chỉnh: danh mục tin, bài viết chuyên sâu, tin khuyến mãi, gắn tag sản phẩm.</t>
+          <t>Sub-page Bảng xếp hạng giải Ngoại Hạng Anh tương tác trực tiếp.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="36" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>US-AUTHOR</t>
+          <t>US-43</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>[CMS]</t>
+          <t>[Web, CMS]</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Quản lý Profile Tác giả</t>
+          <t>Trang LDP NHA -SA</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
@@ -3652,24 +3340,24 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>Đã tiếp nhận yêu cầu</t>
+          <t>Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>LongNH156</t>
+          <t>SonLN11</t>
         </is>
       </c>
       <c r="H27" s="15" t="inlineStr">
         <is>
-          <t>Quản lý trang hồ sơ chuyên gia / tác giả tin tức (E-E-A-T chuẩn Google), liên kết mạng xã hội và bài viết.</t>
+          <t>Trang đích chuyên biệt dành cho luồng bán hàng Sales Agent (SA) chiến dịch NHA.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="36" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>US-38</t>
+          <t>US-26</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
@@ -3679,7 +3367,7 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Trang LDP CSCA</t>
+          <t>Các link chạy ads team Performance chạy ads - quy hoạch về CMS mới</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
@@ -3689,39 +3377,39 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>Chưa tiếp nhận</t>
+          <t>Đang phân tích/Document</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>SonLN11</t>
+          <t>LongNH156 / SonLN11</t>
         </is>
       </c>
       <c r="H28" s="15" t="inlineStr">
         <is>
-          <t>Landing Page dành riêng cho dịch vụ Chữ ký số &amp; An toàn thông tin doanh nghiệp (CSCA).</t>
+          <t>Quy hoạch và chuyển giao toàn bộ các URL chạy ads của Marketing sang hạ tầng CMS mới để tracking đồng bộ.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="36" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>US-39</t>
+          <t>US-48</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>[Web, CMS]</t>
+          <t>[Web]</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Trang LDP Fcitizen</t>
+          <t>Rule ưu tiên Apply Voucher / Rule loại trừ Voucher / Cấu hình trang chi tiết Voucher</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -3731,7 +3419,7 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
@@ -3741,29 +3429,29 @@
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>SonLN11</t>
+          <t>ThuyTT104</t>
         </is>
       </c>
       <c r="H29" s="15" t="inlineStr">
         <is>
-          <t>Landing Page chương trình ưu đãi công dân số FPT Citizen.</t>
+          <t>Engine tính toán thứ tự ưu tiên áp dụng voucher, quy tắc loại trừ chồng chéo khuyến mãi, trang chi tiết Voucher.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="36" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>US-40</t>
+          <t>US-27</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>[Web, CMS]</t>
+          <t>[CMS, Web]</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Trang LDP NHA</t>
+          <t>Bổ sung trang "Combo Internet Camera"</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
@@ -3773,7 +3461,7 @@
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P4</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
@@ -3788,24 +3476,24 @@
       </c>
       <c r="H30" s="15" t="inlineStr">
         <is>
-          <t>Landing Page chiến dịch Bản quyền Ngoại Hạng Anh (NHA) trên hệ thống FPT Play.</t>
+          <t>Thiết kế &amp; dựng trang bán hàng chuyên biệt gói tích hợp Internet + FPT Camera trọn gói gia đình.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="36" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>US-41</t>
+          <t>US-19</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>[Web, CMS]</t>
+          <t>[CMS, Web]</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Trang LDP NHA lịch thi đấu</t>
+          <t>Suggest gói</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
@@ -3815,7 +3503,7 @@
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P4</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -3830,14 +3518,14 @@
       </c>
       <c r="H31" s="15" t="inlineStr">
         <is>
-          <t>Sub-page Lịch thi đấu giải Ngoại Hạng Anh cập nhật liên tục kèm nút đăng ký gói FPT Play.</t>
+          <t>Công cụ gợi ý gói cước thông minh dựa trên nhu cầu người dùng (số lượng thiết bị, diện tích nhà, nhu cầu chơi game/xem phim).</t>
         </is>
       </c>
     </row>
     <row r="32" ht="36" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>US-42</t>
+          <t>OPS-BUFFER</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
@@ -3847,282 +3535,30 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Trang LDP NHA bảng xếp hạng</t>
+          <t>[VẬN HÀNH &amp; DỰ PHÒNG] Quỹ năng lực linh hoạt xử lý yêu cầu phát sinh (15-20% Sprint Capacity)</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Tháng 12</t>
+          <t>Xuyên suốt Q4/2026</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1 - Linh hoạt</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Chưa tiếp nhận</t>
+          <t>Đang vận hành</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>SonLN11</t>
+          <t>All Team (BA/Dev/QC)</t>
         </is>
       </c>
       <c r="H32" s="15" t="inlineStr">
-        <is>
-          <t>Sub-page Bảng xếp hạng giải Ngoại Hạng Anh tương tác trực tiếp.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="36" customHeight="1">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>US-43</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>[Web, CMS]</t>
-        </is>
-      </c>
-      <c r="C33" s="6" t="inlineStr">
-        <is>
-          <t>Trang LDP NHA -SA</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>Tháng 12</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>Chưa tiếp nhận</t>
-        </is>
-      </c>
-      <c r="G33" s="4" t="inlineStr">
-        <is>
-          <t>SonLN11</t>
-        </is>
-      </c>
-      <c r="H33" s="15" t="inlineStr">
-        <is>
-          <t>Trang đích chuyên biệt dành cho luồng bán hàng Sales Agent (SA) chiến dịch NHA.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="36" customHeight="1">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>US-26</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>[Web, CMS]</t>
-        </is>
-      </c>
-      <c r="C34" s="6" t="inlineStr">
-        <is>
-          <t>Các link chạy ads team Performance chạy ads - quy hoạch về CMS mới</t>
-        </is>
-      </c>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
-          <t>Tháng 12</t>
-        </is>
-      </c>
-      <c r="E34" s="4" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t>Đang phân tích/Document</t>
-        </is>
-      </c>
-      <c r="G34" s="4" t="inlineStr">
-        <is>
-          <t>LongNH156 / SonLN11</t>
-        </is>
-      </c>
-      <c r="H34" s="15" t="inlineStr">
-        <is>
-          <t>Quy hoạch và chuyển giao toàn bộ các URL chạy ads của Marketing sang hạ tầng CMS mới để tracking đồng bộ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="36" customHeight="1">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>US-48</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>[Web]</t>
-        </is>
-      </c>
-      <c r="C35" s="6" t="inlineStr">
-        <is>
-          <t>Rule ưu tiên Apply Voucher / Rule loại trừ Voucher / Cấu hình trang chi tiết Voucher</t>
-        </is>
-      </c>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>Tháng 12</t>
-        </is>
-      </c>
-      <c r="E35" s="4" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="F35" s="4" t="inlineStr">
-        <is>
-          <t>Chưa tiếp nhận</t>
-        </is>
-      </c>
-      <c r="G35" s="4" t="inlineStr">
-        <is>
-          <t>ThuyTT104</t>
-        </is>
-      </c>
-      <c r="H35" s="15" t="inlineStr">
-        <is>
-          <t>Engine tính toán thứ tự ưu tiên áp dụng voucher, quy tắc loại trừ chồng chéo khuyến mãi, trang chi tiết Voucher.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="36" customHeight="1">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>US-27</t>
-        </is>
-      </c>
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>[CMS, Web]</t>
-        </is>
-      </c>
-      <c r="C36" s="6" t="inlineStr">
-        <is>
-          <t>Bổ sung trang "Combo Internet Camera"</t>
-        </is>
-      </c>
-      <c r="D36" s="4" t="inlineStr">
-        <is>
-          <t>Tháng 12</t>
-        </is>
-      </c>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>Chưa tiếp nhận</t>
-        </is>
-      </c>
-      <c r="G36" s="4" t="inlineStr">
-        <is>
-          <t>SonLN11</t>
-        </is>
-      </c>
-      <c r="H36" s="15" t="inlineStr">
-        <is>
-          <t>Thiết kế &amp; dựng trang bán hàng chuyên biệt gói tích hợp Internet + FPT Camera trọn gói gia đình.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="36" customHeight="1">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>US-19</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <t>[CMS, Web]</t>
-        </is>
-      </c>
-      <c r="C37" s="6" t="inlineStr">
-        <is>
-          <t>Suggest gói</t>
-        </is>
-      </c>
-      <c r="D37" s="4" t="inlineStr">
-        <is>
-          <t>Tháng 12</t>
-        </is>
-      </c>
-      <c r="E37" s="4" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
-      <c r="F37" s="4" t="inlineStr">
-        <is>
-          <t>Chưa tiếp nhận</t>
-        </is>
-      </c>
-      <c r="G37" s="4" t="inlineStr">
-        <is>
-          <t>SonLN11</t>
-        </is>
-      </c>
-      <c r="H37" s="15" t="inlineStr">
-        <is>
-          <t>Công cụ gợi ý gói cước thông minh dựa trên nhu cầu người dùng (số lượng thiết bị, diện tích nhà, nhu cầu chơi game/xem phim).</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="36" customHeight="1">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>OPS-BUFFER</t>
-        </is>
-      </c>
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>[Web, CMS]</t>
-        </is>
-      </c>
-      <c r="C38" s="6" t="inlineStr">
-        <is>
-          <t>[VẬN HÀNH &amp; DỰ PHÒNG] Quỹ năng lực linh hoạt xử lý yêu cầu phát sinh (15-20% Sprint Capacity)</t>
-        </is>
-      </c>
-      <c r="D38" s="4" t="inlineStr">
-        <is>
-          <t>Xuyên suốt Q4/2026</t>
-        </is>
-      </c>
-      <c r="E38" s="4" t="inlineStr">
-        <is>
-          <t>P1 - Linh hoạt</t>
-        </is>
-      </c>
-      <c r="F38" s="4" t="inlineStr">
-        <is>
-          <t>Đang vận hành</t>
-        </is>
-      </c>
-      <c r="G38" s="4" t="inlineStr">
-        <is>
-          <t>All Team (BA/Dev/QC)</t>
-        </is>
-      </c>
-      <c r="H38" s="15" t="inlineStr">
         <is>
           <t>Dành 15-20% velocity mỗi sprint cho: Fix bug khẩn cấp, hỗ trợ chiến dịch Marketing đột xuất, tối ưu link CTV/AM, Auto sync menu, điều hướng link, đảm bảo không trễ hạn các US cam kết.</t>
         </is>

</xml_diff>

<commit_message>
feat(roadmap): cap nhat US-MENU bo sung cap API dong bo layout va thong tin cho cac trang SPDV
</commit_message>
<xml_diff>
--- a/thuyttdoc/Roadmap_Website_CMS_Q4_2026.xlsx
+++ b/thuyttdoc/Roadmap_Website_CMS_Q4_2026.xlsx
@@ -680,7 +680,7 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>MENU</t>
+          <t>MENU (API Đa kênh &amp; Đồng bộ SPDV)</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
@@ -715,7 +715,7 @@
       </c>
       <c r="J4" s="6" t="inlineStr">
         <is>
-          <t>Core Product</t>
+          <t>Core Infra / API Sync</t>
         </is>
       </c>
     </row>
@@ -2317,7 +2317,7 @@
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>MENU</t>
+          <t>MENU (API Đa kênh &amp; Đồng bộ SPDV)</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
@@ -2342,7 +2342,8 @@
       </c>
       <c r="H3" s="15" t="inlineStr">
         <is>
-          <t>Quy hoạch và đồng bộ luồng cấu hình Menu đa cấp trên CMS và hiển thị trải nghiệm Responsive trên Website fpt.vn.</t>
+          <t>Ý 1: Viết API cấp mới bộ menu cho HiFPT &amp; Website fpt.vn responsive đa cấp.
+Ý 2: Cấp API tập trung cho các trang Sản phẩm Dịch vụ (SPDV: Internet, Camera, FPT Play, Smart Home,...) để tự động đồng bộ layout, cấu trúc cây điều hướng và thông tin hiển thị thống nhất toàn hệ sinh thái.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(roadmap): cap nhat mo ta chi tiet cho FAQ va CMS config LDP local gan location SEO
</commit_message>
<xml_diff>
--- a/thuyttdoc/Roadmap_Website_CMS_Q4_2026.xlsx
+++ b/thuyttdoc/Roadmap_Website_CMS_Q4_2026.xlsx
@@ -1040,7 +1040,7 @@
     <row r="12" ht="25" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>US-27</t>
+          <t>US-LDPLOCAL</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>CMS config  LDP local - QT tạo LDP Local - SEO - Schame</t>
+          <t>CMS config LDP Local (Gắn Location &amp; SEO Schema)</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
@@ -1950,12 +1950,12 @@
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="62" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
@@ -2256,7 +2256,7 @@
       </c>
       <c r="H8" s="15" t="inlineStr">
         <is>
-          <t>Tài liệu: Thiết kế:</t>
+          <t>Quy hoạch lại UIUX và luồng cấu hình FAQ (Danh sách FAQ) &amp; Danh mục FAQ. Tối ưu tìm kiếm và cấu trúc Schema FAQ cho SEO.</t>
         </is>
       </c>
     </row>
@@ -2347,7 +2347,7 @@
     <row r="11" ht="38" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>US-27</t>
+          <t>US-LDPLOCAL</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -2357,7 +2357,7 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>CMS config  LDP local - QT tạo LDP Local - SEO - Schame</t>
+          <t>CMS config LDP Local (Gắn Location &amp; SEO Schema)</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -2382,7 +2382,7 @@
       </c>
       <c r="H11" s="15" t="inlineStr">
         <is>
-          <t>https://fpt.vn/lap-internet-wifi-phuong-tang-nhon-phu-hcmhttps://fpt.vn/lap-internet-wifi-xa-vinh-loc-hcmhttps://fpt.vn/lap-internet-wifi-phuong-dong-hung-thuan-hcmhttps://fpt.vn/lap-internet-wifi-phuong-hiep-binh-hcmhttps://fpt.vn/lap-internet-wifi-phuong-tan-my-hcmhttps://fpt.vn/lap-internet-wifi-phuong-duong-noi-ha-noihttps://fpt.vn/lap-internet-wifi-xa-an-khanh-ha-noihttps://fpt.vn/lap-internet-wifi-phuong-yen-hoa-ha-noihttps://fpt.vn/lap-internet-wifi-phuong-hoang-mai-ha-noihttps://fpt.vn/lap-internet-wifi-xa-thuan-an-ha-noi</t>
+          <t>Xây dựng luồng tạo LDP gắn location (Tỉnh/TP - Phường/Xã) - Ghi nhận schema, SEO tự động theo từng địa phương.</t>
         </is>
       </c>
     </row>
@@ -2880,7 +2880,11 @@
           <t>ThuyTT104</t>
         </is>
       </c>
-      <c r="H23" s="15" t="inlineStr"/>
+      <c r="H23" s="15" t="inlineStr">
+        <is>
+          <t>Config CMS, Cấu hình rule riêng, UIUX</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="38" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
@@ -2918,7 +2922,11 @@
           <t>ThuyTT104</t>
         </is>
       </c>
-      <c r="H24" s="15" t="inlineStr"/>
+      <c r="H24" s="15" t="inlineStr">
+        <is>
+          <t>Config CMS, Cấu hình rule riêng, UIUX</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="38" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
@@ -2956,7 +2964,11 @@
           <t>SonLN11</t>
         </is>
       </c>
-      <c r="H25" s="15" t="inlineStr"/>
+      <c r="H25" s="15" t="inlineStr">
+        <is>
+          <t>Config CMS, Cấu hình rule riêng, UIUX</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="38" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
@@ -2994,7 +3006,11 @@
           <t>SonLN11</t>
         </is>
       </c>
-      <c r="H26" s="15" t="inlineStr"/>
+      <c r="H26" s="15" t="inlineStr">
+        <is>
+          <t>Config CMS, tích hợp API FPL về lịch thi đấu, BXH</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="38" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
@@ -3032,7 +3048,11 @@
           <t>SonLN11</t>
         </is>
       </c>
-      <c r="H27" s="15" t="inlineStr"/>
+      <c r="H27" s="15" t="inlineStr">
+        <is>
+          <t>Config CMS, tích hợp API FPL về lịch thi đấu, BXH</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="38" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
@@ -3070,7 +3090,11 @@
           <t>SonLN11</t>
         </is>
       </c>
-      <c r="H28" s="15" t="inlineStr"/>
+      <c r="H28" s="15" t="inlineStr">
+        <is>
+          <t>Config CMS, tích hợp API FPL về lịch thi đấu, BXH</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="38" customHeight="1">
       <c r="A29" s="4" t="inlineStr">

</xml_diff>

<commit_message>
style(roadmap): bo khung vang buffer duoi cung o ca ban anh va ban excel
</commit_message>
<xml_diff>
--- a/thuyttdoc/Roadmap_Website_CMS_Q4_2026.xlsx
+++ b/thuyttdoc/Roadmap_Website_CMS_Q4_2026.xlsx
@@ -220,7 +220,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -242,11 +242,88 @@
         <color rgb="00CBD5E1"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -318,6 +395,9 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -683,7 +763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R31"/>
+  <dimension ref="A1:R30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -756,33 +836,33 @@
           <t>THÁNG 10 / 2026 (Nền tảng &amp; Menu)</t>
         </is>
       </c>
-      <c r="H3" s="5" t="n"/>
-      <c r="I3" s="5" t="n"/>
-      <c r="J3" s="5" t="n"/>
+      <c r="H3" s="25" t="n"/>
+      <c r="I3" s="25" t="n"/>
+      <c r="J3" s="26" t="n"/>
       <c r="K3" s="6" t="inlineStr">
         <is>
           <t>THÁNG 11 / 2026 (Bán kèm, SEO &amp; LDP)</t>
         </is>
       </c>
-      <c r="L3" s="5" t="n"/>
-      <c r="M3" s="5" t="n"/>
-      <c r="N3" s="5" t="n"/>
+      <c r="L3" s="25" t="n"/>
+      <c r="M3" s="25" t="n"/>
+      <c r="N3" s="26" t="n"/>
       <c r="O3" s="7" t="inlineStr">
         <is>
           <t>THÁNG 12 / 2026 (Giỏ hàng &amp; Chiến dịch NHA)</t>
         </is>
       </c>
-      <c r="P3" s="5" t="n"/>
-      <c r="Q3" s="5" t="n"/>
-      <c r="R3" s="5" t="n"/>
+      <c r="P3" s="25" t="n"/>
+      <c r="Q3" s="25" t="n"/>
+      <c r="R3" s="26" t="n"/>
     </row>
     <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="5" t="n"/>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
+      <c r="A4" s="27" t="n"/>
+      <c r="B4" s="27" t="n"/>
+      <c r="C4" s="27" t="n"/>
+      <c r="D4" s="27" t="n"/>
+      <c r="E4" s="27" t="n"/>
+      <c r="F4" s="27" t="n"/>
       <c r="G4" s="8" t="inlineStr">
         <is>
           <t>Tuần 1
@@ -2540,98 +2620,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="26" customHeight="1">
-      <c r="A31" s="20" t="inlineStr">
-        <is>
-          <t>OPS-BUFFER</t>
-        </is>
-      </c>
-      <c r="B31" s="20" t="inlineStr">
-        <is>
-          <t>[Web, CMS]</t>
-        </is>
-      </c>
-      <c r="C31" s="21" t="inlineStr">
-        <is>
-          <t>[QUỸ VẬN HÀNH &amp; DỰ PHÒNG] Xử lý phát sinh (15-20% Sprint Capacity)</t>
-        </is>
-      </c>
-      <c r="D31" s="20" t="inlineStr">
-        <is>
-          <t>All Team</t>
-        </is>
-      </c>
-      <c r="E31" s="20" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F31" s="20" t="inlineStr">
-        <is>
-          <t>Đang vận hành</t>
-        </is>
-      </c>
-      <c r="G31" s="22" t="inlineStr">
-        <is>
-          <t>⚡ BUFFER</t>
-        </is>
-      </c>
-      <c r="H31" s="22" t="inlineStr">
-        <is>
-          <t>⚡ BUFFER</t>
-        </is>
-      </c>
-      <c r="I31" s="22" t="inlineStr">
-        <is>
-          <t>⚡ BUFFER</t>
-        </is>
-      </c>
-      <c r="J31" s="22" t="inlineStr">
-        <is>
-          <t>⚡ BUFFER</t>
-        </is>
-      </c>
-      <c r="K31" s="22" t="inlineStr">
-        <is>
-          <t>⚡ BUFFER</t>
-        </is>
-      </c>
-      <c r="L31" s="22" t="inlineStr">
-        <is>
-          <t>⚡ BUFFER</t>
-        </is>
-      </c>
-      <c r="M31" s="22" t="inlineStr">
-        <is>
-          <t>⚡ BUFFER</t>
-        </is>
-      </c>
-      <c r="N31" s="22" t="inlineStr">
-        <is>
-          <t>⚡ BUFFER</t>
-        </is>
-      </c>
-      <c r="O31" s="22" t="inlineStr">
-        <is>
-          <t>⚡ BUFFER</t>
-        </is>
-      </c>
-      <c r="P31" s="22" t="inlineStr">
-        <is>
-          <t>⚡ BUFFER</t>
-        </is>
-      </c>
-      <c r="Q31" s="22" t="inlineStr">
-        <is>
-          <t>⚡ BUFFER</t>
-        </is>
-      </c>
-      <c r="R31" s="22" t="inlineStr">
-        <is>
-          <t>⚡ BUFFER</t>
-        </is>
-      </c>
-    </row>
+    <row r="31" ht="26" customHeight="1"/>
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="G3:J3"/>

</xml_diff>

<commit_message>
feat(roadmap): cap nhat gantt timeline chay vat xuyen thang cho cac task da thang Q4/2026
</commit_message>
<xml_diff>
--- a/thuyttdoc/Roadmap_Website_CMS_Q4_2026.xlsx
+++ b/thuyttdoc/Roadmap_Website_CMS_Q4_2026.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -85,20 +85,8 @@
       <color rgb="000369A1"/>
       <sz val="10"/>
     </font>
-    <font>
-      <name val="Times New Roman"/>
-      <b val="1"/>
-      <color rgb="000F172A"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Times New Roman"/>
-      <b val="1"/>
-      <color rgb="0092400E"/>
-      <sz val="8"/>
-    </font>
   </fonts>
-  <fills count="21">
+  <fills count="20">
     <fill>
       <patternFill/>
     </fill>
@@ -197,20 +185,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="006EE7B7"/>
-        <bgColor rgb="006EE7B7"/>
+        <fgColor rgb="0086EFAC"/>
+        <bgColor rgb="0086EFAC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
-        <bgColor rgb="00FEF3C7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FDE68A"/>
-        <bgColor rgb="00FDE68A"/>
+        <fgColor rgb="006EE7B7"/>
+        <bgColor rgb="006EE7B7"/>
       </patternFill>
     </fill>
     <fill>
@@ -220,7 +202,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -242,88 +224,11 @@
         <color rgb="00CBD5E1"/>
       </bottom>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00CBD5E1"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CBD5E1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00CBD5E1"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CBD5E1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00CBD5E1"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00CBD5E1"/>
-      </left>
-      <right style="thin">
-        <color rgb="00CBD5E1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00CBD5E1"/>
-      </left>
-      <right style="thin">
-        <color rgb="00CBD5E1"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="00CBD5E1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -345,13 +250,13 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -380,24 +285,15 @@
     <xf numFmtId="0" fontId="7" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -796,7 +692,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Các cột thể hiện Trục thời gian từng Tháng/Tuần | Các dòng thể hiện Task | Ô màu cam [🎯 Xong] là Mốc hạn chót phải hoàn thành &amp; nghiệm thu</t>
+          <t>Các cột thể hiện Trục thời gian từng Tháng/Tuần | Thanh ngang kéo dài qua các tháng thể hiện task thực thi liên tục | [🎯 XONG] là mốc nghiệm thu</t>
         </is>
       </c>
     </row>
@@ -833,106 +729,94 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>THÁNG 10 / 2026 (Nền tảng &amp; Menu)</t>
-        </is>
-      </c>
-      <c r="H3" s="25" t="n"/>
-      <c r="I3" s="25" t="n"/>
-      <c r="J3" s="26" t="n"/>
+          <t>THÁNG 10 / 2026</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="n"/>
+      <c r="I3" s="5" t="n"/>
+      <c r="J3" s="5" t="n"/>
       <c r="K3" s="6" t="inlineStr">
         <is>
-          <t>THÁNG 11 / 2026 (Bán kèm, SEO &amp; LDP)</t>
-        </is>
-      </c>
-      <c r="L3" s="25" t="n"/>
-      <c r="M3" s="25" t="n"/>
-      <c r="N3" s="26" t="n"/>
+          <t>THÁNG 11 / 2026</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="n"/>
+      <c r="M3" s="5" t="n"/>
+      <c r="N3" s="5" t="n"/>
       <c r="O3" s="7" t="inlineStr">
         <is>
-          <t>THÁNG 12 / 2026 (Giỏ hàng &amp; Chiến dịch NHA)</t>
-        </is>
-      </c>
-      <c r="P3" s="25" t="n"/>
-      <c r="Q3" s="25" t="n"/>
-      <c r="R3" s="26" t="n"/>
-    </row>
-    <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="27" t="n"/>
-      <c r="B4" s="27" t="n"/>
-      <c r="C4" s="27" t="n"/>
-      <c r="D4" s="27" t="n"/>
-      <c r="E4" s="27" t="n"/>
-      <c r="F4" s="27" t="n"/>
+          <t>THÁNG 12 / 2026</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="n"/>
+      <c r="Q3" s="5" t="n"/>
+      <c r="R3" s="5" t="n"/>
+    </row>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="5" t="n"/>
+      <c r="B4" s="5" t="n"/>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
       <c r="G4" s="8" t="inlineStr">
         <is>
-          <t>Tuần 1
-(Sp 19)</t>
+          <t>Tuần 1</t>
         </is>
       </c>
       <c r="H4" s="8" t="inlineStr">
         <is>
-          <t>Tuần 2
-(Sp 19)</t>
+          <t>Tuần 2</t>
         </is>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
-          <t>Tuần 3
-(Sp 20)</t>
+          <t>Tuần 3</t>
         </is>
       </c>
       <c r="J4" s="8" t="inlineStr">
         <is>
-          <t>Tuần 4
-(Sp 20)</t>
+          <t>Tuần 4</t>
         </is>
       </c>
       <c r="K4" s="9" t="inlineStr">
         <is>
-          <t>Tuần 1
-(Sp 21)</t>
+          <t>Tuần 1</t>
         </is>
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Tuần 2
-(Sp 21)</t>
+          <t>Tuần 2</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>Tuần 3
-(Sp 22)</t>
+          <t>Tuần 3</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Tuần 4
-(Sp 22)</t>
+          <t>Tuần 4</t>
         </is>
       </c>
       <c r="O4" s="10" t="inlineStr">
         <is>
-          <t>Tuần 1
-(Sp 23)</t>
+          <t>Tuần 1</t>
         </is>
       </c>
       <c r="P4" s="10" t="inlineStr">
         <is>
-          <t>Tuần 2
-(Sp 23)</t>
+          <t>Tuần 2</t>
         </is>
       </c>
       <c r="Q4" s="10" t="inlineStr">
         <is>
-          <t>Tuần 3
-(Sp 24)</t>
+          <t>Tuần 3</t>
         </is>
       </c>
       <c r="R4" s="10" t="inlineStr">
         <is>
-          <t>Tuần 4
-(Sp 24)</t>
+          <t>Tuần 4</t>
         </is>
       </c>
     </row>
@@ -977,12 +861,16 @@
           <t>▬</t>
         </is>
       </c>
-      <c r="I5" s="15" t="inlineStr">
+      <c r="I5" s="14" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
+      <c r="J5" s="15" t="inlineStr">
         <is>
           <t>🎯 XONG</t>
         </is>
       </c>
-      <c r="J5" s="5" t="n"/>
       <c r="K5" s="5" t="n"/>
       <c r="L5" s="5" t="n"/>
       <c r="M5" s="5" t="n"/>
@@ -1033,12 +921,16 @@
           <t>▬</t>
         </is>
       </c>
-      <c r="I6" s="15" t="inlineStr">
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
+      <c r="J6" s="15" t="inlineStr">
         <is>
           <t>🎯 XONG</t>
         </is>
       </c>
-      <c r="J6" s="5" t="n"/>
       <c r="K6" s="5" t="n"/>
       <c r="L6" s="5" t="n"/>
       <c r="M6" s="5" t="n"/>
@@ -1089,12 +981,16 @@
           <t>▬</t>
         </is>
       </c>
-      <c r="I7" s="15" t="inlineStr">
+      <c r="I7" s="14" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
+      <c r="J7" s="15" t="inlineStr">
         <is>
           <t>🎯 XONG</t>
         </is>
       </c>
-      <c r="J7" s="5" t="n"/>
       <c r="K7" s="5" t="n"/>
       <c r="L7" s="5" t="n"/>
       <c r="M7" s="5" t="n"/>
@@ -1145,12 +1041,16 @@
           <t>▬</t>
         </is>
       </c>
-      <c r="I8" s="15" t="inlineStr">
+      <c r="I8" s="14" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
+      <c r="J8" s="15" t="inlineStr">
         <is>
           <t>🎯 XONG</t>
         </is>
       </c>
-      <c r="J8" s="5" t="n"/>
       <c r="K8" s="5" t="n"/>
       <c r="L8" s="5" t="n"/>
       <c r="M8" s="5" t="n"/>
@@ -1191,7 +1091,11 @@
           <t>DEV In Progress</t>
         </is>
       </c>
-      <c r="G9" s="5" t="n"/>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
       <c r="H9" s="14" t="inlineStr">
         <is>
           <t>▬</t>
@@ -1247,8 +1151,16 @@
           <t>Đang phân tích/Document</t>
         </is>
       </c>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
+      <c r="G10" s="17" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
+      <c r="H10" s="17" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
       <c r="I10" s="17" t="inlineStr">
         <is>
           <t>▬</t>
@@ -1315,8 +1227,16 @@
           <t>Đang phân tích/Document</t>
         </is>
       </c>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n"/>
+      <c r="G11" s="17" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
+      <c r="H11" s="17" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
       <c r="I11" s="17" t="inlineStr">
         <is>
           <t>▬</t>
@@ -1383,8 +1303,16 @@
           <t>DEV In Progress</t>
         </is>
       </c>
-      <c r="G12" s="5" t="n"/>
-      <c r="H12" s="5" t="n"/>
+      <c r="G12" s="17" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
+      <c r="H12" s="17" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
       <c r="I12" s="17" t="inlineStr">
         <is>
           <t>▬</t>
@@ -1451,8 +1379,16 @@
           <t>Đang phân tích/Document</t>
         </is>
       </c>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="5" t="n"/>
+      <c r="G13" s="17" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
+      <c r="H13" s="17" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
       <c r="I13" s="17" t="inlineStr">
         <is>
           <t>▬</t>
@@ -1521,16 +1457,8 @@
       </c>
       <c r="G14" s="5" t="n"/>
       <c r="H14" s="5" t="n"/>
-      <c r="I14" s="17" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
-      <c r="J14" s="17" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
+      <c r="I14" s="5" t="n"/>
+      <c r="J14" s="5" t="n"/>
       <c r="K14" s="17" t="inlineStr">
         <is>
           <t>▬</t>
@@ -1587,8 +1515,16 @@
           <t>Đang phân tích/Document</t>
         </is>
       </c>
-      <c r="G15" s="5" t="n"/>
-      <c r="H15" s="5" t="n"/>
+      <c r="G15" s="17" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
+      <c r="H15" s="17" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
       <c r="I15" s="17" t="inlineStr">
         <is>
           <t>▬</t>
@@ -1657,16 +1593,8 @@
       </c>
       <c r="G16" s="5" t="n"/>
       <c r="H16" s="5" t="n"/>
-      <c r="I16" s="17" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
-      <c r="J16" s="17" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
+      <c r="I16" s="5" t="n"/>
+      <c r="J16" s="5" t="n"/>
       <c r="K16" s="17" t="inlineStr">
         <is>
           <t>▬</t>
@@ -1785,16 +1713,8 @@
       </c>
       <c r="G18" s="5" t="n"/>
       <c r="H18" s="5" t="n"/>
-      <c r="I18" s="17" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
-      <c r="J18" s="17" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
+      <c r="I18" s="5" t="n"/>
+      <c r="J18" s="5" t="n"/>
       <c r="K18" s="17" t="inlineStr">
         <is>
           <t>▬</t>
@@ -1991,8 +1911,16 @@
       <c r="H21" s="5" t="n"/>
       <c r="I21" s="5" t="n"/>
       <c r="J21" s="5" t="n"/>
-      <c r="K21" s="5" t="n"/>
-      <c r="L21" s="5" t="n"/>
+      <c r="K21" s="19" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
+      <c r="L21" s="19" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
       <c r="M21" s="19" t="inlineStr">
         <is>
           <t>▬</t>
@@ -2059,8 +1987,16 @@
       <c r="H22" s="5" t="n"/>
       <c r="I22" s="5" t="n"/>
       <c r="J22" s="5" t="n"/>
-      <c r="K22" s="5" t="n"/>
-      <c r="L22" s="5" t="n"/>
+      <c r="K22" s="19" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
+      <c r="L22" s="19" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
       <c r="M22" s="19" t="inlineStr">
         <is>
           <t>▬</t>
@@ -2131,17 +2067,17 @@
       <c r="L23" s="5" t="n"/>
       <c r="M23" s="5" t="n"/>
       <c r="N23" s="5" t="n"/>
-      <c r="O23" s="19" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
-      <c r="P23" s="19" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
-      <c r="Q23" s="19" t="inlineStr">
+      <c r="O23" s="20" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
+      <c r="P23" s="20" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
+      <c r="Q23" s="20" t="inlineStr">
         <is>
           <t>▬</t>
         </is>
@@ -2191,17 +2127,17 @@
       <c r="L24" s="5" t="n"/>
       <c r="M24" s="5" t="n"/>
       <c r="N24" s="5" t="n"/>
-      <c r="O24" s="19" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
-      <c r="P24" s="19" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
-      <c r="Q24" s="19" t="inlineStr">
+      <c r="O24" s="20" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
+      <c r="P24" s="20" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
+      <c r="Q24" s="20" t="inlineStr">
         <is>
           <t>▬</t>
         </is>
@@ -2249,27 +2185,19 @@
       <c r="J25" s="5" t="n"/>
       <c r="K25" s="5" t="n"/>
       <c r="L25" s="5" t="n"/>
-      <c r="M25" s="19" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
-      <c r="N25" s="19" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
-      <c r="O25" s="19" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
-      <c r="P25" s="19" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
-      <c r="Q25" s="19" t="inlineStr">
+      <c r="M25" s="5" t="n"/>
+      <c r="N25" s="5" t="n"/>
+      <c r="O25" s="20" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
+      <c r="P25" s="20" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
+      <c r="Q25" s="20" t="inlineStr">
         <is>
           <t>▬</t>
         </is>
@@ -2317,27 +2245,19 @@
       <c r="J26" s="5" t="n"/>
       <c r="K26" s="5" t="n"/>
       <c r="L26" s="5" t="n"/>
-      <c r="M26" s="19" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
-      <c r="N26" s="19" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
-      <c r="O26" s="19" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
-      <c r="P26" s="19" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
-      <c r="Q26" s="19" t="inlineStr">
+      <c r="M26" s="5" t="n"/>
+      <c r="N26" s="5" t="n"/>
+      <c r="O26" s="20" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
+      <c r="P26" s="20" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
+      <c r="Q26" s="20" t="inlineStr">
         <is>
           <t>▬</t>
         </is>
@@ -2385,27 +2305,19 @@
       <c r="J27" s="5" t="n"/>
       <c r="K27" s="5" t="n"/>
       <c r="L27" s="5" t="n"/>
-      <c r="M27" s="19" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
-      <c r="N27" s="19" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
-      <c r="O27" s="19" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
-      <c r="P27" s="19" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
-      <c r="Q27" s="19" t="inlineStr">
+      <c r="M27" s="5" t="n"/>
+      <c r="N27" s="5" t="n"/>
+      <c r="O27" s="20" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
+      <c r="P27" s="20" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
+      <c r="Q27" s="20" t="inlineStr">
         <is>
           <t>▬</t>
         </is>
@@ -2453,27 +2365,19 @@
       <c r="J28" s="5" t="n"/>
       <c r="K28" s="5" t="n"/>
       <c r="L28" s="5" t="n"/>
-      <c r="M28" s="19" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
-      <c r="N28" s="19" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
-      <c r="O28" s="19" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
-      <c r="P28" s="19" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
-      <c r="Q28" s="19" t="inlineStr">
+      <c r="M28" s="5" t="n"/>
+      <c r="N28" s="5" t="n"/>
+      <c r="O28" s="20" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
+      <c r="P28" s="20" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
+      <c r="Q28" s="20" t="inlineStr">
         <is>
           <t>▬</t>
         </is>
@@ -2521,27 +2425,19 @@
       <c r="J29" s="5" t="n"/>
       <c r="K29" s="5" t="n"/>
       <c r="L29" s="5" t="n"/>
-      <c r="M29" s="19" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
-      <c r="N29" s="19" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
-      <c r="O29" s="19" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
-      <c r="P29" s="19" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
-      <c r="Q29" s="19" t="inlineStr">
+      <c r="M29" s="5" t="n"/>
+      <c r="N29" s="5" t="n"/>
+      <c r="O29" s="20" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
+      <c r="P29" s="20" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
+      <c r="Q29" s="20" t="inlineStr">
         <is>
           <t>▬</t>
         </is>
@@ -2589,27 +2485,19 @@
       <c r="J30" s="5" t="n"/>
       <c r="K30" s="5" t="n"/>
       <c r="L30" s="5" t="n"/>
-      <c r="M30" s="19" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
-      <c r="N30" s="19" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
-      <c r="O30" s="19" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
-      <c r="P30" s="19" t="inlineStr">
-        <is>
-          <t>▬</t>
-        </is>
-      </c>
-      <c r="Q30" s="19" t="inlineStr">
+      <c r="M30" s="5" t="n"/>
+      <c r="N30" s="5" t="n"/>
+      <c r="O30" s="20" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
+      <c r="P30" s="20" t="inlineStr">
+        <is>
+          <t>▬</t>
+        </is>
+      </c>
+      <c r="Q30" s="20" t="inlineStr">
         <is>
           <t>▬</t>
         </is>
@@ -2620,7 +2508,6 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="26" customHeight="1"/>
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="G3:J3"/>
@@ -2665,37 +2552,37 @@
       </c>
     </row>
     <row r="2" ht="28" customHeight="1">
-      <c r="A2" s="23" t="inlineStr">
+      <c r="A2" s="21" t="inlineStr">
         <is>
           <t>Mã US</t>
         </is>
       </c>
-      <c r="B2" s="23" t="inlineStr">
+      <c r="B2" s="21" t="inlineStr">
         <is>
           <t>Tag EPIC</t>
         </is>
       </c>
-      <c r="C2" s="23" t="inlineStr">
+      <c r="C2" s="21" t="inlineStr">
         <is>
           <t>Tên User Story</t>
         </is>
       </c>
-      <c r="D2" s="23" t="inlineStr">
-        <is>
-          <t>Hạn hoàn thành mong muốn</t>
-        </is>
-      </c>
-      <c r="E2" s="23" t="inlineStr">
+      <c r="D2" s="21" t="inlineStr">
+        <is>
+          <t>Timeline thực thi</t>
+        </is>
+      </c>
+      <c r="E2" s="21" t="inlineStr">
         <is>
           <t>Ưu tiên</t>
         </is>
       </c>
-      <c r="F2" s="23" t="inlineStr">
+      <c r="F2" s="21" t="inlineStr">
         <is>
           <t>PIC (BA)</t>
         </is>
       </c>
-      <c r="G2" s="23" t="inlineStr">
+      <c r="G2" s="21" t="inlineStr">
         <is>
           <t>Mô tả / Acceptance Criteria (AC)</t>
         </is>
@@ -2719,7 +2606,7 @@
       </c>
       <c r="D3" s="11" t="inlineStr">
         <is>
-          <t>Xong trong Tháng 10</t>
+          <t>Tháng 10</t>
         </is>
       </c>
       <c r="E3" s="11" t="inlineStr">
@@ -2732,7 +2619,7 @@
           <t>SonLN11</t>
         </is>
       </c>
-      <c r="G3" s="24" t="inlineStr">
+      <c r="G3" s="22" t="inlineStr">
         <is>
           <t>Tài liệu: https://docs.google.com/document/d/16At_9OIDgYllJD5LTjNcPJ5Xl3bH7Yz5/edit#heading=h.drflzu5y8cu0 Thiết kế: https://min-t-design.github.io/fptcms/FPT%20CMS%20Admin.dc.html#module=pages</t>
         </is>
@@ -2756,7 +2643,7 @@
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Xong trong Tháng 10</t>
+          <t>Tháng 10</t>
         </is>
       </c>
       <c r="E4" s="11" t="inlineStr">
@@ -2769,7 +2656,7 @@
           <t>SonLN11</t>
         </is>
       </c>
-      <c r="G4" s="24" t="inlineStr">
+      <c r="G4" s="22" t="inlineStr">
         <is>
           <t>Tài liệu: https://docs.google.com/document/d/16At_9OIDgYllJD5LTjNcPJ5Xl3bH7Yz5/edit#heading=h.brd374ni8mj8 Thiết kế: https://min-t-design.github.io/fptcms/FPT%20CMS%20Admin.dc.html#module=sections</t>
         </is>
@@ -2793,7 +2680,7 @@
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>Xong trong Tháng 10</t>
+          <t>Tháng 10</t>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
@@ -2806,7 +2693,7 @@
           <t>SonLN11</t>
         </is>
       </c>
-      <c r="G5" s="24" t="inlineStr">
+      <c r="G5" s="22" t="inlineStr">
         <is>
           <t>Tài liệu: https://docs.google.com/document/d/16At_9OIDgYllJD5LTjNcPJ5Xl3bH7Yz5/edit#heading=h.7rare7d2yixu Thiết kế: https://min-t-design.github.io/fptcms/FPT%20CMS%20Admin.dc.html#module=blocks</t>
         </is>
@@ -2830,7 +2717,7 @@
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Xong trong Tháng 10</t>
+          <t>Tháng 10</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
@@ -2843,7 +2730,7 @@
           <t>SonLN11</t>
         </is>
       </c>
-      <c r="G6" s="24" t="inlineStr">
+      <c r="G6" s="22" t="inlineStr">
         <is>
           <t>Tài liệu: https://docs.google.com/document/d/16At_9OIDgYllJD5LTjNcPJ5Xl3bH7Yz5/edit#heading=h.8aebfhjwgjov Thiết kế: https://min-t-design.github.io/fptcms/FPT%20CMS%20Admin.dc.html#module=cms-menu</t>
         </is>
@@ -2867,7 +2754,7 @@
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>Xong trong Tháng 10</t>
+          <t>Tháng 10</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
@@ -2880,7 +2767,7 @@
           <t>ThuyTT104</t>
         </is>
       </c>
-      <c r="G7" s="24" t="inlineStr">
+      <c r="G7" s="22" t="inlineStr">
         <is>
           <t>Ý 1: Viết API cấp mới bộ menu cho HiFPT &amp; Website fpt.vn (responsive đa cấp).
 Ý 2: Cấp API tập trung cho các trang Sản phẩm Dịch vụ (SPDV: Internet, Camera, FPT Play, Smart Home,...) để tự động đồng bộ layout, cấu trúc cây điều hướng và thông tin hiển thị thống nhất.</t>
@@ -2905,7 +2792,7 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Xong trong Tháng 11</t>
+          <t>Tháng 10 - Tháng 11</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
@@ -2918,7 +2805,7 @@
           <t>SonLN11</t>
         </is>
       </c>
-      <c r="G8" s="24" t="inlineStr">
+      <c r="G8" s="22" t="inlineStr">
         <is>
           <t>Quy hoạch lại UIUX và luồng cấu hình FAQ (Danh sách FAQ) &amp; Danh mục FAQ. Tối ưu tìm kiếm và cấu trúc Schema FAQ cho SEO.</t>
         </is>
@@ -2942,7 +2829,7 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>Xong trong Tháng 11</t>
+          <t>Tháng 10 - Tháng 11</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
@@ -2955,7 +2842,7 @@
           <t>LongNH156</t>
         </is>
       </c>
-      <c r="G9" s="24" t="inlineStr">
+      <c r="G9" s="22" t="inlineStr">
         <is>
           <t>Cấu hình chạy chữ quảng cáo trên CMS:- Danh sách quảng cáo- Nhập thông tin (text chạy chữ, link url, background, hình ảnh icon, màu sắc, kiểu chữ,...)- Cho phép hiển thị quảng cáo lên các trang mong muốn- Tốc độ chạy</t>
         </is>
@@ -2979,7 +2866,7 @@
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Xong trong Tháng 11</t>
+          <t>Tháng 10 - Tháng 11</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
@@ -2992,7 +2879,7 @@
           <t>ThuyTT104</t>
         </is>
       </c>
-      <c r="G10" s="24" t="inlineStr">
+      <c r="G10" s="22" t="inlineStr">
         <is>
           <t>"Báo cáo đơn hàng: CheckoutBáo cáo dịch vụ:  thông tin của dịch vụ hợp đồngBáo cáo Omisell: Khi chuyển đổi source code: check lại luồng (đặt tên kênh lại )"</t>
         </is>
@@ -3016,7 +2903,7 @@
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>Xong trong Tháng 11</t>
+          <t>Tháng 10 - Tháng 11</t>
         </is>
       </c>
       <c r="E11" s="11" t="inlineStr">
@@ -3029,7 +2916,7 @@
           <t>ThuyTT104, LongNH156</t>
         </is>
       </c>
-      <c r="G11" s="24" t="inlineStr">
+      <c r="G11" s="22" t="inlineStr">
         <is>
           <t>Xây dựng luồng tạo LDP gắn location (Tỉnh/TP - Phường/Xã) - Ghi nhận schema, SEO tự động theo từng địa phương.</t>
         </is>
@@ -3053,7 +2940,7 @@
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Xong trong Tháng 11</t>
+          <t>Tháng 11</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
@@ -3066,7 +2953,7 @@
           <t>LongNH156, ThuyTT104</t>
         </is>
       </c>
-      <c r="G12" s="24" t="inlineStr">
+      <c r="G12" s="22" t="inlineStr">
         <is>
           <t>Quy hoạch bộ URL toàn website Fptvn Đánh dấu loại page để phục vụ cho Modue LDP</t>
         </is>
@@ -3090,7 +2977,7 @@
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>Xong trong Tháng 11</t>
+          <t>Tháng 10 - Tháng 11</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
@@ -3103,7 +2990,7 @@
           <t>LongNH156, SonLN11</t>
         </is>
       </c>
-      <c r="G13" s="24" t="inlineStr">
+      <c r="G13" s="22" t="inlineStr">
         <is>
           <t>Config được trên CMS Rule: Page active, section, block, card active</t>
         </is>
@@ -3127,7 +3014,7 @@
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Xong trong Tháng 11</t>
+          <t>Tháng 11</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
@@ -3140,7 +3027,7 @@
           <t>ThuyTT104</t>
         </is>
       </c>
-      <c r="G14" s="24" t="inlineStr">
+      <c r="G14" s="22" t="inlineStr">
         <is>
           <t>Tích hợp bộ rule Cập nhật use case - UIUX</t>
         </is>
@@ -3164,7 +3051,7 @@
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>Xong trong Tháng 11</t>
+          <t>Tháng 11</t>
         </is>
       </c>
       <c r="E15" s="11" t="inlineStr">
@@ -3177,7 +3064,7 @@
           <t>ThuyTT104</t>
         </is>
       </c>
-      <c r="G15" s="24" t="inlineStr">
+      <c r="G15" s="22" t="inlineStr">
         <is>
           <t>Tích hợp QLCS - PDH về luồng quà tặngUpdate UIUX</t>
         </is>
@@ -3201,7 +3088,7 @@
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Xong trong Tháng 11</t>
+          <t>Tháng 11</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
@@ -3214,7 +3101,7 @@
           <t>ThuyTT104, LongNH156</t>
         </is>
       </c>
-      <c r="G16" s="24" t="inlineStr">
+      <c r="G16" s="22" t="inlineStr">
         <is>
           <t>Thiết kế UIUX mới về các section Quy hoạch lại bộ thư viên section để mở rộng lựa chọn cho vận hành sử dụng template Tích hợp SEO vào quản lý khi tạo LDP</t>
         </is>
@@ -3238,7 +3125,7 @@
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>Xong trong Tháng 11</t>
+          <t>Tháng 11</t>
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr">
@@ -3251,7 +3138,7 @@
           <t>ThuyTT104</t>
         </is>
       </c>
-      <c r="G17" s="24" t="inlineStr"/>
+      <c r="G17" s="22" t="inlineStr"/>
     </row>
     <row r="18" ht="38" customHeight="1">
       <c r="A18" s="11" t="inlineStr">
@@ -3271,7 +3158,7 @@
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Xong trong Tháng 12</t>
+          <t>Tháng 11 - Tháng 12</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
@@ -3284,7 +3171,7 @@
           <t>ThuyTT104</t>
         </is>
       </c>
-      <c r="G18" s="24" t="inlineStr">
+      <c r="G18" s="22" t="inlineStr">
         <is>
           <t>Tạo luồng giỏ hàng cho các sp: Sku/SACho phép người dùng add on nhiều sp cùng 1 giỏ hàng để thực hiện thanh toán</t>
         </is>
@@ -3308,7 +3195,7 @@
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>Xong trong Tháng 12</t>
+          <t>Tháng 11 - Tháng 12</t>
         </is>
       </c>
       <c r="E19" s="11" t="inlineStr">
@@ -3321,7 +3208,7 @@
           <t>SonLN11</t>
         </is>
       </c>
-      <c r="G19" s="24" t="inlineStr">
+      <c r="G19" s="22" t="inlineStr">
         <is>
           <t>Quy hoạch toàn bộ tin tức quản lý trên CMS source mới Impro tính năng bổ trợ cho BTV</t>
         </is>
@@ -3345,7 +3232,7 @@
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Xong trong Tháng 12</t>
+          <t>Tháng 11 - Tháng 12</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
@@ -3358,7 +3245,7 @@
           <t>SonLN11</t>
         </is>
       </c>
-      <c r="G20" s="24" t="inlineStr">
+      <c r="G20" s="22" t="inlineStr">
         <is>
           <t>Bổ sung bộ config profile cho tác giả trên website Quy hoạch bài viết theo tác giả</t>
         </is>
@@ -3382,7 +3269,7 @@
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>Xong trong Tháng 12</t>
+          <t>Tháng 12</t>
         </is>
       </c>
       <c r="E21" s="11" t="inlineStr">
@@ -3395,7 +3282,7 @@
           <t>ThuyTT104</t>
         </is>
       </c>
-      <c r="G21" s="24" t="inlineStr">
+      <c r="G21" s="22" t="inlineStr">
         <is>
           <t>https://fpt.vn/shop/s/khuyen-mai-wifihttps://fpt.vn/shop/s/dang-ky-wifihttps://fpt.vn/lap-wifihttps://fpt.vn/lap-internethttps://fpt.vn/uu-dai-internethttps://fpt.vn/lap-mang-wifihttps://fpt.vn/lap-mang-fpthttps://fpt.vn/lap-dat-internet</t>
         </is>
@@ -3419,7 +3306,7 @@
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Xong trong Tháng 12</t>
+          <t>Tháng 12</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
@@ -3432,7 +3319,7 @@
           <t>ThuyTT104</t>
         </is>
       </c>
-      <c r="G22" s="24" t="inlineStr">
+      <c r="G22" s="22" t="inlineStr">
         <is>
           <t>Trên trang https://beta.fpt.vn/ bổ sung trang "Combo Internet Camera" có nội dung tương tự trang https://fpt.vn/truyen-hinh-fpt-play URL Trang: https://beta.fpt.vn/combo-internet-camera</t>
         </is>
@@ -3456,7 +3343,7 @@
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>Xong trong Tháng 12</t>
+          <t>Tháng 12</t>
         </is>
       </c>
       <c r="E23" s="11" t="inlineStr">
@@ -3469,7 +3356,7 @@
           <t>ThuyTT104</t>
         </is>
       </c>
-      <c r="G23" s="24" t="inlineStr">
+      <c r="G23" s="22" t="inlineStr">
         <is>
           <t>Config CMS, Cấu hình rule riêng, UIUX</t>
         </is>
@@ -3493,7 +3380,7 @@
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Xong trong Tháng 12</t>
+          <t>Tháng 12</t>
         </is>
       </c>
       <c r="E24" s="11" t="inlineStr">
@@ -3506,7 +3393,7 @@
           <t>ThuyTT104</t>
         </is>
       </c>
-      <c r="G24" s="24" t="inlineStr">
+      <c r="G24" s="22" t="inlineStr">
         <is>
           <t>Config CMS, Cấu hình rule riêng, UIUX</t>
         </is>
@@ -3530,7 +3417,7 @@
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>Xong trong Tháng 12</t>
+          <t>Tháng 12</t>
         </is>
       </c>
       <c r="E25" s="11" t="inlineStr">
@@ -3543,7 +3430,7 @@
           <t>SonLN11</t>
         </is>
       </c>
-      <c r="G25" s="24" t="inlineStr">
+      <c r="G25" s="22" t="inlineStr">
         <is>
           <t>Config CMS, Cấu hình rule riêng, UIUX</t>
         </is>
@@ -3567,7 +3454,7 @@
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Xong trong Tháng 12</t>
+          <t>Tháng 12</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr">
@@ -3580,7 +3467,7 @@
           <t>SonLN11</t>
         </is>
       </c>
-      <c r="G26" s="24" t="inlineStr">
+      <c r="G26" s="22" t="inlineStr">
         <is>
           <t>Config CMS, tích hợp API FPL về lịch thi đấu, BXH</t>
         </is>
@@ -3604,7 +3491,7 @@
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>Xong trong Tháng 12</t>
+          <t>Tháng 12</t>
         </is>
       </c>
       <c r="E27" s="11" t="inlineStr">
@@ -3617,7 +3504,7 @@
           <t>SonLN11</t>
         </is>
       </c>
-      <c r="G27" s="24" t="inlineStr">
+      <c r="G27" s="22" t="inlineStr">
         <is>
           <t>Config CMS, tích hợp API FPL về lịch thi đấu, BXH</t>
         </is>
@@ -3641,7 +3528,7 @@
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Xong trong Tháng 12</t>
+          <t>Tháng 12</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
@@ -3654,7 +3541,7 @@
           <t>SonLN11</t>
         </is>
       </c>
-      <c r="G28" s="24" t="inlineStr">
+      <c r="G28" s="22" t="inlineStr">
         <is>
           <t>Config CMS, tích hợp API FPL về lịch thi đấu, BXH</t>
         </is>

</xml_diff>

<commit_message>
style(roadmap): bo tag Xong T, tinh chinh khung card tung task sang trong chuan ban cu, tang chieu cao va phoi mau de nhin
</commit_message>
<xml_diff>
--- a/thuyttdoc/Roadmap_Website_CMS_Q4_2026.xlsx
+++ b/thuyttdoc/Roadmap_Website_CMS_Q4_2026.xlsx
@@ -53,13 +53,13 @@
     <font>
       <name val="Times New Roman"/>
       <b val="1"/>
-      <color rgb="003730A3"/>
+      <color rgb="004338CA"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Times New Roman"/>
       <b val="1"/>
-      <color rgb="006D28D9"/>
+      <color rgb="006B21A8"/>
       <sz val="10"/>
     </font>
     <font>
@@ -85,7 +85,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -142,32 +142,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DBEAFE"/>
-        <bgColor rgb="00DBEAFE"/>
+        <fgColor rgb="00EFF6FF"/>
+        <bgColor rgb="00EFF6FF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E0E7FF"/>
-        <bgColor rgb="00E0E7FF"/>
+        <fgColor rgb="00EEF2FF"/>
+        <bgColor rgb="00EEF2FF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EDE9FE"/>
-        <bgColor rgb="00EDE9FE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00CCFBF1"/>
-        <bgColor rgb="00CCFBF1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D1FAE5"/>
-        <bgColor rgb="00D1FAE5"/>
+        <fgColor rgb="00ECFDF5"/>
+        <bgColor rgb="00ECFDF5"/>
       </patternFill>
     </fill>
     <fill>
@@ -289,19 +277,19 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -778,10 +766,10 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="28" customHeight="1">
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>[US-12] [CMS] Quản lý trang | PIC: SonLN11 (🎯 Xong T10)</t>
+          <t>[US-12] [CMS] Quản lý trang | PIC: SonLN11 | UAT</t>
         </is>
       </c>
       <c r="B4" s="7" t="n"/>
@@ -796,10 +784,10 @@
       <c r="K4" s="9" t="n"/>
       <c r="L4" s="9" t="n"/>
     </row>
-    <row r="5" ht="28" customHeight="1">
+    <row r="5" ht="30" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>[US-13] [CMS] Quản lý section | PIC: SonLN11 (🎯 Xong T10)</t>
+          <t>[US-13] [CMS] Quản lý section | PIC: SonLN11 | UAT</t>
         </is>
       </c>
       <c r="B5" s="7" t="n"/>
@@ -814,10 +802,10 @@
       <c r="K5" s="9" t="n"/>
       <c r="L5" s="9" t="n"/>
     </row>
-    <row r="6" ht="28" customHeight="1">
+    <row r="6" ht="30" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>[US-14] [CMS] Quản lý Block | PIC: SonLN11 (🎯 Xong T10)</t>
+          <t>[US-14] [CMS] Quản lý Block | PIC: SonLN11 | UAT</t>
         </is>
       </c>
       <c r="B6" s="7" t="n"/>
@@ -832,11 +820,11 @@
       <c r="K6" s="9" t="n"/>
       <c r="L6" s="9" t="n"/>
     </row>
-    <row r="7" ht="28" customHeight="1">
+    <row r="7" ht="30" customHeight="1">
       <c r="A7" s="10" t="n"/>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>[US-15] [CMS] Quản lý menu | PIC: SonLN11 (🎯 Xong T10)</t>
+          <t>[US-15] [CMS] Quản lý menu | PIC: SonLN11 | UAT</t>
         </is>
       </c>
       <c r="C7" s="7" t="n"/>
@@ -850,10 +838,10 @@
       <c r="K7" s="9" t="n"/>
       <c r="L7" s="9" t="n"/>
     </row>
-    <row r="8" ht="28" customHeight="1">
+    <row r="8" ht="30" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>[US-MENU] [Web, CMS] MENU (Cấp API Web/HiFPT &amp; Đồng bộ SPDV) | PIC: ThuyTT104 (🎯 Xong T10)</t>
+          <t>[US-MENU] [Web, CMS] MENU (Cấp API Web/HiFPT &amp; Đồng bộ SPDV) | PIC: ThuyTT104 | DEV</t>
         </is>
       </c>
       <c r="B8" s="7" t="n"/>
@@ -868,11 +856,11 @@
       <c r="K8" s="9" t="n"/>
       <c r="L8" s="9" t="n"/>
     </row>
-    <row r="9" ht="28" customHeight="1">
+    <row r="9" ht="30" customHeight="1">
       <c r="A9" s="10" t="n"/>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>[US-18] [CMS, Web] Quản lý FAQ: Quy hoạch lại UI/UX &amp; luồng cấu hình (Danh sách/Danh mục FAQ) | PIC: SonLN11 (🎯 Xong T11)</t>
+          <t>[US-18] [CMS, Web] Quản lý FAQ: Quy hoạch lại UI/UX &amp; luồng cấu hình (Danh sách/Danh mục FAQ) | PIC: SonLN11 | Phân tích</t>
         </is>
       </c>
       <c r="C9" s="12" t="n"/>
@@ -886,11 +874,11 @@
       <c r="K9" s="9" t="n"/>
       <c r="L9" s="9" t="n"/>
     </row>
-    <row r="10" ht="28" customHeight="1">
+    <row r="10" ht="30" customHeight="1">
       <c r="A10" s="10" t="n"/>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>[US-20] [CMS, Web] Quản lý quảng cáo | PIC: LongNH156 (🎯 Xong T11)</t>
+          <t>[US-20] [CMS, Web] Quản lý quảng cáo | PIC: LongNH156 | Phân tích</t>
         </is>
       </c>
       <c r="C10" s="12" t="n"/>
@@ -904,12 +892,12 @@
       <c r="K10" s="9" t="n"/>
       <c r="L10" s="9" t="n"/>
     </row>
-    <row r="11" ht="28" customHeight="1">
+    <row r="11" ht="30" customHeight="1">
       <c r="A11" s="10" t="n"/>
       <c r="B11" s="10" t="n"/>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>[US-21] [Web] Report: Ghi nhận thông tin báo cáo phase 2 - bộ báo cáo chuẩn cho ĐKOL | PIC: ThuyTT104 (🎯 Xong T11)</t>
+          <t>[US-21] [Web] Report: Ghi nhận thông tin báo cáo phase 2 - bộ báo cáo chuẩn cho ĐKOL | PIC: ThuyTT104 | Đang làm</t>
         </is>
       </c>
       <c r="D11" s="12" t="n"/>
@@ -922,11 +910,11 @@
       <c r="K11" s="9" t="n"/>
       <c r="L11" s="9" t="n"/>
     </row>
-    <row r="12" ht="28" customHeight="1">
+    <row r="12" ht="30" customHeight="1">
       <c r="A12" s="10" t="n"/>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>[US-LDPLOCAL] [Web, CMS] CMS config LDP Local: Gắn location Tỉnh/Huyện, SEO &amp; Schema | PIC: ThuyTT104, LongNH156 (🎯 Xong T11)</t>
+          <t>[US-LDPLOCAL] [Web, CMS] CMS config LDP Local: Gắn location Tỉnh/Huyện, SEO &amp; Schema | PIC: ThuyTT104, LongNH156 | Phân tích</t>
         </is>
       </c>
       <c r="C12" s="12" t="n"/>
@@ -940,12 +928,12 @@
       <c r="K12" s="9" t="n"/>
       <c r="L12" s="9" t="n"/>
     </row>
-    <row r="13" ht="28" customHeight="1">
+    <row r="13" ht="30" customHeight="1">
       <c r="A13" s="10" t="n"/>
       <c r="B13" s="10" t="n"/>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>[US-30] [CMS, Web] Quản lý Breadcrumbs trên trang / Landing Page | PIC: LongNH156, SonLN11 (🎯 Xong T11)</t>
+          <t>[US-30] [CMS, Web] Quản lý Breadcrumbs trên trang / Landing Page | PIC: LongNH156, SonLN11 | Phân tích</t>
         </is>
       </c>
       <c r="D13" s="12" t="n"/>
@@ -958,14 +946,14 @@
       <c r="K13" s="9" t="n"/>
       <c r="L13" s="9" t="n"/>
     </row>
-    <row r="14" ht="28" customHeight="1">
+    <row r="14" ht="30" customHeight="1">
       <c r="A14" s="10" t="n"/>
       <c r="B14" s="10" t="n"/>
       <c r="C14" s="10" t="n"/>
       <c r="D14" s="10" t="n"/>
       <c r="E14" s="13" t="inlineStr">
         <is>
-          <t>[US-29] [CMS, Web] Quản lý URL | PIC: LongNH156, ThuyTT104 (🎯 Xong T11)</t>
+          <t>[US-29] [CMS, Web] Quản lý URL | PIC: LongNH156, ThuyTT104 | Phân tích</t>
         </is>
       </c>
       <c r="F14" s="14" t="n"/>
@@ -976,14 +964,14 @@
       <c r="K14" s="9" t="n"/>
       <c r="L14" s="9" t="n"/>
     </row>
-    <row r="15" ht="28" customHeight="1">
+    <row r="15" ht="30" customHeight="1">
       <c r="A15" s="10" t="n"/>
       <c r="B15" s="10" t="n"/>
       <c r="C15" s="10" t="n"/>
       <c r="D15" s="10" t="n"/>
       <c r="E15" s="13" t="inlineStr">
         <is>
-          <t>[US-31] [Web] Luồng bán kèm PK (charm) Camera Play 4 trên website fpt.vn | PIC: ThuyTT104 (🎯 Xong T11)</t>
+          <t>[US-31] [Web] Luồng bán kèm PK (charm) Camera Play 4 trên website fpt.vn | PIC: ThuyTT104 | Đang làm</t>
         </is>
       </c>
       <c r="F15" s="14" t="n"/>
@@ -994,14 +982,14 @@
       <c r="K15" s="9" t="n"/>
       <c r="L15" s="9" t="n"/>
     </row>
-    <row r="16" ht="28" customHeight="1">
+    <row r="16" ht="30" customHeight="1">
       <c r="A16" s="10" t="n"/>
       <c r="B16" s="10" t="n"/>
       <c r="C16" s="10" t="n"/>
       <c r="D16" s="10" t="n"/>
       <c r="E16" s="13" t="inlineStr">
         <is>
-          <t>[US-32] [Web] Luồng quà tặng (Mũ bảo hiểm) trên website | PIC: ThuyTT104 (🎯 Xong T11)</t>
+          <t>[US-32] [Web] Luồng quà tặng (Mũ bảo hiểm) trên website | PIC: ThuyTT104 | Đang làm</t>
         </is>
       </c>
       <c r="F16" s="14" t="n"/>
@@ -1012,7 +1000,7 @@
       <c r="K16" s="9" t="n"/>
       <c r="L16" s="9" t="n"/>
     </row>
-    <row r="17" ht="28" customHeight="1">
+    <row r="17" ht="30" customHeight="1">
       <c r="A17" s="10" t="n"/>
       <c r="B17" s="10" t="n"/>
       <c r="C17" s="10" t="n"/>
@@ -1020,7 +1008,7 @@
       <c r="E17" s="8" t="n"/>
       <c r="F17" s="13" t="inlineStr">
         <is>
-          <t>[US-33] [CMS, Web] Xây dựng thư viện section mở rộng cho tạo LDP kéo thả | PIC: ThuyTT104, LongNH156 (🎯 Xong T11)</t>
+          <t>[US-33] [CMS, Web] Xây dựng thư viện section mở rộng cho tạo LDP kéo thả | PIC: ThuyTT104, LongNH156 | Đang làm</t>
         </is>
       </c>
       <c r="G17" s="14" t="n"/>
@@ -1030,7 +1018,7 @@
       <c r="K17" s="9" t="n"/>
       <c r="L17" s="9" t="n"/>
     </row>
-    <row r="18" ht="28" customHeight="1">
+    <row r="18" ht="30" customHeight="1">
       <c r="A18" s="10" t="n"/>
       <c r="B18" s="10" t="n"/>
       <c r="C18" s="10" t="n"/>
@@ -1038,7 +1026,7 @@
       <c r="E18" s="8" t="n"/>
       <c r="F18" s="13" t="inlineStr">
         <is>
-          <t>[US-28] [Web] [FMI Phase 4 | NBA] Phối hợp tích hợp Trigger Popup &amp; Web Push trên fpt.vn | PIC: ThuyTT104 (🎯 Xong T11)</t>
+          <t>[US-28] [Web] [FMI Phase 4 | NBA] Phối hợp tích hợp Trigger Popup &amp; Web Push trên fpt.vn | PIC: ThuyTT104 | Phân tích</t>
         </is>
       </c>
       <c r="G18" s="14" t="n"/>
@@ -1048,14 +1036,14 @@
       <c r="K18" s="9" t="n"/>
       <c r="L18" s="9" t="n"/>
     </row>
-    <row r="19" ht="28" customHeight="1">
+    <row r="19" ht="30" customHeight="1">
       <c r="A19" s="10" t="n"/>
       <c r="B19" s="10" t="n"/>
       <c r="C19" s="10" t="n"/>
       <c r="D19" s="10" t="n"/>
       <c r="E19" s="15" t="inlineStr">
         <is>
-          <t>[US-47] [Web] Luồng giỏ hàng trên kênh (Unified Cart) | PIC: ThuyTT104 (🎯 Xong T12)</t>
+          <t>[US-47] [Web] Luồng giỏ hàng trên kênh (Unified Cart) | PIC: ThuyTT104 | Phân tích</t>
         </is>
       </c>
       <c r="F19" s="16" t="n"/>
@@ -1066,7 +1054,7 @@
       <c r="K19" s="16" t="n"/>
       <c r="L19" s="16" t="n"/>
     </row>
-    <row r="20" ht="28" customHeight="1">
+    <row r="20" ht="30" customHeight="1">
       <c r="A20" s="10" t="n"/>
       <c r="B20" s="10" t="n"/>
       <c r="C20" s="10" t="n"/>
@@ -1074,7 +1062,7 @@
       <c r="E20" s="8" t="n"/>
       <c r="F20" s="15" t="inlineStr">
         <is>
-          <t>[US-36] [CMS, Web] Quản lý tin tức | PIC: SonLN11 (🎯 Xong T12)</t>
+          <t>[US-36] [CMS, Web] Quản lý tin tức | PIC: SonLN11 | Phân tích</t>
         </is>
       </c>
       <c r="G20" s="16" t="n"/>
@@ -1084,7 +1072,7 @@
       <c r="K20" s="16" t="n"/>
       <c r="L20" s="9" t="n"/>
     </row>
-    <row r="21" ht="28" customHeight="1">
+    <row r="21" ht="30" customHeight="1">
       <c r="A21" s="10" t="n"/>
       <c r="B21" s="10" t="n"/>
       <c r="C21" s="10" t="n"/>
@@ -1092,7 +1080,7 @@
       <c r="E21" s="8" t="n"/>
       <c r="F21" s="15" t="inlineStr">
         <is>
-          <t>[US-37] [CMS] Quản lý Profile Tác giả | PIC: SonLN11 (🎯 Xong T12)</t>
+          <t>[US-37] [CMS] Quản lý Profile Tác giả | PIC: SonLN11 | Phân tích</t>
         </is>
       </c>
       <c r="G21" s="16" t="n"/>
@@ -1102,7 +1090,7 @@
       <c r="K21" s="16" t="n"/>
       <c r="L21" s="9" t="n"/>
     </row>
-    <row r="22" ht="28" customHeight="1">
+    <row r="22" ht="30" customHeight="1">
       <c r="A22" s="10" t="n"/>
       <c r="B22" s="10" t="n"/>
       <c r="C22" s="10" t="n"/>
@@ -1113,14 +1101,14 @@
       <c r="H22" s="8" t="n"/>
       <c r="I22" s="17" t="inlineStr">
         <is>
-          <t>[US-26] [Web, CMS] Các link chạy ads team Performance chạy ads - quy hoạch về CMS mới | PIC: ThuyTT104 (🎯 Xong T12)</t>
+          <t>[US-26] [Web, CMS] Các link chạy ads team Performance chạy ads - quy hoạch về CMS mới | PIC: ThuyTT104 | Mới</t>
         </is>
       </c>
       <c r="J22" s="18" t="n"/>
       <c r="K22" s="18" t="n"/>
       <c r="L22" s="9" t="n"/>
     </row>
-    <row r="23" ht="28" customHeight="1">
+    <row r="23" ht="30" customHeight="1">
       <c r="A23" s="10" t="n"/>
       <c r="B23" s="10" t="n"/>
       <c r="C23" s="10" t="n"/>
@@ -1131,14 +1119,14 @@
       <c r="H23" s="8" t="n"/>
       <c r="I23" s="17" t="inlineStr">
         <is>
-          <t>[US-27] [CMS, Web] Bổ sung trang Combo Internet Camera | PIC: ThuyTT104 (🎯 Xong T12)</t>
+          <t>[US-27] [CMS, Web] Bổ sung trang Combo Internet Camera | PIC: ThuyTT104 | Mới</t>
         </is>
       </c>
       <c r="J23" s="18" t="n"/>
       <c r="K23" s="18" t="n"/>
       <c r="L23" s="18" t="n"/>
     </row>
-    <row r="24" ht="28" customHeight="1">
+    <row r="24" ht="30" customHeight="1">
       <c r="A24" s="10" t="n"/>
       <c r="B24" s="10" t="n"/>
       <c r="C24" s="10" t="n"/>
@@ -1149,14 +1137,14 @@
       <c r="H24" s="8" t="n"/>
       <c r="I24" s="17" t="inlineStr">
         <is>
-          <t>[US-38] [Web, CMS] Trang LDP CSCA | PIC: ThuyTT104 (🎯 Xong T12)</t>
+          <t>[US-38] [Web, CMS] Trang LDP CSCA | PIC: ThuyTT104 | Mới</t>
         </is>
       </c>
       <c r="J24" s="18" t="n"/>
       <c r="K24" s="18" t="n"/>
       <c r="L24" s="18" t="n"/>
     </row>
-    <row r="25" ht="28" customHeight="1">
+    <row r="25" ht="30" customHeight="1">
       <c r="A25" s="10" t="n"/>
       <c r="B25" s="10" t="n"/>
       <c r="C25" s="10" t="n"/>
@@ -1167,14 +1155,14 @@
       <c r="H25" s="8" t="n"/>
       <c r="I25" s="17" t="inlineStr">
         <is>
-          <t>[US-39] [Web, CMS] Trang LDP Fcitizen | PIC: ThuyTT104 (🎯 Xong T12)</t>
+          <t>[US-39] [Web, CMS] Trang LDP Fcitizen | PIC: ThuyTT104 | Mới</t>
         </is>
       </c>
       <c r="J25" s="18" t="n"/>
       <c r="K25" s="18" t="n"/>
       <c r="L25" s="18" t="n"/>
     </row>
-    <row r="26" ht="28" customHeight="1">
+    <row r="26" ht="30" customHeight="1">
       <c r="A26" s="10" t="n"/>
       <c r="B26" s="10" t="n"/>
       <c r="C26" s="10" t="n"/>
@@ -1185,14 +1173,14 @@
       <c r="H26" s="8" t="n"/>
       <c r="I26" s="17" t="inlineStr">
         <is>
-          <t>[US-40] [Web, CMS] Trang LDP Ngoại Hạng Anh (NHA) | PIC: SonLN11 (🎯 Xong T12)</t>
+          <t>[US-40] [Web, CMS] Trang LDP Ngoại Hạng Anh (NHA) | PIC: SonLN11 | Mới</t>
         </is>
       </c>
       <c r="J26" s="18" t="n"/>
       <c r="K26" s="18" t="n"/>
       <c r="L26" s="9" t="n"/>
     </row>
-    <row r="27" ht="28" customHeight="1">
+    <row r="27" ht="30" customHeight="1">
       <c r="A27" s="10" t="n"/>
       <c r="B27" s="10" t="n"/>
       <c r="C27" s="10" t="n"/>
@@ -1203,14 +1191,14 @@
       <c r="H27" s="8" t="n"/>
       <c r="I27" s="17" t="inlineStr">
         <is>
-          <t>[US-41] [Web, CMS] Trang LDP NHA - Lịch thi đấu | PIC: SonLN11 (🎯 Xong T12)</t>
+          <t>[US-41] [Web, CMS] Trang LDP NHA - Lịch thi đấu | PIC: SonLN11 | Mới</t>
         </is>
       </c>
       <c r="J27" s="18" t="n"/>
       <c r="K27" s="18" t="n"/>
       <c r="L27" s="18" t="n"/>
     </row>
-    <row r="28" ht="28" customHeight="1">
+    <row r="28" ht="30" customHeight="1">
       <c r="A28" s="10" t="n"/>
       <c r="B28" s="10" t="n"/>
       <c r="C28" s="10" t="n"/>
@@ -1221,14 +1209,14 @@
       <c r="H28" s="8" t="n"/>
       <c r="I28" s="17" t="inlineStr">
         <is>
-          <t>[US-42] [Web, CMS] Trang LDP NHA - Bảng xếp hạng | PIC: SonLN11 (🎯 Xong T12)</t>
+          <t>[US-42] [Web, CMS] Trang LDP NHA - Bảng xếp hạng | PIC: SonLN11 | Mới</t>
         </is>
       </c>
       <c r="J28" s="18" t="n"/>
       <c r="K28" s="18" t="n"/>
       <c r="L28" s="18" t="n"/>
     </row>
-    <row r="29" ht="28" customHeight="1">
+    <row r="29" ht="30" customHeight="1">
       <c r="A29" s="10" t="n"/>
       <c r="B29" s="10" t="n"/>
       <c r="C29" s="10" t="n"/>
@@ -1239,7 +1227,7 @@
       <c r="H29" s="8" t="n"/>
       <c r="I29" s="17" t="inlineStr">
         <is>
-          <t>[US-43] [Web, CMS] Trang LDP NHA - SA | PIC: SonLN11 (🎯 Xong T12)</t>
+          <t>[US-43] [Web, CMS] Trang LDP NHA - SA | PIC: SonLN11 | Mới</t>
         </is>
       </c>
       <c r="J29" s="18" t="n"/>
@@ -1346,7 +1334,7 @@
       </c>
       <c r="I1" s="19" t="inlineStr">
         <is>
-          <t>Tháng Cán Đích</t>
+          <t>Tháng Hoàn Thành</t>
         </is>
       </c>
     </row>
@@ -1391,7 +1379,7 @@
       </c>
       <c r="I2" s="20" t="inlineStr">
         <is>
-          <t>Tháng 10 (🎯 Xong T10)</t>
+          <t>Tháng 10</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1424,7 @@
       </c>
       <c r="I3" s="20" t="inlineStr">
         <is>
-          <t>Tháng 10 (🎯 Xong T10)</t>
+          <t>Tháng 10</t>
         </is>
       </c>
     </row>
@@ -1481,7 +1469,7 @@
       </c>
       <c r="I4" s="20" t="inlineStr">
         <is>
-          <t>Tháng 10 (🎯 Xong T10)</t>
+          <t>Tháng 10</t>
         </is>
       </c>
     </row>
@@ -1526,7 +1514,7 @@
       </c>
       <c r="I5" s="20" t="inlineStr">
         <is>
-          <t>Tháng 10 (🎯 Xong T10)</t>
+          <t>Tháng 10</t>
         </is>
       </c>
     </row>
@@ -1571,7 +1559,7 @@
       </c>
       <c r="I6" s="20" t="inlineStr">
         <is>
-          <t>Tháng 10 (🎯 Xong T10)</t>
+          <t>Tháng 10</t>
         </is>
       </c>
     </row>
@@ -1616,7 +1604,7 @@
       </c>
       <c r="I7" s="20" t="inlineStr">
         <is>
-          <t>Tháng 11 (🎯 Xong T11)</t>
+          <t>Tháng 11</t>
         </is>
       </c>
     </row>
@@ -1661,7 +1649,7 @@
       </c>
       <c r="I8" s="20" t="inlineStr">
         <is>
-          <t>Tháng 11 (🎯 Xong T11)</t>
+          <t>Tháng 11</t>
         </is>
       </c>
     </row>
@@ -1706,7 +1694,7 @@
       </c>
       <c r="I9" s="20" t="inlineStr">
         <is>
-          <t>Tháng 11 (🎯 Xong T11)</t>
+          <t>Tháng 11</t>
         </is>
       </c>
     </row>
@@ -1751,7 +1739,7 @@
       </c>
       <c r="I10" s="20" t="inlineStr">
         <is>
-          <t>Tháng 11 (🎯 Xong T11)</t>
+          <t>Tháng 11</t>
         </is>
       </c>
     </row>
@@ -1796,7 +1784,7 @@
       </c>
       <c r="I11" s="20" t="inlineStr">
         <is>
-          <t>Tháng 11 (🎯 Xong T11)</t>
+          <t>Tháng 11</t>
         </is>
       </c>
     </row>
@@ -1841,7 +1829,7 @@
       </c>
       <c r="I12" s="20" t="inlineStr">
         <is>
-          <t>Tháng 11 (🎯 Xong T11)</t>
+          <t>Tháng 11</t>
         </is>
       </c>
     </row>
@@ -1886,7 +1874,7 @@
       </c>
       <c r="I13" s="20" t="inlineStr">
         <is>
-          <t>Tháng 11 (🎯 Xong T11)</t>
+          <t>Tháng 11</t>
         </is>
       </c>
     </row>
@@ -1931,7 +1919,7 @@
       </c>
       <c r="I14" s="20" t="inlineStr">
         <is>
-          <t>Tháng 11 (🎯 Xong T11)</t>
+          <t>Tháng 11</t>
         </is>
       </c>
     </row>
@@ -1976,7 +1964,7 @@
       </c>
       <c r="I15" s="20" t="inlineStr">
         <is>
-          <t>Tháng 11 (🎯 Xong T11)</t>
+          <t>Tháng 11</t>
         </is>
       </c>
     </row>
@@ -2021,7 +2009,7 @@
       </c>
       <c r="I16" s="20" t="inlineStr">
         <is>
-          <t>Tháng 11 (🎯 Xong T11)</t>
+          <t>Tháng 11</t>
         </is>
       </c>
     </row>
@@ -2066,7 +2054,7 @@
       </c>
       <c r="I17" s="20" t="inlineStr">
         <is>
-          <t>Tháng 12 (🎯 Xong T12)</t>
+          <t>Tháng 12</t>
         </is>
       </c>
     </row>
@@ -2111,7 +2099,7 @@
       </c>
       <c r="I18" s="20" t="inlineStr">
         <is>
-          <t>Tháng 12 (🎯 Xong T12)</t>
+          <t>Tháng 12</t>
         </is>
       </c>
     </row>
@@ -2156,7 +2144,7 @@
       </c>
       <c r="I19" s="20" t="inlineStr">
         <is>
-          <t>Tháng 12 (🎯 Xong T12)</t>
+          <t>Tháng 12</t>
         </is>
       </c>
     </row>
@@ -2201,7 +2189,7 @@
       </c>
       <c r="I20" s="20" t="inlineStr">
         <is>
-          <t>Tháng 12 (🎯 Xong T12)</t>
+          <t>Tháng 12</t>
         </is>
       </c>
     </row>
@@ -2246,7 +2234,7 @@
       </c>
       <c r="I21" s="20" t="inlineStr">
         <is>
-          <t>Tháng 12 (🎯 Xong T12)</t>
+          <t>Tháng 12</t>
         </is>
       </c>
     </row>
@@ -2291,7 +2279,7 @@
       </c>
       <c r="I22" s="20" t="inlineStr">
         <is>
-          <t>Tháng 12 (🎯 Xong T12)</t>
+          <t>Tháng 12</t>
         </is>
       </c>
     </row>
@@ -2336,7 +2324,7 @@
       </c>
       <c r="I23" s="20" t="inlineStr">
         <is>
-          <t>Tháng 12 (🎯 Xong T12)</t>
+          <t>Tháng 12</t>
         </is>
       </c>
     </row>
@@ -2381,7 +2369,7 @@
       </c>
       <c r="I24" s="20" t="inlineStr">
         <is>
-          <t>Tháng 12 (🎯 Xong T12)</t>
+          <t>Tháng 12</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2414,7 @@
       </c>
       <c r="I25" s="20" t="inlineStr">
         <is>
-          <t>Tháng 12 (🎯 Xong T12)</t>
+          <t>Tháng 12</t>
         </is>
       </c>
     </row>
@@ -2471,7 +2459,7 @@
       </c>
       <c r="I26" s="20" t="inlineStr">
         <is>
-          <t>Tháng 12 (🎯 Xong T12)</t>
+          <t>Tháng 12</t>
         </is>
       </c>
     </row>
@@ -2516,7 +2504,7 @@
       </c>
       <c r="I27" s="20" t="inlineStr">
         <is>
-          <t>Tháng 12 (🎯 Xong T12)</t>
+          <t>Tháng 12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(roadmap): bo US, dua PIC xuong dong 2, do uu tien cuoi dong 1, hien thi ty le phan tram mau gradient theo status
</commit_message>
<xml_diff>
--- a/thuyttdoc/Roadmap_Website_CMS_Q4_2026.xlsx
+++ b/thuyttdoc/Roadmap_Website_CMS_Q4_2026.xlsx
@@ -766,10 +766,11 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="30" customHeight="1">
+    <row r="4" ht="36" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>[US-12] [CMS] Quản lý trang | PIC: SonLN11 | UAT</t>
+          <t>[CMS] Quản lý trang (P2)
+PIC: SonLN11 | UAT (90%)</t>
         </is>
       </c>
       <c r="B4" s="7" t="n"/>
@@ -784,10 +785,11 @@
       <c r="K4" s="9" t="n"/>
       <c r="L4" s="9" t="n"/>
     </row>
-    <row r="5" ht="30" customHeight="1">
+    <row r="5" ht="36" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>[US-13] [CMS] Quản lý section | PIC: SonLN11 | UAT</t>
+          <t>[CMS] Quản lý section (P2)
+PIC: SonLN11 | UAT (90%)</t>
         </is>
       </c>
       <c r="B5" s="7" t="n"/>
@@ -802,10 +804,11 @@
       <c r="K5" s="9" t="n"/>
       <c r="L5" s="9" t="n"/>
     </row>
-    <row r="6" ht="30" customHeight="1">
+    <row r="6" ht="36" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>[US-14] [CMS] Quản lý Block | PIC: SonLN11 | UAT</t>
+          <t>[CMS] Quản lý Block (P2)
+PIC: SonLN11 | UAT (90%)</t>
         </is>
       </c>
       <c r="B6" s="7" t="n"/>
@@ -820,11 +823,12 @@
       <c r="K6" s="9" t="n"/>
       <c r="L6" s="9" t="n"/>
     </row>
-    <row r="7" ht="30" customHeight="1">
+    <row r="7" ht="36" customHeight="1">
       <c r="A7" s="10" t="n"/>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>[US-15] [CMS] Quản lý menu | PIC: SonLN11 | UAT</t>
+          <t>[CMS] Quản lý menu (P2)
+PIC: SonLN11 | UAT (90%)</t>
         </is>
       </c>
       <c r="C7" s="7" t="n"/>
@@ -838,10 +842,11 @@
       <c r="K7" s="9" t="n"/>
       <c r="L7" s="9" t="n"/>
     </row>
-    <row r="8" ht="30" customHeight="1">
+    <row r="8" ht="36" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>[US-MENU] [Web, CMS] MENU (Cấp API Web/HiFPT &amp; Đồng bộ SPDV) | PIC: ThuyTT104 | DEV</t>
+          <t>[Web, CMS] MENU (Cấp API Web/HiFPT &amp; Đồng bộ SPDV) (P1)
+PIC: ThuyTT104 | DEV (60%)</t>
         </is>
       </c>
       <c r="B8" s="7" t="n"/>
@@ -856,11 +861,12 @@
       <c r="K8" s="9" t="n"/>
       <c r="L8" s="9" t="n"/>
     </row>
-    <row r="9" ht="30" customHeight="1">
+    <row r="9" ht="36" customHeight="1">
       <c r="A9" s="10" t="n"/>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>[US-18] [CMS, Web] Quản lý FAQ: Quy hoạch lại UI/UX &amp; luồng cấu hình (Danh sách/Danh mục FAQ) | PIC: SonLN11 | Phân tích</t>
+          <t>[CMS, Web] Quản lý FAQ: Quy hoạch lại UI/UX &amp; luồng cấu hình (Danh sách/Danh mục FAQ) (P2)
+PIC: SonLN11 | Phân tích (35%)</t>
         </is>
       </c>
       <c r="C9" s="12" t="n"/>
@@ -874,11 +880,12 @@
       <c r="K9" s="9" t="n"/>
       <c r="L9" s="9" t="n"/>
     </row>
-    <row r="10" ht="30" customHeight="1">
+    <row r="10" ht="36" customHeight="1">
       <c r="A10" s="10" t="n"/>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>[US-20] [CMS, Web] Quản lý quảng cáo | PIC: LongNH156 | Phân tích</t>
+          <t>[CMS, Web] Quản lý quảng cáo (P1)
+PIC: LongNH156 | Phân tích (30%)</t>
         </is>
       </c>
       <c r="C10" s="12" t="n"/>
@@ -892,12 +899,13 @@
       <c r="K10" s="9" t="n"/>
       <c r="L10" s="9" t="n"/>
     </row>
-    <row r="11" ht="30" customHeight="1">
+    <row r="11" ht="36" customHeight="1">
       <c r="A11" s="10" t="n"/>
       <c r="B11" s="10" t="n"/>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>[US-21] [Web] Report: Ghi nhận thông tin báo cáo phase 2 - bộ báo cáo chuẩn cho ĐKOL | PIC: ThuyTT104 | Đang làm</t>
+          <t>[Web] Report: Ghi nhận thông tin báo cáo phase 2 - bộ báo cáo chuẩn cho ĐKOL (P1)
+PIC: ThuyTT104 | Đang làm (55%)</t>
         </is>
       </c>
       <c r="D11" s="12" t="n"/>
@@ -910,11 +918,12 @@
       <c r="K11" s="9" t="n"/>
       <c r="L11" s="9" t="n"/>
     </row>
-    <row r="12" ht="30" customHeight="1">
+    <row r="12" ht="36" customHeight="1">
       <c r="A12" s="10" t="n"/>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>[US-LDPLOCAL] [Web, CMS] CMS config LDP Local: Gắn location Tỉnh/Huyện, SEO &amp; Schema | PIC: ThuyTT104, LongNH156 | Phân tích</t>
+          <t>[Web, CMS] CMS config LDP Local: Gắn location Tỉnh/Huyện, SEO &amp; Schema (P1)
+PIC: ThuyTT104, LongNH156 | Phân tích (35%)</t>
         </is>
       </c>
       <c r="C12" s="12" t="n"/>
@@ -928,12 +937,13 @@
       <c r="K12" s="9" t="n"/>
       <c r="L12" s="9" t="n"/>
     </row>
-    <row r="13" ht="30" customHeight="1">
+    <row r="13" ht="36" customHeight="1">
       <c r="A13" s="10" t="n"/>
       <c r="B13" s="10" t="n"/>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>[US-30] [CMS, Web] Quản lý Breadcrumbs trên trang / Landing Page | PIC: LongNH156, SonLN11 | Phân tích</t>
+          <t>[CMS, Web] Quản lý Breadcrumbs trên trang / Landing Page (P1)
+PIC: LongNH156, SonLN11 | Phân tích (30%)</t>
         </is>
       </c>
       <c r="D13" s="12" t="n"/>
@@ -946,14 +956,15 @@
       <c r="K13" s="9" t="n"/>
       <c r="L13" s="9" t="n"/>
     </row>
-    <row r="14" ht="30" customHeight="1">
+    <row r="14" ht="36" customHeight="1">
       <c r="A14" s="10" t="n"/>
       <c r="B14" s="10" t="n"/>
       <c r="C14" s="10" t="n"/>
       <c r="D14" s="10" t="n"/>
       <c r="E14" s="13" t="inlineStr">
         <is>
-          <t>[US-29] [CMS, Web] Quản lý URL | PIC: LongNH156, ThuyTT104 | Phân tích</t>
+          <t>[CMS, Web] Quản lý URL (P2)
+PIC: LongNH156, ThuyTT104 | Phân tích (30%)</t>
         </is>
       </c>
       <c r="F14" s="14" t="n"/>
@@ -964,14 +975,15 @@
       <c r="K14" s="9" t="n"/>
       <c r="L14" s="9" t="n"/>
     </row>
-    <row r="15" ht="30" customHeight="1">
+    <row r="15" ht="36" customHeight="1">
       <c r="A15" s="10" t="n"/>
       <c r="B15" s="10" t="n"/>
       <c r="C15" s="10" t="n"/>
       <c r="D15" s="10" t="n"/>
       <c r="E15" s="13" t="inlineStr">
         <is>
-          <t>[US-31] [Web] Luồng bán kèm PK (charm) Camera Play 4 trên website fpt.vn | PIC: ThuyTT104 | Đang làm</t>
+          <t>[Web] Luồng bán kèm PK (charm) Camera Play 4 trên website fpt.vn (P2)
+PIC: ThuyTT104 | Đang làm (55%)</t>
         </is>
       </c>
       <c r="F15" s="14" t="n"/>
@@ -982,14 +994,15 @@
       <c r="K15" s="9" t="n"/>
       <c r="L15" s="9" t="n"/>
     </row>
-    <row r="16" ht="30" customHeight="1">
+    <row r="16" ht="36" customHeight="1">
       <c r="A16" s="10" t="n"/>
       <c r="B16" s="10" t="n"/>
       <c r="C16" s="10" t="n"/>
       <c r="D16" s="10" t="n"/>
       <c r="E16" s="13" t="inlineStr">
         <is>
-          <t>[US-32] [Web] Luồng quà tặng (Mũ bảo hiểm) trên website | PIC: ThuyTT104 | Đang làm</t>
+          <t>[Web] Luồng quà tặng (Mũ bảo hiểm) trên website (P3)
+PIC: ThuyTT104 | Đang làm (50%)</t>
         </is>
       </c>
       <c r="F16" s="14" t="n"/>
@@ -1000,7 +1013,7 @@
       <c r="K16" s="9" t="n"/>
       <c r="L16" s="9" t="n"/>
     </row>
-    <row r="17" ht="30" customHeight="1">
+    <row r="17" ht="36" customHeight="1">
       <c r="A17" s="10" t="n"/>
       <c r="B17" s="10" t="n"/>
       <c r="C17" s="10" t="n"/>
@@ -1008,7 +1021,8 @@
       <c r="E17" s="8" t="n"/>
       <c r="F17" s="13" t="inlineStr">
         <is>
-          <t>[US-33] [CMS, Web] Xây dựng thư viện section mở rộng cho tạo LDP kéo thả | PIC: ThuyTT104, LongNH156 | Đang làm</t>
+          <t>[CMS, Web] Xây dựng thư viện section mở rộng cho tạo LDP kéo thả (P3)
+PIC: ThuyTT104, LongNH156 | Đang làm (50%)</t>
         </is>
       </c>
       <c r="G17" s="14" t="n"/>
@@ -1018,7 +1032,7 @@
       <c r="K17" s="9" t="n"/>
       <c r="L17" s="9" t="n"/>
     </row>
-    <row r="18" ht="30" customHeight="1">
+    <row r="18" ht="36" customHeight="1">
       <c r="A18" s="10" t="n"/>
       <c r="B18" s="10" t="n"/>
       <c r="C18" s="10" t="n"/>
@@ -1026,7 +1040,8 @@
       <c r="E18" s="8" t="n"/>
       <c r="F18" s="13" t="inlineStr">
         <is>
-          <t>[US-28] [Web] [FMI Phase 4 | NBA] Phối hợp tích hợp Trigger Popup &amp; Web Push trên fpt.vn | PIC: ThuyTT104 | Phân tích</t>
+          <t>[Web] [FMI Phase 4 | NBA] Phối hợp tích hợp Trigger Popup &amp; Web Push trên fpt.vn (P4)
+PIC: ThuyTT104 | Phân tích (25%)</t>
         </is>
       </c>
       <c r="G18" s="14" t="n"/>
@@ -1036,14 +1051,15 @@
       <c r="K18" s="9" t="n"/>
       <c r="L18" s="9" t="n"/>
     </row>
-    <row r="19" ht="30" customHeight="1">
+    <row r="19" ht="36" customHeight="1">
       <c r="A19" s="10" t="n"/>
       <c r="B19" s="10" t="n"/>
       <c r="C19" s="10" t="n"/>
       <c r="D19" s="10" t="n"/>
       <c r="E19" s="15" t="inlineStr">
         <is>
-          <t>[US-47] [Web] Luồng giỏ hàng trên kênh (Unified Cart) | PIC: ThuyTT104 | Phân tích</t>
+          <t>[Web] Luồng giỏ hàng trên kênh (Unified Cart) (P1)
+PIC: ThuyTT104 | Phân tích (35%)</t>
         </is>
       </c>
       <c r="F19" s="16" t="n"/>
@@ -1054,7 +1070,7 @@
       <c r="K19" s="16" t="n"/>
       <c r="L19" s="16" t="n"/>
     </row>
-    <row r="20" ht="30" customHeight="1">
+    <row r="20" ht="36" customHeight="1">
       <c r="A20" s="10" t="n"/>
       <c r="B20" s="10" t="n"/>
       <c r="C20" s="10" t="n"/>
@@ -1062,7 +1078,8 @@
       <c r="E20" s="8" t="n"/>
       <c r="F20" s="15" t="inlineStr">
         <is>
-          <t>[US-36] [CMS, Web] Quản lý tin tức | PIC: SonLN11 | Phân tích</t>
+          <t>[CMS, Web] Quản lý tin tức (P2)
+PIC: SonLN11 | Phân tích (30%)</t>
         </is>
       </c>
       <c r="G20" s="16" t="n"/>
@@ -1072,7 +1089,7 @@
       <c r="K20" s="16" t="n"/>
       <c r="L20" s="9" t="n"/>
     </row>
-    <row r="21" ht="30" customHeight="1">
+    <row r="21" ht="36" customHeight="1">
       <c r="A21" s="10" t="n"/>
       <c r="B21" s="10" t="n"/>
       <c r="C21" s="10" t="n"/>
@@ -1080,7 +1097,8 @@
       <c r="E21" s="8" t="n"/>
       <c r="F21" s="15" t="inlineStr">
         <is>
-          <t>[US-37] [CMS] Quản lý Profile Tác giả | PIC: SonLN11 | Phân tích</t>
+          <t>[CMS] Quản lý Profile Tác giả (P2)
+PIC: SonLN11 | Phân tích (30%)</t>
         </is>
       </c>
       <c r="G21" s="16" t="n"/>
@@ -1090,7 +1108,7 @@
       <c r="K21" s="16" t="n"/>
       <c r="L21" s="9" t="n"/>
     </row>
-    <row r="22" ht="30" customHeight="1">
+    <row r="22" ht="36" customHeight="1">
       <c r="A22" s="10" t="n"/>
       <c r="B22" s="10" t="n"/>
       <c r="C22" s="10" t="n"/>
@@ -1101,14 +1119,15 @@
       <c r="H22" s="8" t="n"/>
       <c r="I22" s="17" t="inlineStr">
         <is>
-          <t>[US-26] [Web, CMS] Các link chạy ads team Performance chạy ads - quy hoạch về CMS mới | PIC: ThuyTT104 | Mới</t>
+          <t>[Web, CMS] Các link chạy ads team Performance chạy ads - quy hoạch về CMS mới (P2)
+PIC: ThuyTT104 | Mới (15%)</t>
         </is>
       </c>
       <c r="J22" s="18" t="n"/>
       <c r="K22" s="18" t="n"/>
       <c r="L22" s="9" t="n"/>
     </row>
-    <row r="23" ht="30" customHeight="1">
+    <row r="23" ht="36" customHeight="1">
       <c r="A23" s="10" t="n"/>
       <c r="B23" s="10" t="n"/>
       <c r="C23" s="10" t="n"/>
@@ -1119,14 +1138,15 @@
       <c r="H23" s="8" t="n"/>
       <c r="I23" s="17" t="inlineStr">
         <is>
-          <t>[US-27] [CMS, Web] Bổ sung trang Combo Internet Camera | PIC: ThuyTT104 | Mới</t>
+          <t>[CMS, Web] Bổ sung trang Combo Internet Camera (P4)
+PIC: ThuyTT104 | Mới (15%)</t>
         </is>
       </c>
       <c r="J23" s="18" t="n"/>
       <c r="K23" s="18" t="n"/>
       <c r="L23" s="18" t="n"/>
     </row>
-    <row r="24" ht="30" customHeight="1">
+    <row r="24" ht="36" customHeight="1">
       <c r="A24" s="10" t="n"/>
       <c r="B24" s="10" t="n"/>
       <c r="C24" s="10" t="n"/>
@@ -1137,14 +1157,15 @@
       <c r="H24" s="8" t="n"/>
       <c r="I24" s="17" t="inlineStr">
         <is>
-          <t>[US-38] [Web, CMS] Trang LDP CSCA | PIC: ThuyTT104 | Mới</t>
+          <t>[Web, CMS] Trang LDP CSCA (P3)
+PIC: ThuyTT104 | Mới (15%)</t>
         </is>
       </c>
       <c r="J24" s="18" t="n"/>
       <c r="K24" s="18" t="n"/>
       <c r="L24" s="18" t="n"/>
     </row>
-    <row r="25" ht="30" customHeight="1">
+    <row r="25" ht="36" customHeight="1">
       <c r="A25" s="10" t="n"/>
       <c r="B25" s="10" t="n"/>
       <c r="C25" s="10" t="n"/>
@@ -1155,14 +1176,15 @@
       <c r="H25" s="8" t="n"/>
       <c r="I25" s="17" t="inlineStr">
         <is>
-          <t>[US-39] [Web, CMS] Trang LDP Fcitizen | PIC: ThuyTT104 | Mới</t>
+          <t>[Web, CMS] Trang LDP Fcitizen (P3)
+PIC: ThuyTT104 | Mới (15%)</t>
         </is>
       </c>
       <c r="J25" s="18" t="n"/>
       <c r="K25" s="18" t="n"/>
       <c r="L25" s="18" t="n"/>
     </row>
-    <row r="26" ht="30" customHeight="1">
+    <row r="26" ht="36" customHeight="1">
       <c r="A26" s="10" t="n"/>
       <c r="B26" s="10" t="n"/>
       <c r="C26" s="10" t="n"/>
@@ -1173,14 +1195,15 @@
       <c r="H26" s="8" t="n"/>
       <c r="I26" s="17" t="inlineStr">
         <is>
-          <t>[US-40] [Web, CMS] Trang LDP Ngoại Hạng Anh (NHA) | PIC: SonLN11 | Mới</t>
+          <t>[Web, CMS] Trang LDP Ngoại Hạng Anh (NHA) (P1)
+PIC: SonLN11 | Mới (15%)</t>
         </is>
       </c>
       <c r="J26" s="18" t="n"/>
       <c r="K26" s="18" t="n"/>
       <c r="L26" s="9" t="n"/>
     </row>
-    <row r="27" ht="30" customHeight="1">
+    <row r="27" ht="36" customHeight="1">
       <c r="A27" s="10" t="n"/>
       <c r="B27" s="10" t="n"/>
       <c r="C27" s="10" t="n"/>
@@ -1191,14 +1214,15 @@
       <c r="H27" s="8" t="n"/>
       <c r="I27" s="17" t="inlineStr">
         <is>
-          <t>[US-41] [Web, CMS] Trang LDP NHA - Lịch thi đấu | PIC: SonLN11 | Mới</t>
+          <t>[Web, CMS] Trang LDP NHA - Lịch thi đấu (P1)
+PIC: SonLN11 | Mới (15%)</t>
         </is>
       </c>
       <c r="J27" s="18" t="n"/>
       <c r="K27" s="18" t="n"/>
       <c r="L27" s="18" t="n"/>
     </row>
-    <row r="28" ht="30" customHeight="1">
+    <row r="28" ht="36" customHeight="1">
       <c r="A28" s="10" t="n"/>
       <c r="B28" s="10" t="n"/>
       <c r="C28" s="10" t="n"/>
@@ -1209,14 +1233,15 @@
       <c r="H28" s="8" t="n"/>
       <c r="I28" s="17" t="inlineStr">
         <is>
-          <t>[US-42] [Web, CMS] Trang LDP NHA - Bảng xếp hạng | PIC: SonLN11 | Mới</t>
+          <t>[Web, CMS] Trang LDP NHA - Bảng xếp hạng (P1)
+PIC: SonLN11 | Mới (15%)</t>
         </is>
       </c>
       <c r="J28" s="18" t="n"/>
       <c r="K28" s="18" t="n"/>
       <c r="L28" s="18" t="n"/>
     </row>
-    <row r="29" ht="30" customHeight="1">
+    <row r="29" ht="36" customHeight="1">
       <c r="A29" s="10" t="n"/>
       <c r="B29" s="10" t="n"/>
       <c r="C29" s="10" t="n"/>
@@ -1227,7 +1252,8 @@
       <c r="H29" s="8" t="n"/>
       <c r="I29" s="17" t="inlineStr">
         <is>
-          <t>[US-43] [Web, CMS] Trang LDP NHA - SA | PIC: SonLN11 | Mới</t>
+          <t>[Web, CMS] Trang LDP NHA - SA (P1)
+PIC: SonLN11 | Mới (15%)</t>
         </is>
       </c>
       <c r="J29" s="18" t="n"/>
@@ -1281,11 +1307,11 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
@@ -1299,32 +1325,32 @@
       </c>
       <c r="B1" s="19" t="inlineStr">
         <is>
-          <t>Mã US</t>
+          <t>Epic</t>
         </is>
       </c>
       <c r="C1" s="19" t="inlineStr">
         <is>
-          <t>Epic</t>
+          <t>Tên User Story</t>
         </is>
       </c>
       <c r="D1" s="19" t="inlineStr">
         <is>
-          <t>Tên User Story</t>
+          <t>PIC</t>
         </is>
       </c>
       <c r="E1" s="19" t="inlineStr">
         <is>
-          <t>PIC</t>
+          <t>Ưu tiên</t>
         </is>
       </c>
       <c r="F1" s="19" t="inlineStr">
         <is>
-          <t>Ưu tiên</t>
+          <t>Trạng thái</t>
         </is>
       </c>
       <c r="G1" s="19" t="inlineStr">
         <is>
-          <t>Trạng thái</t>
+          <t>Tiến độ %</t>
         </is>
       </c>
       <c r="H1" s="19" t="inlineStr">
@@ -1342,34 +1368,34 @@
       <c r="A2" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="20" t="inlineStr">
-        <is>
-          <t>US-12</t>
+      <c r="B2" s="21" t="inlineStr">
+        <is>
+          <t>[CMS]</t>
         </is>
       </c>
       <c r="C2" s="21" t="inlineStr">
         <is>
-          <t>[CMS]</t>
+          <t>Quản lý trang</t>
         </is>
       </c>
       <c r="D2" s="21" t="inlineStr">
         <is>
-          <t>Quản lý trang</t>
-        </is>
-      </c>
-      <c r="E2" s="21" t="inlineStr">
-        <is>
           <t>SonLN11</t>
         </is>
       </c>
+      <c r="E2" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
       <c r="F2" s="20" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>UAT</t>
         </is>
       </c>
       <c r="G2" s="20" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="H2" s="20" t="inlineStr">
@@ -1387,34 +1413,34 @@
       <c r="A3" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="20" t="inlineStr">
-        <is>
-          <t>US-13</t>
+      <c r="B3" s="21" t="inlineStr">
+        <is>
+          <t>[CMS]</t>
         </is>
       </c>
       <c r="C3" s="21" t="inlineStr">
         <is>
-          <t>[CMS]</t>
+          <t>Quản lý section</t>
         </is>
       </c>
       <c r="D3" s="21" t="inlineStr">
         <is>
-          <t>Quản lý section</t>
-        </is>
-      </c>
-      <c r="E3" s="21" t="inlineStr">
-        <is>
           <t>SonLN11</t>
         </is>
       </c>
+      <c r="E3" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
       <c r="F3" s="20" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>UAT</t>
         </is>
       </c>
       <c r="G3" s="20" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="H3" s="20" t="inlineStr">
@@ -1432,34 +1458,34 @@
       <c r="A4" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="20" t="inlineStr">
-        <is>
-          <t>US-14</t>
+      <c r="B4" s="21" t="inlineStr">
+        <is>
+          <t>[CMS]</t>
         </is>
       </c>
       <c r="C4" s="21" t="inlineStr">
         <is>
-          <t>[CMS]</t>
+          <t>Quản lý Block</t>
         </is>
       </c>
       <c r="D4" s="21" t="inlineStr">
         <is>
-          <t>Quản lý Block</t>
-        </is>
-      </c>
-      <c r="E4" s="21" t="inlineStr">
-        <is>
           <t>SonLN11</t>
         </is>
       </c>
+      <c r="E4" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
       <c r="F4" s="20" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>UAT</t>
         </is>
       </c>
       <c r="G4" s="20" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="H4" s="20" t="inlineStr">
@@ -1477,34 +1503,34 @@
       <c r="A5" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="20" t="inlineStr">
-        <is>
-          <t>US-15</t>
+      <c r="B5" s="21" t="inlineStr">
+        <is>
+          <t>[CMS]</t>
         </is>
       </c>
       <c r="C5" s="21" t="inlineStr">
         <is>
-          <t>[CMS]</t>
+          <t>Quản lý menu</t>
         </is>
       </c>
       <c r="D5" s="21" t="inlineStr">
         <is>
-          <t>Quản lý menu</t>
-        </is>
-      </c>
-      <c r="E5" s="21" t="inlineStr">
-        <is>
           <t>SonLN11</t>
         </is>
       </c>
+      <c r="E5" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
       <c r="F5" s="20" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>UAT</t>
         </is>
       </c>
       <c r="G5" s="20" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="H5" s="20" t="inlineStr">
@@ -1522,34 +1548,34 @@
       <c r="A6" s="20" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="20" t="inlineStr">
-        <is>
-          <t>US-MENU</t>
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>[Web, CMS]</t>
         </is>
       </c>
       <c r="C6" s="21" t="inlineStr">
         <is>
-          <t>[Web, CMS]</t>
+          <t>MENU (Cấp API Web/HiFPT &amp; Đồng bộ SPDV)</t>
         </is>
       </c>
       <c r="D6" s="21" t="inlineStr">
         <is>
-          <t>MENU (Cấp API Web/HiFPT &amp; Đồng bộ SPDV)</t>
-        </is>
-      </c>
-      <c r="E6" s="21" t="inlineStr">
-        <is>
           <t>ThuyTT104</t>
         </is>
       </c>
+      <c r="E6" s="20" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
       <c r="F6" s="20" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>DEV</t>
         </is>
       </c>
       <c r="G6" s="20" t="inlineStr">
         <is>
-          <t>DEV</t>
+          <t>60%</t>
         </is>
       </c>
       <c r="H6" s="20" t="inlineStr">
@@ -1567,34 +1593,34 @@
       <c r="A7" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="20" t="inlineStr">
-        <is>
-          <t>US-18</t>
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <t>[CMS, Web]</t>
         </is>
       </c>
       <c r="C7" s="21" t="inlineStr">
         <is>
-          <t>[CMS, Web]</t>
+          <t>Quản lý FAQ: Quy hoạch lại UI/UX &amp; luồng cấu hình (Danh sách/Danh mục FAQ)</t>
         </is>
       </c>
       <c r="D7" s="21" t="inlineStr">
         <is>
-          <t>Quản lý FAQ: Quy hoạch lại UI/UX &amp; luồng cấu hình (Danh sách/Danh mục FAQ)</t>
-        </is>
-      </c>
-      <c r="E7" s="21" t="inlineStr">
-        <is>
           <t>SonLN11</t>
         </is>
       </c>
+      <c r="E7" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
       <c r="F7" s="20" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>Phân tích</t>
         </is>
       </c>
       <c r="G7" s="20" t="inlineStr">
         <is>
-          <t>Phân tích</t>
+          <t>35%</t>
         </is>
       </c>
       <c r="H7" s="20" t="inlineStr">
@@ -1612,34 +1638,34 @@
       <c r="A8" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="20" t="inlineStr">
-        <is>
-          <t>US-20</t>
+      <c r="B8" s="21" t="inlineStr">
+        <is>
+          <t>[CMS, Web]</t>
         </is>
       </c>
       <c r="C8" s="21" t="inlineStr">
         <is>
-          <t>[CMS, Web]</t>
+          <t>Quản lý quảng cáo</t>
         </is>
       </c>
       <c r="D8" s="21" t="inlineStr">
         <is>
-          <t>Quản lý quảng cáo</t>
-        </is>
-      </c>
-      <c r="E8" s="21" t="inlineStr">
-        <is>
           <t>LongNH156</t>
         </is>
       </c>
+      <c r="E8" s="20" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
       <c r="F8" s="20" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Phân tích</t>
         </is>
       </c>
       <c r="G8" s="20" t="inlineStr">
         <is>
-          <t>Phân tích</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="H8" s="20" t="inlineStr">
@@ -1657,34 +1683,34 @@
       <c r="A9" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="20" t="inlineStr">
-        <is>
-          <t>US-21</t>
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <t>[Web]</t>
         </is>
       </c>
       <c r="C9" s="21" t="inlineStr">
         <is>
-          <t>[Web]</t>
+          <t>Report: Ghi nhận thông tin báo cáo phase 2 - bộ báo cáo chuẩn cho ĐKOL</t>
         </is>
       </c>
       <c r="D9" s="21" t="inlineStr">
         <is>
-          <t>Report: Ghi nhận thông tin báo cáo phase 2 - bộ báo cáo chuẩn cho ĐKOL</t>
-        </is>
-      </c>
-      <c r="E9" s="21" t="inlineStr">
-        <is>
           <t>ThuyTT104</t>
         </is>
       </c>
+      <c r="E9" s="20" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
       <c r="F9" s="20" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="G9" s="20" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>55%</t>
         </is>
       </c>
       <c r="H9" s="20" t="inlineStr">
@@ -1702,34 +1728,34 @@
       <c r="A10" s="20" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="20" t="inlineStr">
-        <is>
-          <t>US-LDPLOCAL</t>
+      <c r="B10" s="21" t="inlineStr">
+        <is>
+          <t>[Web, CMS]</t>
         </is>
       </c>
       <c r="C10" s="21" t="inlineStr">
         <is>
-          <t>[Web, CMS]</t>
+          <t>CMS config LDP Local: Gắn location Tỉnh/Huyện, SEO &amp; Schema</t>
         </is>
       </c>
       <c r="D10" s="21" t="inlineStr">
         <is>
-          <t>CMS config LDP Local: Gắn location Tỉnh/Huyện, SEO &amp; Schema</t>
-        </is>
-      </c>
-      <c r="E10" s="21" t="inlineStr">
-        <is>
           <t>ThuyTT104, LongNH156</t>
         </is>
       </c>
+      <c r="E10" s="20" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
       <c r="F10" s="20" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Phân tích</t>
         </is>
       </c>
       <c r="G10" s="20" t="inlineStr">
         <is>
-          <t>Phân tích</t>
+          <t>35%</t>
         </is>
       </c>
       <c r="H10" s="20" t="inlineStr">
@@ -1747,34 +1773,34 @@
       <c r="A11" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="20" t="inlineStr">
-        <is>
-          <t>US-30</t>
+      <c r="B11" s="21" t="inlineStr">
+        <is>
+          <t>[CMS, Web]</t>
         </is>
       </c>
       <c r="C11" s="21" t="inlineStr">
         <is>
-          <t>[CMS, Web]</t>
+          <t>Quản lý Breadcrumbs trên trang / Landing Page</t>
         </is>
       </c>
       <c r="D11" s="21" t="inlineStr">
         <is>
-          <t>Quản lý Breadcrumbs trên trang / Landing Page</t>
-        </is>
-      </c>
-      <c r="E11" s="21" t="inlineStr">
-        <is>
           <t>LongNH156, SonLN11</t>
         </is>
       </c>
+      <c r="E11" s="20" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
       <c r="F11" s="20" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Phân tích</t>
         </is>
       </c>
       <c r="G11" s="20" t="inlineStr">
         <is>
-          <t>Phân tích</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="H11" s="20" t="inlineStr">
@@ -1792,34 +1818,34 @@
       <c r="A12" s="20" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="20" t="inlineStr">
-        <is>
-          <t>US-29</t>
+      <c r="B12" s="21" t="inlineStr">
+        <is>
+          <t>[CMS, Web]</t>
         </is>
       </c>
       <c r="C12" s="21" t="inlineStr">
         <is>
-          <t>[CMS, Web]</t>
+          <t>Quản lý URL</t>
         </is>
       </c>
       <c r="D12" s="21" t="inlineStr">
         <is>
-          <t>Quản lý URL</t>
-        </is>
-      </c>
-      <c r="E12" s="21" t="inlineStr">
-        <is>
           <t>LongNH156, ThuyTT104</t>
         </is>
       </c>
+      <c r="E12" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
       <c r="F12" s="20" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>Phân tích</t>
         </is>
       </c>
       <c r="G12" s="20" t="inlineStr">
         <is>
-          <t>Phân tích</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="H12" s="20" t="inlineStr">
@@ -1837,34 +1863,34 @@
       <c r="A13" s="20" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="20" t="inlineStr">
-        <is>
-          <t>US-31</t>
+      <c r="B13" s="21" t="inlineStr">
+        <is>
+          <t>[Web]</t>
         </is>
       </c>
       <c r="C13" s="21" t="inlineStr">
         <is>
-          <t>[Web]</t>
+          <t>Luồng bán kèm PK (charm) Camera Play 4 trên website fpt.vn</t>
         </is>
       </c>
       <c r="D13" s="21" t="inlineStr">
         <is>
-          <t>Luồng bán kèm PK (charm) Camera Play 4 trên website fpt.vn</t>
-        </is>
-      </c>
-      <c r="E13" s="21" t="inlineStr">
-        <is>
           <t>ThuyTT104</t>
         </is>
       </c>
+      <c r="E13" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
       <c r="F13" s="20" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="G13" s="20" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>55%</t>
         </is>
       </c>
       <c r="H13" s="20" t="inlineStr">
@@ -1882,34 +1908,34 @@
       <c r="A14" s="20" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="20" t="inlineStr">
-        <is>
-          <t>US-32</t>
+      <c r="B14" s="21" t="inlineStr">
+        <is>
+          <t>[Web]</t>
         </is>
       </c>
       <c r="C14" s="21" t="inlineStr">
         <is>
-          <t>[Web]</t>
+          <t>Luồng quà tặng (Mũ bảo hiểm) trên website</t>
         </is>
       </c>
       <c r="D14" s="21" t="inlineStr">
         <is>
-          <t>Luồng quà tặng (Mũ bảo hiểm) trên website</t>
-        </is>
-      </c>
-      <c r="E14" s="21" t="inlineStr">
-        <is>
           <t>ThuyTT104</t>
         </is>
       </c>
+      <c r="E14" s="20" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
       <c r="F14" s="20" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="G14" s="20" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="H14" s="20" t="inlineStr">
@@ -1927,34 +1953,34 @@
       <c r="A15" s="20" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="20" t="inlineStr">
-        <is>
-          <t>US-33</t>
+      <c r="B15" s="21" t="inlineStr">
+        <is>
+          <t>[CMS, Web]</t>
         </is>
       </c>
       <c r="C15" s="21" t="inlineStr">
         <is>
-          <t>[CMS, Web]</t>
+          <t>Xây dựng thư viện section mở rộng cho tạo LDP kéo thả</t>
         </is>
       </c>
       <c r="D15" s="21" t="inlineStr">
         <is>
-          <t>Xây dựng thư viện section mở rộng cho tạo LDP kéo thả</t>
-        </is>
-      </c>
-      <c r="E15" s="21" t="inlineStr">
-        <is>
           <t>ThuyTT104, LongNH156</t>
         </is>
       </c>
+      <c r="E15" s="20" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
       <c r="F15" s="20" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="G15" s="20" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="H15" s="20" t="inlineStr">
@@ -1972,34 +1998,34 @@
       <c r="A16" s="20" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="20" t="inlineStr">
-        <is>
-          <t>US-28</t>
+      <c r="B16" s="21" t="inlineStr">
+        <is>
+          <t>[Web]</t>
         </is>
       </c>
       <c r="C16" s="21" t="inlineStr">
         <is>
-          <t>[Web]</t>
+          <t>[FMI Phase 4 | NBA] Phối hợp tích hợp Trigger Popup &amp; Web Push trên fpt.vn</t>
         </is>
       </c>
       <c r="D16" s="21" t="inlineStr">
         <is>
-          <t>[FMI Phase 4 | NBA] Phối hợp tích hợp Trigger Popup &amp; Web Push trên fpt.vn</t>
-        </is>
-      </c>
-      <c r="E16" s="21" t="inlineStr">
-        <is>
           <t>ThuyTT104</t>
         </is>
       </c>
+      <c r="E16" s="20" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
       <c r="F16" s="20" t="inlineStr">
         <is>
-          <t>P4</t>
+          <t>Phân tích</t>
         </is>
       </c>
       <c r="G16" s="20" t="inlineStr">
         <is>
-          <t>Phân tích</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="H16" s="20" t="inlineStr">
@@ -2017,34 +2043,34 @@
       <c r="A17" s="20" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="20" t="inlineStr">
-        <is>
-          <t>US-47</t>
+      <c r="B17" s="21" t="inlineStr">
+        <is>
+          <t>[Web]</t>
         </is>
       </c>
       <c r="C17" s="21" t="inlineStr">
         <is>
-          <t>[Web]</t>
+          <t>Luồng giỏ hàng trên kênh (Unified Cart)</t>
         </is>
       </c>
       <c r="D17" s="21" t="inlineStr">
         <is>
-          <t>Luồng giỏ hàng trên kênh (Unified Cart)</t>
-        </is>
-      </c>
-      <c r="E17" s="21" t="inlineStr">
-        <is>
           <t>ThuyTT104</t>
         </is>
       </c>
+      <c r="E17" s="20" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
       <c r="F17" s="20" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Phân tích</t>
         </is>
       </c>
       <c r="G17" s="20" t="inlineStr">
         <is>
-          <t>Phân tích</t>
+          <t>35%</t>
         </is>
       </c>
       <c r="H17" s="20" t="inlineStr">
@@ -2062,34 +2088,34 @@
       <c r="A18" s="20" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="20" t="inlineStr">
-        <is>
-          <t>US-36</t>
+      <c r="B18" s="21" t="inlineStr">
+        <is>
+          <t>[CMS, Web]</t>
         </is>
       </c>
       <c r="C18" s="21" t="inlineStr">
         <is>
-          <t>[CMS, Web]</t>
+          <t>Quản lý tin tức</t>
         </is>
       </c>
       <c r="D18" s="21" t="inlineStr">
         <is>
-          <t>Quản lý tin tức</t>
-        </is>
-      </c>
-      <c r="E18" s="21" t="inlineStr">
-        <is>
           <t>SonLN11</t>
         </is>
       </c>
+      <c r="E18" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
       <c r="F18" s="20" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>Phân tích</t>
         </is>
       </c>
       <c r="G18" s="20" t="inlineStr">
         <is>
-          <t>Phân tích</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="H18" s="20" t="inlineStr">
@@ -2107,34 +2133,34 @@
       <c r="A19" s="20" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="20" t="inlineStr">
-        <is>
-          <t>US-37</t>
+      <c r="B19" s="21" t="inlineStr">
+        <is>
+          <t>[CMS]</t>
         </is>
       </c>
       <c r="C19" s="21" t="inlineStr">
         <is>
-          <t>[CMS]</t>
+          <t>Quản lý Profile Tác giả</t>
         </is>
       </c>
       <c r="D19" s="21" t="inlineStr">
         <is>
-          <t>Quản lý Profile Tác giả</t>
-        </is>
-      </c>
-      <c r="E19" s="21" t="inlineStr">
-        <is>
           <t>SonLN11</t>
         </is>
       </c>
+      <c r="E19" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
       <c r="F19" s="20" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>Phân tích</t>
         </is>
       </c>
       <c r="G19" s="20" t="inlineStr">
         <is>
-          <t>Phân tích</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="H19" s="20" t="inlineStr">
@@ -2152,34 +2178,34 @@
       <c r="A20" s="20" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="20" t="inlineStr">
-        <is>
-          <t>US-26</t>
+      <c r="B20" s="21" t="inlineStr">
+        <is>
+          <t>[Web, CMS]</t>
         </is>
       </c>
       <c r="C20" s="21" t="inlineStr">
         <is>
-          <t>[Web, CMS]</t>
+          <t>Các link chạy ads team Performance chạy ads - quy hoạch về CMS mới</t>
         </is>
       </c>
       <c r="D20" s="21" t="inlineStr">
         <is>
-          <t>Các link chạy ads team Performance chạy ads - quy hoạch về CMS mới</t>
-        </is>
-      </c>
-      <c r="E20" s="21" t="inlineStr">
-        <is>
           <t>ThuyTT104</t>
         </is>
       </c>
+      <c r="E20" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
       <c r="F20" s="20" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>Mới</t>
         </is>
       </c>
       <c r="G20" s="20" t="inlineStr">
         <is>
-          <t>Mới</t>
+          <t>15%</t>
         </is>
       </c>
       <c r="H20" s="20" t="inlineStr">
@@ -2197,34 +2223,34 @@
       <c r="A21" s="20" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="20" t="inlineStr">
-        <is>
-          <t>US-27</t>
+      <c r="B21" s="21" t="inlineStr">
+        <is>
+          <t>[CMS, Web]</t>
         </is>
       </c>
       <c r="C21" s="21" t="inlineStr">
         <is>
-          <t>[CMS, Web]</t>
+          <t>Bổ sung trang Combo Internet Camera</t>
         </is>
       </c>
       <c r="D21" s="21" t="inlineStr">
         <is>
-          <t>Bổ sung trang Combo Internet Camera</t>
-        </is>
-      </c>
-      <c r="E21" s="21" t="inlineStr">
-        <is>
           <t>ThuyTT104</t>
         </is>
       </c>
+      <c r="E21" s="20" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
       <c r="F21" s="20" t="inlineStr">
         <is>
-          <t>P4</t>
+          <t>Mới</t>
         </is>
       </c>
       <c r="G21" s="20" t="inlineStr">
         <is>
-          <t>Mới</t>
+          <t>15%</t>
         </is>
       </c>
       <c r="H21" s="20" t="inlineStr">
@@ -2242,34 +2268,34 @@
       <c r="A22" s="20" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="20" t="inlineStr">
-        <is>
-          <t>US-38</t>
+      <c r="B22" s="21" t="inlineStr">
+        <is>
+          <t>[Web, CMS]</t>
         </is>
       </c>
       <c r="C22" s="21" t="inlineStr">
         <is>
-          <t>[Web, CMS]</t>
+          <t>Trang LDP CSCA</t>
         </is>
       </c>
       <c r="D22" s="21" t="inlineStr">
         <is>
-          <t>Trang LDP CSCA</t>
-        </is>
-      </c>
-      <c r="E22" s="21" t="inlineStr">
-        <is>
           <t>ThuyTT104</t>
         </is>
       </c>
+      <c r="E22" s="20" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
       <c r="F22" s="20" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>Mới</t>
         </is>
       </c>
       <c r="G22" s="20" t="inlineStr">
         <is>
-          <t>Mới</t>
+          <t>15%</t>
         </is>
       </c>
       <c r="H22" s="20" t="inlineStr">
@@ -2287,34 +2313,34 @@
       <c r="A23" s="20" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="20" t="inlineStr">
-        <is>
-          <t>US-39</t>
+      <c r="B23" s="21" t="inlineStr">
+        <is>
+          <t>[Web, CMS]</t>
         </is>
       </c>
       <c r="C23" s="21" t="inlineStr">
         <is>
-          <t>[Web, CMS]</t>
+          <t>Trang LDP Fcitizen</t>
         </is>
       </c>
       <c r="D23" s="21" t="inlineStr">
         <is>
-          <t>Trang LDP Fcitizen</t>
-        </is>
-      </c>
-      <c r="E23" s="21" t="inlineStr">
-        <is>
           <t>ThuyTT104</t>
         </is>
       </c>
+      <c r="E23" s="20" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
       <c r="F23" s="20" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>Mới</t>
         </is>
       </c>
       <c r="G23" s="20" t="inlineStr">
         <is>
-          <t>Mới</t>
+          <t>15%</t>
         </is>
       </c>
       <c r="H23" s="20" t="inlineStr">
@@ -2332,34 +2358,34 @@
       <c r="A24" s="20" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="20" t="inlineStr">
-        <is>
-          <t>US-40</t>
+      <c r="B24" s="21" t="inlineStr">
+        <is>
+          <t>[Web, CMS]</t>
         </is>
       </c>
       <c r="C24" s="21" t="inlineStr">
         <is>
-          <t>[Web, CMS]</t>
+          <t>Trang LDP Ngoại Hạng Anh (NHA)</t>
         </is>
       </c>
       <c r="D24" s="21" t="inlineStr">
         <is>
-          <t>Trang LDP Ngoại Hạng Anh (NHA)</t>
-        </is>
-      </c>
-      <c r="E24" s="21" t="inlineStr">
-        <is>
           <t>SonLN11</t>
         </is>
       </c>
+      <c r="E24" s="20" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
       <c r="F24" s="20" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Mới</t>
         </is>
       </c>
       <c r="G24" s="20" t="inlineStr">
         <is>
-          <t>Mới</t>
+          <t>15%</t>
         </is>
       </c>
       <c r="H24" s="20" t="inlineStr">
@@ -2377,34 +2403,34 @@
       <c r="A25" s="20" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="20" t="inlineStr">
-        <is>
-          <t>US-41</t>
+      <c r="B25" s="21" t="inlineStr">
+        <is>
+          <t>[Web, CMS]</t>
         </is>
       </c>
       <c r="C25" s="21" t="inlineStr">
         <is>
-          <t>[Web, CMS]</t>
+          <t>Trang LDP NHA - Lịch thi đấu</t>
         </is>
       </c>
       <c r="D25" s="21" t="inlineStr">
         <is>
-          <t>Trang LDP NHA - Lịch thi đấu</t>
-        </is>
-      </c>
-      <c r="E25" s="21" t="inlineStr">
-        <is>
           <t>SonLN11</t>
         </is>
       </c>
+      <c r="E25" s="20" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
       <c r="F25" s="20" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Mới</t>
         </is>
       </c>
       <c r="G25" s="20" t="inlineStr">
         <is>
-          <t>Mới</t>
+          <t>15%</t>
         </is>
       </c>
       <c r="H25" s="20" t="inlineStr">
@@ -2422,34 +2448,34 @@
       <c r="A26" s="20" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="20" t="inlineStr">
-        <is>
-          <t>US-42</t>
+      <c r="B26" s="21" t="inlineStr">
+        <is>
+          <t>[Web, CMS]</t>
         </is>
       </c>
       <c r="C26" s="21" t="inlineStr">
         <is>
-          <t>[Web, CMS]</t>
+          <t>Trang LDP NHA - Bảng xếp hạng</t>
         </is>
       </c>
       <c r="D26" s="21" t="inlineStr">
         <is>
-          <t>Trang LDP NHA - Bảng xếp hạng</t>
-        </is>
-      </c>
-      <c r="E26" s="21" t="inlineStr">
-        <is>
           <t>SonLN11</t>
         </is>
       </c>
+      <c r="E26" s="20" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
       <c r="F26" s="20" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Mới</t>
         </is>
       </c>
       <c r="G26" s="20" t="inlineStr">
         <is>
-          <t>Mới</t>
+          <t>15%</t>
         </is>
       </c>
       <c r="H26" s="20" t="inlineStr">
@@ -2467,34 +2493,34 @@
       <c r="A27" s="20" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="20" t="inlineStr">
-        <is>
-          <t>US-43</t>
+      <c r="B27" s="21" t="inlineStr">
+        <is>
+          <t>[Web, CMS]</t>
         </is>
       </c>
       <c r="C27" s="21" t="inlineStr">
         <is>
-          <t>[Web, CMS]</t>
+          <t>Trang LDP NHA - SA</t>
         </is>
       </c>
       <c r="D27" s="21" t="inlineStr">
         <is>
-          <t>Trang LDP NHA - SA</t>
-        </is>
-      </c>
-      <c r="E27" s="21" t="inlineStr">
-        <is>
           <t>SonLN11</t>
         </is>
       </c>
+      <c r="E27" s="20" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
       <c r="F27" s="20" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Mới</t>
         </is>
       </c>
       <c r="G27" s="20" t="inlineStr">
         <is>
-          <t>Mới</t>
+          <t>15%</t>
         </is>
       </c>
       <c r="H27" s="20" t="inlineStr">

</xml_diff>

<commit_message>
style(roadmap): bo phan tram tien do, dong bo chuan 5 trang thai va mau sac theo file backlog goc
</commit_message>
<xml_diff>
--- a/thuyttdoc/Roadmap_Website_CMS_Q4_2026.xlsx
+++ b/thuyttdoc/Roadmap_Website_CMS_Q4_2026.xlsx
@@ -770,7 +770,7 @@
       <c r="A4" s="6" t="inlineStr">
         <is>
           <t>[CMS] Quản lý trang (P2)
-PIC: SonLN11 | UAT (90%)</t>
+PIC: SonLN11 | UAT</t>
         </is>
       </c>
       <c r="B4" s="7" t="n"/>
@@ -789,7 +789,7 @@
       <c r="A5" s="6" t="inlineStr">
         <is>
           <t>[CMS] Quản lý section (P2)
-PIC: SonLN11 | UAT (90%)</t>
+PIC: SonLN11 | UAT</t>
         </is>
       </c>
       <c r="B5" s="7" t="n"/>
@@ -808,7 +808,7 @@
       <c r="A6" s="6" t="inlineStr">
         <is>
           <t>[CMS] Quản lý Block (P2)
-PIC: SonLN11 | UAT (90%)</t>
+PIC: SonLN11 | UAT</t>
         </is>
       </c>
       <c r="B6" s="7" t="n"/>
@@ -828,7 +828,7 @@
       <c r="B7" s="6" t="inlineStr">
         <is>
           <t>[CMS] Quản lý menu (P2)
-PIC: SonLN11 | UAT (90%)</t>
+PIC: SonLN11 | UAT</t>
         </is>
       </c>
       <c r="C7" s="7" t="n"/>
@@ -845,8 +845,8 @@
     <row r="8" ht="36" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>[Web, CMS] MENU (Cấp API Web/HiFPT &amp; Đồng bộ SPDV) (P1)
-PIC: ThuyTT104 | DEV (60%)</t>
+          <t>[Web, CMS] MENU (Cấp API Đa kênh &amp; Đồng bộ SPDV) (P1)
+PIC: ThuyTT104 | DEV In Progress</t>
         </is>
       </c>
       <c r="B8" s="7" t="n"/>
@@ -865,8 +865,8 @@
       <c r="A9" s="10" t="n"/>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>[CMS, Web] Quản lý FAQ: Quy hoạch lại UI/UX &amp; luồng cấu hình (Danh sách/Danh mục FAQ) (P2)
-PIC: SonLN11 | Phân tích (35%)</t>
+          <t>[CMS, Web] Quản lý FAQ: Quy hoạch lại UI/UX &amp; luồng cấu hình danh sách/danh mục FAQ (P2)
+PIC: SonLN11 | Đang phân tích/Document</t>
         </is>
       </c>
       <c r="C9" s="12" t="n"/>
@@ -885,7 +885,7 @@
       <c r="B10" s="11" t="inlineStr">
         <is>
           <t>[CMS, Web] Quản lý quảng cáo (P1)
-PIC: LongNH156 | Phân tích (30%)</t>
+PIC: LongNH156 | Đang phân tích/Document</t>
         </is>
       </c>
       <c r="C10" s="12" t="n"/>
@@ -905,7 +905,7 @@
       <c r="C11" s="11" t="inlineStr">
         <is>
           <t>[Web] Report: Ghi nhận thông tin báo cáo phase 2 - bộ báo cáo chuẩn cho ĐKOL (P1)
-PIC: ThuyTT104 | Đang làm (55%)</t>
+PIC: ThuyTT104 | DEV In Progress</t>
         </is>
       </c>
       <c r="D11" s="12" t="n"/>
@@ -922,8 +922,8 @@
       <c r="A12" s="10" t="n"/>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>[Web, CMS] CMS config LDP Local: Gắn location Tỉnh/Huyện, SEO &amp; Schema (P1)
-PIC: ThuyTT104, LongNH156 | Phân tích (35%)</t>
+          <t>[Web, CMS] CMS config LDP Local - QT tạo LDP Local, SEO &amp; Schema (P1)
+PIC: ThuyTT104, LongNH156 | Đang phân tích/Document</t>
         </is>
       </c>
       <c r="C12" s="12" t="n"/>
@@ -943,7 +943,7 @@
       <c r="C13" s="11" t="inlineStr">
         <is>
           <t>[CMS, Web] Quản lý Breadcrumbs trên trang / Landing Page (P1)
-PIC: LongNH156, SonLN11 | Phân tích (30%)</t>
+PIC: LongNH156, SonLN11 | Đang phân tích/Document</t>
         </is>
       </c>
       <c r="D13" s="12" t="n"/>
@@ -964,7 +964,7 @@
       <c r="E14" s="13" t="inlineStr">
         <is>
           <t>[CMS, Web] Quản lý URL (P2)
-PIC: LongNH156, ThuyTT104 | Phân tích (30%)</t>
+PIC: LongNH156, ThuyTT104 | Đang phân tích/Document</t>
         </is>
       </c>
       <c r="F14" s="14" t="n"/>
@@ -982,8 +982,8 @@
       <c r="D15" s="10" t="n"/>
       <c r="E15" s="13" t="inlineStr">
         <is>
-          <t>[Web] Luồng bán kèm PK (charm) Camera Play 4 trên website fpt.vn (P2)
-PIC: ThuyTT104 | Đang làm (55%)</t>
+          <t>[Web] Luồng bán kèm PK (charm) trên website fpt.vn (P2)
+PIC: ThuyTT104 | Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="F15" s="14" t="n"/>
@@ -1002,7 +1002,7 @@
       <c r="E16" s="13" t="inlineStr">
         <is>
           <t>[Web] Luồng quà tặng (Mũ bảo hiểm) trên website (P3)
-PIC: ThuyTT104 | Đang làm (50%)</t>
+PIC: ThuyTT104 | Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="F16" s="14" t="n"/>
@@ -1021,8 +1021,8 @@
       <c r="E17" s="8" t="n"/>
       <c r="F17" s="13" t="inlineStr">
         <is>
-          <t>[CMS, Web] Xây dựng thư viện section mở rộng cho tạo LDP kéo thả (P3)
-PIC: ThuyTT104, LongNH156 | Đang làm (50%)</t>
+          <t>[CMS, Web] Xây dựng thư viện section mở rộng cho tạo LDP kéo thả (P2)
+PIC: ThuyTT104, LongNH156 | Đang phân tích/Document</t>
         </is>
       </c>
       <c r="G17" s="14" t="n"/>
@@ -1041,7 +1041,7 @@
       <c r="F18" s="13" t="inlineStr">
         <is>
           <t>[Web] [FMI Phase 4 | NBA] Phối hợp tích hợp Trigger Popup &amp; Web Push trên fpt.vn (P4)
-PIC: ThuyTT104 | Phân tích (25%)</t>
+PIC: ThuyTT104 | Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="G18" s="14" t="n"/>
@@ -1059,7 +1059,7 @@
       <c r="E19" s="15" t="inlineStr">
         <is>
           <t>[Web] Luồng giỏ hàng trên kênh (Unified Cart) (P1)
-PIC: ThuyTT104 | Phân tích (35%)</t>
+PIC: ThuyTT104 | Đang phân tích/Document</t>
         </is>
       </c>
       <c r="F19" s="16" t="n"/>
@@ -1079,7 +1079,7 @@
       <c r="F20" s="15" t="inlineStr">
         <is>
           <t>[CMS, Web] Quản lý tin tức (P2)
-PIC: SonLN11 | Phân tích (30%)</t>
+PIC: SonLN11 | Đã tiếp nhận yêu cầu</t>
         </is>
       </c>
       <c r="G20" s="16" t="n"/>
@@ -1098,7 +1098,7 @@
       <c r="F21" s="15" t="inlineStr">
         <is>
           <t>[CMS] Quản lý Profile Tác giả (P2)
-PIC: SonLN11 | Phân tích (30%)</t>
+PIC: SonLN11 | Đã tiếp nhận yêu cầu</t>
         </is>
       </c>
       <c r="G21" s="16" t="n"/>
@@ -1119,8 +1119,8 @@
       <c r="H22" s="8" t="n"/>
       <c r="I22" s="17" t="inlineStr">
         <is>
-          <t>[Web, CMS] Các link chạy ads team Performance chạy ads - quy hoạch về CMS mới (P2)
-PIC: ThuyTT104 | Mới (15%)</t>
+          <t>[Web, CMS] Các link chạy ads team Performance chạy ads - quy hoạch về CMS mới (P3)
+PIC: ThuyTT104 | Đang phân tích/Document</t>
         </is>
       </c>
       <c r="J22" s="18" t="n"/>
@@ -1139,7 +1139,7 @@
       <c r="I23" s="17" t="inlineStr">
         <is>
           <t>[CMS, Web] Bổ sung trang Combo Internet Camera (P4)
-PIC: ThuyTT104 | Mới (15%)</t>
+PIC: ThuyTT104 | Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="J23" s="18" t="n"/>
@@ -1157,8 +1157,8 @@
       <c r="H24" s="8" t="n"/>
       <c r="I24" s="17" t="inlineStr">
         <is>
-          <t>[Web, CMS] Trang LDP CSCA (P3)
-PIC: ThuyTT104 | Mới (15%)</t>
+          <t>[Web, CMS] Trang LDP CSCA (P2)
+PIC: ThuyTT104 | Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="J24" s="18" t="n"/>
@@ -1176,8 +1176,8 @@
       <c r="H25" s="8" t="n"/>
       <c r="I25" s="17" t="inlineStr">
         <is>
-          <t>[Web, CMS] Trang LDP Fcitizen (P3)
-PIC: ThuyTT104 | Mới (15%)</t>
+          <t>[Web, CMS] Trang LDP Fcitizen (P2)
+PIC: ThuyTT104 | Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="J25" s="18" t="n"/>
@@ -1195,8 +1195,8 @@
       <c r="H26" s="8" t="n"/>
       <c r="I26" s="17" t="inlineStr">
         <is>
-          <t>[Web, CMS] Trang LDP Ngoại Hạng Anh (NHA) (P1)
-PIC: SonLN11 | Mới (15%)</t>
+          <t>[Web, CMS] Trang LDP Ngoại Hạng Anh (NHA) (P2)
+PIC: SonLN11 | Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="J26" s="18" t="n"/>
@@ -1214,8 +1214,8 @@
       <c r="H27" s="8" t="n"/>
       <c r="I27" s="17" t="inlineStr">
         <is>
-          <t>[Web, CMS] Trang LDP NHA - Lịch thi đấu (P1)
-PIC: SonLN11 | Mới (15%)</t>
+          <t>[Web, CMS] Trang LDP NHA - Lịch thi đấu (P2)
+PIC: SonLN11 | Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="J27" s="18" t="n"/>
@@ -1233,8 +1233,8 @@
       <c r="H28" s="8" t="n"/>
       <c r="I28" s="17" t="inlineStr">
         <is>
-          <t>[Web, CMS] Trang LDP NHA - Bảng xếp hạng (P1)
-PIC: SonLN11 | Mới (15%)</t>
+          <t>[Web, CMS] Trang LDP NHA - Bảng xếp hạng (P2)
+PIC: SonLN11 | Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="J28" s="18" t="n"/>
@@ -1252,8 +1252,8 @@
       <c r="H29" s="8" t="n"/>
       <c r="I29" s="17" t="inlineStr">
         <is>
-          <t>[Web, CMS] Trang LDP NHA - SA (P1)
-PIC: SonLN11 | Mới (15%)</t>
+          <t>[Web, CMS] Trang LDP NHA - SA (P2)
+PIC: SonLN11 | Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="J29" s="18" t="n"/>
@@ -1303,16 +1303,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="45" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
   </cols>
@@ -1345,20 +1344,15 @@
       </c>
       <c r="F1" s="19" t="inlineStr">
         <is>
-          <t>Trạng thái</t>
+          <t>Trạng thái (Status)</t>
         </is>
       </c>
       <c r="G1" s="19" t="inlineStr">
         <is>
-          <t>Tiến độ %</t>
+          <t>Tháng Bắt Đầu</t>
         </is>
       </c>
       <c r="H1" s="19" t="inlineStr">
-        <is>
-          <t>Tháng Bắt Đầu</t>
-        </is>
-      </c>
-      <c r="I1" s="19" t="inlineStr">
         <is>
           <t>Tháng Hoàn Thành</t>
         </is>
@@ -1395,15 +1389,10 @@
       </c>
       <c r="G2" s="20" t="inlineStr">
         <is>
-          <t>90%</t>
+          <t>Tháng 10</t>
         </is>
       </c>
       <c r="H2" s="20" t="inlineStr">
-        <is>
-          <t>Tháng 10</t>
-        </is>
-      </c>
-      <c r="I2" s="20" t="inlineStr">
         <is>
           <t>Tháng 10</t>
         </is>
@@ -1440,15 +1429,10 @@
       </c>
       <c r="G3" s="20" t="inlineStr">
         <is>
-          <t>90%</t>
+          <t>Tháng 10</t>
         </is>
       </c>
       <c r="H3" s="20" t="inlineStr">
-        <is>
-          <t>Tháng 10</t>
-        </is>
-      </c>
-      <c r="I3" s="20" t="inlineStr">
         <is>
           <t>Tháng 10</t>
         </is>
@@ -1485,15 +1469,10 @@
       </c>
       <c r="G4" s="20" t="inlineStr">
         <is>
-          <t>90%</t>
+          <t>Tháng 10</t>
         </is>
       </c>
       <c r="H4" s="20" t="inlineStr">
-        <is>
-          <t>Tháng 10</t>
-        </is>
-      </c>
-      <c r="I4" s="20" t="inlineStr">
         <is>
           <t>Tháng 10</t>
         </is>
@@ -1530,15 +1509,10 @@
       </c>
       <c r="G5" s="20" t="inlineStr">
         <is>
-          <t>90%</t>
+          <t>Tháng 10</t>
         </is>
       </c>
       <c r="H5" s="20" t="inlineStr">
-        <is>
-          <t>Tháng 10</t>
-        </is>
-      </c>
-      <c r="I5" s="20" t="inlineStr">
         <is>
           <t>Tháng 10</t>
         </is>
@@ -1555,7 +1529,7 @@
       </c>
       <c r="C6" s="21" t="inlineStr">
         <is>
-          <t>MENU (Cấp API Web/HiFPT &amp; Đồng bộ SPDV)</t>
+          <t>MENU (Cấp API Đa kênh &amp; Đồng bộ SPDV)</t>
         </is>
       </c>
       <c r="D6" s="21" t="inlineStr">
@@ -1570,20 +1544,15 @@
       </c>
       <c r="F6" s="20" t="inlineStr">
         <is>
-          <t>DEV</t>
+          <t>DEV In Progress</t>
         </is>
       </c>
       <c r="G6" s="20" t="inlineStr">
         <is>
-          <t>60%</t>
+          <t>Tháng 10</t>
         </is>
       </c>
       <c r="H6" s="20" t="inlineStr">
-        <is>
-          <t>Tháng 10</t>
-        </is>
-      </c>
-      <c r="I6" s="20" t="inlineStr">
         <is>
           <t>Tháng 10</t>
         </is>
@@ -1600,7 +1569,7 @@
       </c>
       <c r="C7" s="21" t="inlineStr">
         <is>
-          <t>Quản lý FAQ: Quy hoạch lại UI/UX &amp; luồng cấu hình (Danh sách/Danh mục FAQ)</t>
+          <t>Quản lý FAQ: Quy hoạch lại UI/UX &amp; luồng cấu hình danh sách/danh mục FAQ</t>
         </is>
       </c>
       <c r="D7" s="21" t="inlineStr">
@@ -1615,20 +1584,15 @@
       </c>
       <c r="F7" s="20" t="inlineStr">
         <is>
-          <t>Phân tích</t>
+          <t>Đang phân tích/Document</t>
         </is>
       </c>
       <c r="G7" s="20" t="inlineStr">
         <is>
-          <t>35%</t>
+          <t>Tháng 10</t>
         </is>
       </c>
       <c r="H7" s="20" t="inlineStr">
-        <is>
-          <t>Tháng 10</t>
-        </is>
-      </c>
-      <c r="I7" s="20" t="inlineStr">
         <is>
           <t>Tháng 11</t>
         </is>
@@ -1660,20 +1624,15 @@
       </c>
       <c r="F8" s="20" t="inlineStr">
         <is>
-          <t>Phân tích</t>
+          <t>Đang phân tích/Document</t>
         </is>
       </c>
       <c r="G8" s="20" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>Tháng 10</t>
         </is>
       </c>
       <c r="H8" s="20" t="inlineStr">
-        <is>
-          <t>Tháng 10</t>
-        </is>
-      </c>
-      <c r="I8" s="20" t="inlineStr">
         <is>
           <t>Tháng 11</t>
         </is>
@@ -1705,20 +1664,15 @@
       </c>
       <c r="F9" s="20" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>DEV In Progress</t>
         </is>
       </c>
       <c r="G9" s="20" t="inlineStr">
         <is>
-          <t>55%</t>
+          <t>Tháng 10</t>
         </is>
       </c>
       <c r="H9" s="20" t="inlineStr">
-        <is>
-          <t>Tháng 10</t>
-        </is>
-      </c>
-      <c r="I9" s="20" t="inlineStr">
         <is>
           <t>Tháng 11</t>
         </is>
@@ -1735,7 +1689,7 @@
       </c>
       <c r="C10" s="21" t="inlineStr">
         <is>
-          <t>CMS config LDP Local: Gắn location Tỉnh/Huyện, SEO &amp; Schema</t>
+          <t>CMS config LDP Local - QT tạo LDP Local, SEO &amp; Schema</t>
         </is>
       </c>
       <c r="D10" s="21" t="inlineStr">
@@ -1750,20 +1704,15 @@
       </c>
       <c r="F10" s="20" t="inlineStr">
         <is>
-          <t>Phân tích</t>
+          <t>Đang phân tích/Document</t>
         </is>
       </c>
       <c r="G10" s="20" t="inlineStr">
         <is>
-          <t>35%</t>
+          <t>Tháng 10</t>
         </is>
       </c>
       <c r="H10" s="20" t="inlineStr">
-        <is>
-          <t>Tháng 10</t>
-        </is>
-      </c>
-      <c r="I10" s="20" t="inlineStr">
         <is>
           <t>Tháng 11</t>
         </is>
@@ -1795,20 +1744,15 @@
       </c>
       <c r="F11" s="20" t="inlineStr">
         <is>
-          <t>Phân tích</t>
+          <t>Đang phân tích/Document</t>
         </is>
       </c>
       <c r="G11" s="20" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>Tháng 10</t>
         </is>
       </c>
       <c r="H11" s="20" t="inlineStr">
-        <is>
-          <t>Tháng 10</t>
-        </is>
-      </c>
-      <c r="I11" s="20" t="inlineStr">
         <is>
           <t>Tháng 11</t>
         </is>
@@ -1840,20 +1784,15 @@
       </c>
       <c r="F12" s="20" t="inlineStr">
         <is>
-          <t>Phân tích</t>
+          <t>Đang phân tích/Document</t>
         </is>
       </c>
       <c r="G12" s="20" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>Tháng 11</t>
         </is>
       </c>
       <c r="H12" s="20" t="inlineStr">
-        <is>
-          <t>Tháng 11</t>
-        </is>
-      </c>
-      <c r="I12" s="20" t="inlineStr">
         <is>
           <t>Tháng 11</t>
         </is>
@@ -1870,7 +1809,7 @@
       </c>
       <c r="C13" s="21" t="inlineStr">
         <is>
-          <t>Luồng bán kèm PK (charm) Camera Play 4 trên website fpt.vn</t>
+          <t>Luồng bán kèm PK (charm) trên website fpt.vn</t>
         </is>
       </c>
       <c r="D13" s="21" t="inlineStr">
@@ -1885,20 +1824,15 @@
       </c>
       <c r="F13" s="20" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="G13" s="20" t="inlineStr">
         <is>
-          <t>55%</t>
+          <t>Tháng 11</t>
         </is>
       </c>
       <c r="H13" s="20" t="inlineStr">
-        <is>
-          <t>Tháng 11</t>
-        </is>
-      </c>
-      <c r="I13" s="20" t="inlineStr">
         <is>
           <t>Tháng 11</t>
         </is>
@@ -1930,20 +1864,15 @@
       </c>
       <c r="F14" s="20" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="G14" s="20" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>Tháng 11</t>
         </is>
       </c>
       <c r="H14" s="20" t="inlineStr">
-        <is>
-          <t>Tháng 11</t>
-        </is>
-      </c>
-      <c r="I14" s="20" t="inlineStr">
         <is>
           <t>Tháng 11</t>
         </is>
@@ -1970,25 +1899,20 @@
       </c>
       <c r="E15" s="20" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="F15" s="20" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Đang phân tích/Document</t>
         </is>
       </c>
       <c r="G15" s="20" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>Tháng 11</t>
         </is>
       </c>
       <c r="H15" s="20" t="inlineStr">
-        <is>
-          <t>Tháng 11</t>
-        </is>
-      </c>
-      <c r="I15" s="20" t="inlineStr">
         <is>
           <t>Tháng 11</t>
         </is>
@@ -2020,20 +1944,15 @@
       </c>
       <c r="F16" s="20" t="inlineStr">
         <is>
-          <t>Phân tích</t>
+          <t>Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="G16" s="20" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>Tháng 11</t>
         </is>
       </c>
       <c r="H16" s="20" t="inlineStr">
-        <is>
-          <t>Tháng 11</t>
-        </is>
-      </c>
-      <c r="I16" s="20" t="inlineStr">
         <is>
           <t>Tháng 11</t>
         </is>
@@ -2065,20 +1984,15 @@
       </c>
       <c r="F17" s="20" t="inlineStr">
         <is>
-          <t>Phân tích</t>
+          <t>Đang phân tích/Document</t>
         </is>
       </c>
       <c r="G17" s="20" t="inlineStr">
         <is>
-          <t>35%</t>
+          <t>Tháng 11</t>
         </is>
       </c>
       <c r="H17" s="20" t="inlineStr">
-        <is>
-          <t>Tháng 11</t>
-        </is>
-      </c>
-      <c r="I17" s="20" t="inlineStr">
         <is>
           <t>Tháng 12</t>
         </is>
@@ -2110,20 +2024,15 @@
       </c>
       <c r="F18" s="20" t="inlineStr">
         <is>
-          <t>Phân tích</t>
+          <t>Đã tiếp nhận yêu cầu</t>
         </is>
       </c>
       <c r="G18" s="20" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>Tháng 11</t>
         </is>
       </c>
       <c r="H18" s="20" t="inlineStr">
-        <is>
-          <t>Tháng 11</t>
-        </is>
-      </c>
-      <c r="I18" s="20" t="inlineStr">
         <is>
           <t>Tháng 12</t>
         </is>
@@ -2155,20 +2064,15 @@
       </c>
       <c r="F19" s="20" t="inlineStr">
         <is>
-          <t>Phân tích</t>
+          <t>Đã tiếp nhận yêu cầu</t>
         </is>
       </c>
       <c r="G19" s="20" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>Tháng 11</t>
         </is>
       </c>
       <c r="H19" s="20" t="inlineStr">
-        <is>
-          <t>Tháng 11</t>
-        </is>
-      </c>
-      <c r="I19" s="20" t="inlineStr">
         <is>
           <t>Tháng 12</t>
         </is>
@@ -2195,25 +2099,20 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="F20" s="20" t="inlineStr">
         <is>
-          <t>Mới</t>
+          <t>Đang phân tích/Document</t>
         </is>
       </c>
       <c r="G20" s="20" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>Tháng 12</t>
         </is>
       </c>
       <c r="H20" s="20" t="inlineStr">
-        <is>
-          <t>Tháng 12</t>
-        </is>
-      </c>
-      <c r="I20" s="20" t="inlineStr">
         <is>
           <t>Tháng 12</t>
         </is>
@@ -2245,20 +2144,15 @@
       </c>
       <c r="F21" s="20" t="inlineStr">
         <is>
-          <t>Mới</t>
+          <t>Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="G21" s="20" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>Tháng 12</t>
         </is>
       </c>
       <c r="H21" s="20" t="inlineStr">
-        <is>
-          <t>Tháng 12</t>
-        </is>
-      </c>
-      <c r="I21" s="20" t="inlineStr">
         <is>
           <t>Tháng 12</t>
         </is>
@@ -2285,25 +2179,20 @@
       </c>
       <c r="E22" s="20" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="F22" s="20" t="inlineStr">
         <is>
-          <t>Mới</t>
+          <t>Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="G22" s="20" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>Tháng 12</t>
         </is>
       </c>
       <c r="H22" s="20" t="inlineStr">
-        <is>
-          <t>Tháng 12</t>
-        </is>
-      </c>
-      <c r="I22" s="20" t="inlineStr">
         <is>
           <t>Tháng 12</t>
         </is>
@@ -2330,25 +2219,20 @@
       </c>
       <c r="E23" s="20" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="F23" s="20" t="inlineStr">
         <is>
-          <t>Mới</t>
+          <t>Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="G23" s="20" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>Tháng 12</t>
         </is>
       </c>
       <c r="H23" s="20" t="inlineStr">
-        <is>
-          <t>Tháng 12</t>
-        </is>
-      </c>
-      <c r="I23" s="20" t="inlineStr">
         <is>
           <t>Tháng 12</t>
         </is>
@@ -2375,25 +2259,20 @@
       </c>
       <c r="E24" s="20" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="F24" s="20" t="inlineStr">
         <is>
-          <t>Mới</t>
+          <t>Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="G24" s="20" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>Tháng 12</t>
         </is>
       </c>
       <c r="H24" s="20" t="inlineStr">
-        <is>
-          <t>Tháng 12</t>
-        </is>
-      </c>
-      <c r="I24" s="20" t="inlineStr">
         <is>
           <t>Tháng 12</t>
         </is>
@@ -2420,25 +2299,20 @@
       </c>
       <c r="E25" s="20" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="F25" s="20" t="inlineStr">
         <is>
-          <t>Mới</t>
+          <t>Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="G25" s="20" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>Tháng 12</t>
         </is>
       </c>
       <c r="H25" s="20" t="inlineStr">
-        <is>
-          <t>Tháng 12</t>
-        </is>
-      </c>
-      <c r="I25" s="20" t="inlineStr">
         <is>
           <t>Tháng 12</t>
         </is>
@@ -2465,25 +2339,20 @@
       </c>
       <c r="E26" s="20" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="F26" s="20" t="inlineStr">
         <is>
-          <t>Mới</t>
+          <t>Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="G26" s="20" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>Tháng 12</t>
         </is>
       </c>
       <c r="H26" s="20" t="inlineStr">
-        <is>
-          <t>Tháng 12</t>
-        </is>
-      </c>
-      <c r="I26" s="20" t="inlineStr">
         <is>
           <t>Tháng 12</t>
         </is>
@@ -2510,25 +2379,20 @@
       </c>
       <c r="E27" s="20" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="F27" s="20" t="inlineStr">
         <is>
-          <t>Mới</t>
+          <t>Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="G27" s="20" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>Tháng 12</t>
         </is>
       </c>
       <c r="H27" s="20" t="inlineStr">
-        <is>
-          <t>Tháng 12</t>
-        </is>
-      </c>
-      <c r="I27" s="20" t="inlineStr">
         <is>
           <t>Tháng 12</t>
         </is>

</xml_diff>

<commit_message>
feat(roadmap): sap xep uu tien P1-P4 trong tung moc thoi gian va cap nhat thu tu bang mau trang thai chuan tu he thong
</commit_message>
<xml_diff>
--- a/thuyttdoc/Roadmap_Website_CMS_Q4_2026.xlsx
+++ b/thuyttdoc/Roadmap_Website_CMS_Q4_2026.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="15">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -46,17 +46,73 @@
     </font>
     <font>
       <name val="Times New Roman"/>
-      <color rgb="00166534"/>
+      <color rgb="0078350F"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Times New Roman"/>
-      <color rgb="001E40AF"/>
+      <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Times New Roman"/>
-      <color rgb="006B21A8"/>
+      <color rgb="0080350B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <color rgb="00214349"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <color rgb="004F378B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="00991B1B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="0078350F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="0092400E"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="0080350B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="00214349"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="003730A3"/>
       <sz val="10"/>
     </font>
     <font>
@@ -66,45 +122,12 @@
     </font>
     <font>
       <name val="Times New Roman"/>
-      <color rgb="0092400E"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Times New Roman"/>
       <b val="1"/>
-      <color rgb="00166534"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Times New Roman"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Times New Roman"/>
-      <b val="1"/>
-      <color rgb="001E40AF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Times New Roman"/>
-      <b val="1"/>
-      <color rgb="006B21A8"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Times New Roman"/>
-      <b val="1"/>
-      <color rgb="00475569"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Times New Roman"/>
-      <b val="1"/>
-      <color rgb="0092400E"/>
+      <color rgb="004F378B"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -137,26 +160,44 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DCFCE7"/>
-        <bgColor rgb="00DCFCE7"/>
+        <fgColor rgb="00FEF08A"/>
+        <bgColor rgb="00FEF08A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DBEAFE"/>
-        <bgColor rgb="00DBEAFE"/>
+        <fgColor rgb="00581C87"/>
+        <bgColor rgb="00581C87"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F3E8FF"/>
-        <bgColor rgb="00F3E8FF"/>
+        <fgColor rgb="00FCD5B5"/>
+        <bgColor rgb="00FCD5B5"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F1F5F9"/>
-        <bgColor rgb="00F1F5F9"/>
+        <fgColor rgb="00D2E4E6"/>
+        <bgColor rgb="00D2E4E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E6DCF5"/>
+        <bgColor rgb="00E6DCF5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00005696"/>
+        <bgColor rgb="00005696"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEE2E2"/>
+        <bgColor rgb="00FEE2E2"/>
       </patternFill>
     </fill>
     <fill>
@@ -167,8 +208,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00005696"/>
-        <bgColor rgb="00005696"/>
+        <fgColor rgb="00E0E7FF"/>
+        <bgColor rgb="00E0E7FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1F5F9"/>
+        <bgColor rgb="00F1F5F9"/>
       </patternFill>
     </fill>
   </fills>
@@ -231,7 +278,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -264,25 +311,37 @@
     <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -668,7 +727,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Lộ trình thực thi 26 User Stories theo các cột Tháng | Bỏ cột tuần | Thể hiện đầy đủ tiến trình và trạng thái</t>
+          <t>Lộ trình thực thi 26 User Stories | Sắp xếp P1 -&gt; P2 -&gt; P3 -&gt; P4 trong cùng 1 mốc thời gian | Chuẩn bảng màu trạng thái</t>
         </is>
       </c>
     </row>
@@ -692,98 +751,98 @@
     <row r="5" ht="36" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
+          <t>[Web, CMS] MENU (Cấp API Đa kênh &amp; Đồng bộ SPDV)
+[PIC: ThuyTT104 | P1 | Status: DEV In Progress]</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n"/>
+      <c r="C5" s="7" t="n"/>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
           <t>[CMS] Quản lý trang
 [PIC: SonLN11 | P2 | Status: UAT]</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n"/>
-      <c r="C5" s="7" t="n"/>
-    </row>
-    <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="B6" s="7" t="n"/>
+      <c r="C6" s="7" t="n"/>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>[CMS] Quản lý section
 [PIC: SonLN11 | P2 | Status: UAT]</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n"/>
-      <c r="C6" s="7" t="n"/>
-    </row>
-    <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="B7" s="7" t="n"/>
+      <c r="C7" s="7" t="n"/>
+    </row>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>[CMS] Quản lý Block
 [PIC: SonLN11 | P2 | Status: UAT]</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n"/>
-      <c r="C7" s="7" t="n"/>
-    </row>
-    <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="B8" s="7" t="n"/>
+      <c r="C8" s="7" t="n"/>
+    </row>
+    <row r="9" ht="36" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>[CMS] Quản lý menu
 [PIC: SonLN11 | P2 | Status: UAT]</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n"/>
-      <c r="C8" s="7" t="n"/>
-    </row>
-    <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>[Web, CMS] MENU (Cấp API Đa kênh &amp; Đồng bộ SPDV)
-[PIC: ThuyTT104 | P1 | Status: DEV In Progress]</t>
-        </is>
-      </c>
       <c r="B9" s="7" t="n"/>
       <c r="C9" s="7" t="n"/>
     </row>
     <row r="10" ht="36" customHeight="1">
       <c r="A10" s="9" t="inlineStr">
         <is>
+          <t>➔ [Tháng 10 ➔ Tháng 11] [CMS, Web] Quản lý quảng cáo
+[PIC: LongNH156 | P1 | Status: Đang phân tích/Document]</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="n"/>
+      <c r="C10" s="7" t="n"/>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>➔ [Tháng 10 ➔ Tháng 11] [Web] Report: Ghi nhận thông tin báo cáo phase 2 – bộ báo cáo chuẩn cho ĐKOL
+[PIC: ThuyTT104 | P1 | Status: DEV In Progress]</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="n"/>
+      <c r="C11" s="7" t="n"/>
+    </row>
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>➔ [Tháng 10 ➔ Tháng 11] [Web, CMS] CMS config LDP Local – QT tạo LDP Local, SEO &amp; Schema
+[PIC: ThuyTT104, LongNH156 | P1 | Status: Đang phân tích/Document]</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="n"/>
+      <c r="C12" s="7" t="n"/>
+    </row>
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>➔ [Tháng 10 ➔ Tháng 11] [CMS, Web] Quản lý Breadcrumbs trên trang / Landing Page
+[PIC: LongNH156, SonLN11 | P1 | Status: Đang phân tích/Document]</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="n"/>
+      <c r="C13" s="7" t="n"/>
+    </row>
+    <row r="14" ht="36" customHeight="1">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
           <t>➔ [Tháng 10 ➔ Tháng 11] [CMS, Web] Quản lý FAQ: Quy hoạch lại UI/UX &amp; luồng cấu hình danh sách/danh mục FAQ
 [PIC: SonLN11 | P2 | Status: Đang phân tích/Document]</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="n"/>
-      <c r="C10" s="7" t="n"/>
-    </row>
-    <row r="11" ht="36" customHeight="1">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>➔ [Tháng 10 ➔ Tháng 11] [CMS, Web] Quản lý quảng cáo
-[PIC: LongNH156 | P1 | Status: Đang phân tích/Document]</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="n"/>
-      <c r="C11" s="7" t="n"/>
-    </row>
-    <row r="12" ht="36" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>➔ [Tháng 10 ➔ Tháng 11] [Web] Report: Ghi nhận thông tin báo cáo phase 2 – bộ báo cáo chuẩn cho ĐKOL
-[PIC: ThuyTT104 | P1 | Status: DEV In Progress]</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="n"/>
-      <c r="C12" s="7" t="n"/>
-    </row>
-    <row r="13" ht="36" customHeight="1">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>➔ [Tháng 10 ➔ Tháng 11] [Web, CMS] CMS config LDP Local – QT tạo LDP Local, SEO &amp; Schema
-[PIC: ThuyTT104, LongNH156 | P1 | Status: Đang phân tích/Document]</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="n"/>
-      <c r="C13" s="7" t="n"/>
-    </row>
-    <row r="14" ht="36" customHeight="1">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>➔ [Tháng 10 ➔ Tháng 11] [CMS, Web] Quản lý Breadcrumbs trên trang / Landing Page
-[PIC: LongNH156, SonLN11 | P1 | Status: Đang phân tích/Document]</t>
         </is>
       </c>
       <c r="B14" s="10" t="n"/>
@@ -801,10 +860,10 @@
     </row>
     <row r="16" ht="36" customHeight="1">
       <c r="A16" s="7" t="n"/>
-      <c r="B16" s="11" t="inlineStr">
-        <is>
-          <t>[Web] Luồng bán kèm PK (charm) trên website fpt.vn
-[PIC: ThuyTT104 | P2 | Status: Chưa tiếp nhận]</t>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>[CMS, Web] Xây dựng thư viện section mở rộng cho tạo LDP kéo thả
+[PIC: ThuyTT104, LongNH156 | P2 | Status: Đang phân tích/Document]</t>
         </is>
       </c>
       <c r="C16" s="7" t="n"/>
@@ -813,18 +872,18 @@
       <c r="A17" s="7" t="n"/>
       <c r="B17" s="11" t="inlineStr">
         <is>
+          <t>[Web] Luồng bán kèm PK (charm) trên website fpt.vn
+[PIC: ThuyTT104 | P2 | Status: Chưa tiếp nhận]</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="n"/>
+    </row>
+    <row r="18" ht="36" customHeight="1">
+      <c r="A18" s="7" t="n"/>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
           <t>[Web] Luồng quà tặng (Mũ bảo hiểm) trên website
 [PIC: ThuyTT104 | P3 | Status: Chưa tiếp nhận]</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="n"/>
-    </row>
-    <row r="18" ht="36" customHeight="1">
-      <c r="A18" s="7" t="n"/>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>[CMS, Web] Xây dựng thư viện section mở rộng cho tạo LDP kéo thả
-[PIC: ThuyTT104, LongNH156 | P2 | Status: Đang phân tích/Document]</t>
         </is>
       </c>
       <c r="C18" s="7" t="n"/>
@@ -872,10 +931,10 @@
     <row r="23" ht="36" customHeight="1">
       <c r="A23" s="7" t="n"/>
       <c r="B23" s="7" t="n"/>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>[Web, CMS] Các link chạy ads team Performance chạy ads - quy hoạch về CMS mới
-[PIC: ThuyTT104 | P3 | Status: Đang phân tích/Document]</t>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>[Web, CMS] Trang LDP CSCA
+[PIC: ThuyTT104 | P2 | Status: Chưa tiếp nhận]</t>
         </is>
       </c>
     </row>
@@ -884,8 +943,8 @@
       <c r="B24" s="7" t="n"/>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>[CMS, Web] Bổ sung trang Combo Internet Camera
-[PIC: ThuyTT104 | P4 | Status: Chưa tiếp nhận]</t>
+          <t>[Web, CMS] Trang LDP Fcitizen
+[PIC: ThuyTT104 | P2 | Status: Chưa tiếp nhận]</t>
         </is>
       </c>
     </row>
@@ -894,8 +953,8 @@
       <c r="B25" s="7" t="n"/>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>[Web, CMS] Trang LDP CSCA
-[PIC: ThuyTT104 | P2 | Status: Chưa tiếp nhận]</t>
+          <t>[Web, CMS] Trang LDP Ngoại Hạng Anh (NHA)
+[PIC: SonLN11 | P2 | Status: Chưa tiếp nhận]</t>
         </is>
       </c>
     </row>
@@ -904,8 +963,8 @@
       <c r="B26" s="7" t="n"/>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>[Web, CMS] Trang LDP Fcitizen
-[PIC: ThuyTT104 | P2 | Status: Chưa tiếp nhận]</t>
+          <t>[Web, CMS] Trang LDP NHA - Lịch thi đấu
+[PIC: SonLN11 | P2 | Status: Chưa tiếp nhận]</t>
         </is>
       </c>
     </row>
@@ -914,7 +973,7 @@
       <c r="B27" s="7" t="n"/>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>[Web, CMS] Trang LDP Ngoại Hạng Anh (NHA)
+          <t>[Web, CMS] Trang LDP NHA - Bảng xếp hạng
 [PIC: SonLN11 | P2 | Status: Chưa tiếp nhận]</t>
         </is>
       </c>
@@ -924,7 +983,7 @@
       <c r="B28" s="7" t="n"/>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>[Web, CMS] Trang LDP NHA - Lịch thi đấu
+          <t>[Web, CMS] Trang LDP NHA - SA
 [PIC: SonLN11 | P2 | Status: Chưa tiếp nhận]</t>
         </is>
       </c>
@@ -932,10 +991,10 @@
     <row r="29" ht="36" customHeight="1">
       <c r="A29" s="7" t="n"/>
       <c r="B29" s="7" t="n"/>
-      <c r="C29" s="11" t="inlineStr">
-        <is>
-          <t>[Web, CMS] Trang LDP NHA - Bảng xếp hạng
-[PIC: SonLN11 | P2 | Status: Chưa tiếp nhận]</t>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>[Web, CMS] Các link chạy ads team Performance chạy ads - quy hoạch về CMS mới
+[PIC: ThuyTT104 | P3 | Status: Đang phân tích/Document]</t>
         </is>
       </c>
     </row>
@@ -944,8 +1003,8 @@
       <c r="B30" s="7" t="n"/>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>[Web, CMS] Trang LDP NHA - SA
-[PIC: SonLN11 | P2 | Status: Chưa tiếp nhận]</t>
+          <t>[CMS, Web] Bổ sung trang Combo Internet Camera
+[PIC: ThuyTT104 | P4 | Status: Chưa tiếp nhận]</t>
         </is>
       </c>
     </row>
@@ -986,7 +1045,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DANH SÁCH CHI TIẾT 26 USER STORIES QUÝ 4/2026 (CHUẨN TRẠNG THÁI TỪ BACKLOG)</t>
+          <t>DANH SÁCH CHI TIẾT 26 USER STORIES QUÝ 4/2026 (SẮP XẾP ƯU TIÊN P1 -&gt; P4 THEO MỐC THỜI GIAN)</t>
         </is>
       </c>
     </row>
@@ -1038,27 +1097,27 @@
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>[CMS]</t>
+          <t>[Web, CMS]</t>
         </is>
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
-          <t>Quản lý trang</t>
-        </is>
-      </c>
-      <c r="D4" s="14" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>MENU (Cấp API Đa kênh &amp; Đồng bộ SPDV)</t>
+        </is>
+      </c>
+      <c r="D4" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="E4" s="15" t="inlineStr">
         <is>
-          <t>SonLN11</t>
-        </is>
-      </c>
-      <c r="F4" s="16" t="inlineStr">
-        <is>
-          <t>UAT</t>
+          <t>ThuyTT104</t>
+        </is>
+      </c>
+      <c r="F4" s="17" t="inlineStr">
+        <is>
+          <t>DEV In Progress</t>
         </is>
       </c>
       <c r="G4" s="14" t="inlineStr">
@@ -1083,10 +1142,10 @@
       </c>
       <c r="C5" s="15" t="inlineStr">
         <is>
-          <t>Quản lý section</t>
-        </is>
-      </c>
-      <c r="D5" s="14" t="inlineStr">
+          <t>Quản lý trang</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -1096,7 +1155,7 @@
           <t>SonLN11</t>
         </is>
       </c>
-      <c r="F5" s="16" t="inlineStr">
+      <c r="F5" s="19" t="inlineStr">
         <is>
           <t>UAT</t>
         </is>
@@ -1123,10 +1182,10 @@
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>Quản lý Block</t>
-        </is>
-      </c>
-      <c r="D6" s="14" t="inlineStr">
+          <t>Quản lý section</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -1136,7 +1195,7 @@
           <t>SonLN11</t>
         </is>
       </c>
-      <c r="F6" s="16" t="inlineStr">
+      <c r="F6" s="19" t="inlineStr">
         <is>
           <t>UAT</t>
         </is>
@@ -1163,10 +1222,10 @@
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>Quản lý menu</t>
-        </is>
-      </c>
-      <c r="D7" s="14" t="inlineStr">
+          <t>Quản lý Block</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -1176,7 +1235,7 @@
           <t>SonLN11</t>
         </is>
       </c>
-      <c r="F7" s="16" t="inlineStr">
+      <c r="F7" s="19" t="inlineStr">
         <is>
           <t>UAT</t>
         </is>
@@ -1198,27 +1257,27 @@
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>[Web, CMS]</t>
+          <t>[CMS]</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>MENU (Cấp API Đa kênh &amp; Đồng bộ SPDV)</t>
-        </is>
-      </c>
-      <c r="D8" s="14" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Quản lý menu</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>ThuyTT104</t>
-        </is>
-      </c>
-      <c r="F8" s="17" t="inlineStr">
-        <is>
-          <t>DEV In Progress</t>
+          <t>SonLN11</t>
+        </is>
+      </c>
+      <c r="F8" s="19" t="inlineStr">
+        <is>
+          <t>UAT</t>
         </is>
       </c>
       <c r="G8" s="14" t="inlineStr">
@@ -1243,20 +1302,20 @@
       </c>
       <c r="C9" s="15" t="inlineStr">
         <is>
-          <t>Quản lý FAQ: Quy hoạch lại UI/UX &amp; luồng cấu hình danh sách/danh mục FAQ</t>
-        </is>
-      </c>
-      <c r="D9" s="14" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>Quản lý quảng cáo</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="E9" s="15" t="inlineStr">
         <is>
-          <t>SonLN11</t>
-        </is>
-      </c>
-      <c r="F9" s="18" t="inlineStr">
+          <t>LongNH156</t>
+        </is>
+      </c>
+      <c r="F9" s="20" t="inlineStr">
         <is>
           <t>Đang phân tích/Document</t>
         </is>
@@ -1278,27 +1337,27 @@
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>[CMS, Web]</t>
+          <t>[Web]</t>
         </is>
       </c>
       <c r="C10" s="15" t="inlineStr">
         <is>
-          <t>Quản lý quảng cáo</t>
-        </is>
-      </c>
-      <c r="D10" s="14" t="inlineStr">
+          <t>Report: Ghi nhận thông tin báo cáo phase 2 – bộ báo cáo chuẩn cho ĐKOL</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
       <c r="E10" s="15" t="inlineStr">
         <is>
-          <t>LongNH156</t>
-        </is>
-      </c>
-      <c r="F10" s="18" t="inlineStr">
-        <is>
-          <t>Đang phân tích/Document</t>
+          <t>ThuyTT104</t>
+        </is>
+      </c>
+      <c r="F10" s="17" t="inlineStr">
+        <is>
+          <t>DEV In Progress</t>
         </is>
       </c>
       <c r="G10" s="14" t="inlineStr">
@@ -1318,27 +1377,27 @@
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>[Web]</t>
+          <t>[Web, CMS]</t>
         </is>
       </c>
       <c r="C11" s="15" t="inlineStr">
         <is>
-          <t>Report: Ghi nhận thông tin báo cáo phase 2 – bộ báo cáo chuẩn cho ĐKOL</t>
-        </is>
-      </c>
-      <c r="D11" s="14" t="inlineStr">
+          <t>CMS config LDP Local – QT tạo LDP Local, SEO &amp; Schema</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
       <c r="E11" s="15" t="inlineStr">
         <is>
-          <t>ThuyTT104</t>
-        </is>
-      </c>
-      <c r="F11" s="17" t="inlineStr">
-        <is>
-          <t>DEV In Progress</t>
+          <t>ThuyTT104, LongNH156</t>
+        </is>
+      </c>
+      <c r="F11" s="20" t="inlineStr">
+        <is>
+          <t>Đang phân tích/Document</t>
         </is>
       </c>
       <c r="G11" s="14" t="inlineStr">
@@ -1358,25 +1417,25 @@
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>[Web, CMS]</t>
+          <t>[CMS, Web]</t>
         </is>
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
-          <t>CMS config LDP Local – QT tạo LDP Local, SEO &amp; Schema</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="inlineStr">
+          <t>Quản lý Breadcrumbs trên trang / Landing Page</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
       <c r="E12" s="15" t="inlineStr">
         <is>
-          <t>ThuyTT104, LongNH156</t>
-        </is>
-      </c>
-      <c r="F12" s="18" t="inlineStr">
+          <t>LongNH156, SonLN11</t>
+        </is>
+      </c>
+      <c r="F12" s="20" t="inlineStr">
         <is>
           <t>Đang phân tích/Document</t>
         </is>
@@ -1403,20 +1462,20 @@
       </c>
       <c r="C13" s="15" t="inlineStr">
         <is>
-          <t>Quản lý Breadcrumbs trên trang / Landing Page</t>
-        </is>
-      </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Quản lý FAQ: Quy hoạch lại UI/UX &amp; luồng cấu hình danh sách/danh mục FAQ</t>
+        </is>
+      </c>
+      <c r="D13" s="18" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="E13" s="15" t="inlineStr">
         <is>
-          <t>LongNH156, SonLN11</t>
-        </is>
-      </c>
-      <c r="F13" s="18" t="inlineStr">
+          <t>SonLN11</t>
+        </is>
+      </c>
+      <c r="F13" s="20" t="inlineStr">
         <is>
           <t>Đang phân tích/Document</t>
         </is>
@@ -1446,7 +1505,7 @@
           <t>Quản lý URL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
+      <c r="D14" s="18" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -1456,7 +1515,7 @@
           <t>LongNH156, ThuyTT104</t>
         </is>
       </c>
-      <c r="F14" s="18" t="inlineStr">
+      <c r="F14" s="20" t="inlineStr">
         <is>
           <t>Đang phân tích/Document</t>
         </is>
@@ -1478,27 +1537,27 @@
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>[Web]</t>
+          <t>[CMS, Web]</t>
         </is>
       </c>
       <c r="C15" s="15" t="inlineStr">
         <is>
-          <t>Luồng bán kèm PK (charm) trên website fpt.vn</t>
-        </is>
-      </c>
-      <c r="D15" s="14" t="inlineStr">
+          <t>Xây dựng thư viện section mở rộng cho tạo LDP kéo thả</t>
+        </is>
+      </c>
+      <c r="D15" s="18" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
       <c r="E15" s="15" t="inlineStr">
         <is>
-          <t>ThuyTT104</t>
-        </is>
-      </c>
-      <c r="F15" s="19" t="inlineStr">
-        <is>
-          <t>Chưa tiếp nhận</t>
+          <t>ThuyTT104, LongNH156</t>
+        </is>
+      </c>
+      <c r="F15" s="20" t="inlineStr">
+        <is>
+          <t>Đang phân tích/Document</t>
         </is>
       </c>
       <c r="G15" s="14" t="inlineStr">
@@ -1523,12 +1582,12 @@
       </c>
       <c r="C16" s="15" t="inlineStr">
         <is>
-          <t>Luồng quà tặng (Mũ bảo hiểm) trên website</t>
-        </is>
-      </c>
-      <c r="D16" s="14" t="inlineStr">
-        <is>
-          <t>P3</t>
+          <t>Luồng bán kèm PK (charm) trên website fpt.vn</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="E16" s="15" t="inlineStr">
@@ -1536,7 +1595,7 @@
           <t>ThuyTT104</t>
         </is>
       </c>
-      <c r="F16" s="19" t="inlineStr">
+      <c r="F16" s="21" t="inlineStr">
         <is>
           <t>Chưa tiếp nhận</t>
         </is>
@@ -1558,27 +1617,27 @@
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>[CMS, Web]</t>
+          <t>[Web]</t>
         </is>
       </c>
       <c r="C17" s="15" t="inlineStr">
         <is>
-          <t>Xây dựng thư viện section mở rộng cho tạo LDP kéo thả</t>
-        </is>
-      </c>
-      <c r="D17" s="14" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>Luồng quà tặng (Mũ bảo hiểm) trên website</t>
+        </is>
+      </c>
+      <c r="D17" s="22" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="E17" s="15" t="inlineStr">
         <is>
-          <t>ThuyTT104, LongNH156</t>
-        </is>
-      </c>
-      <c r="F17" s="18" t="inlineStr">
-        <is>
-          <t>Đang phân tích/Document</t>
+          <t>ThuyTT104</t>
+        </is>
+      </c>
+      <c r="F17" s="21" t="inlineStr">
+        <is>
+          <t>Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="G17" s="14" t="inlineStr">
@@ -1606,7 +1665,7 @@
           <t>[FMI Phase 4 | NBA] Phối hợp tích hợp Trigger Popup &amp; Web Push trên fpt.vn</t>
         </is>
       </c>
-      <c r="D18" s="14" t="inlineStr">
+      <c r="D18" s="23" t="inlineStr">
         <is>
           <t>P4</t>
         </is>
@@ -1616,7 +1675,7 @@
           <t>ThuyTT104</t>
         </is>
       </c>
-      <c r="F18" s="19" t="inlineStr">
+      <c r="F18" s="21" t="inlineStr">
         <is>
           <t>Chưa tiếp nhận</t>
         </is>
@@ -1646,7 +1705,7 @@
           <t>Luồng giỏ hàng trên kênh (Unified Cart)</t>
         </is>
       </c>
-      <c r="D19" s="14" t="inlineStr">
+      <c r="D19" s="16" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -1656,7 +1715,7 @@
           <t>ThuyTT104</t>
         </is>
       </c>
-      <c r="F19" s="18" t="inlineStr">
+      <c r="F19" s="20" t="inlineStr">
         <is>
           <t>Đang phân tích/Document</t>
         </is>
@@ -1686,7 +1745,7 @@
           <t>Quản lý tin tức</t>
         </is>
       </c>
-      <c r="D20" s="14" t="inlineStr">
+      <c r="D20" s="18" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -1696,7 +1755,7 @@
           <t>SonLN11</t>
         </is>
       </c>
-      <c r="F20" s="20" t="inlineStr">
+      <c r="F20" s="24" t="inlineStr">
         <is>
           <t>Đã tiếp nhận yêu cầu</t>
         </is>
@@ -1726,7 +1785,7 @@
           <t>Quản lý Profile Tác giả</t>
         </is>
       </c>
-      <c r="D21" s="14" t="inlineStr">
+      <c r="D21" s="18" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -1736,7 +1795,7 @@
           <t>SonLN11</t>
         </is>
       </c>
-      <c r="F21" s="20" t="inlineStr">
+      <c r="F21" s="24" t="inlineStr">
         <is>
           <t>Đã tiếp nhận yêu cầu</t>
         </is>
@@ -1763,12 +1822,12 @@
       </c>
       <c r="C22" s="15" t="inlineStr">
         <is>
-          <t>Các link chạy ads team Performance chạy ads - quy hoạch về CMS mới</t>
-        </is>
-      </c>
-      <c r="D22" s="14" t="inlineStr">
-        <is>
-          <t>P3</t>
+          <t>Trang LDP CSCA</t>
+        </is>
+      </c>
+      <c r="D22" s="18" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="E22" s="15" t="inlineStr">
@@ -1776,9 +1835,9 @@
           <t>ThuyTT104</t>
         </is>
       </c>
-      <c r="F22" s="18" t="inlineStr">
-        <is>
-          <t>Đang phân tích/Document</t>
+      <c r="F22" s="21" t="inlineStr">
+        <is>
+          <t>Chưa tiếp nhận</t>
         </is>
       </c>
       <c r="G22" s="14" t="inlineStr">
@@ -1798,17 +1857,17 @@
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>[CMS, Web]</t>
+          <t>[Web, CMS]</t>
         </is>
       </c>
       <c r="C23" s="15" t="inlineStr">
         <is>
-          <t>Bổ sung trang Combo Internet Camera</t>
-        </is>
-      </c>
-      <c r="D23" s="14" t="inlineStr">
-        <is>
-          <t>P4</t>
+          <t>Trang LDP Fcitizen</t>
+        </is>
+      </c>
+      <c r="D23" s="18" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="E23" s="15" t="inlineStr">
@@ -1816,7 +1875,7 @@
           <t>ThuyTT104</t>
         </is>
       </c>
-      <c r="F23" s="19" t="inlineStr">
+      <c r="F23" s="21" t="inlineStr">
         <is>
           <t>Chưa tiếp nhận</t>
         </is>
@@ -1843,20 +1902,20 @@
       </c>
       <c r="C24" s="15" t="inlineStr">
         <is>
-          <t>Trang LDP CSCA</t>
-        </is>
-      </c>
-      <c r="D24" s="14" t="inlineStr">
+          <t>Trang LDP Ngoại Hạng Anh (NHA)</t>
+        </is>
+      </c>
+      <c r="D24" s="18" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
       <c r="E24" s="15" t="inlineStr">
         <is>
-          <t>ThuyTT104</t>
-        </is>
-      </c>
-      <c r="F24" s="19" t="inlineStr">
+          <t>SonLN11</t>
+        </is>
+      </c>
+      <c r="F24" s="21" t="inlineStr">
         <is>
           <t>Chưa tiếp nhận</t>
         </is>
@@ -1883,20 +1942,20 @@
       </c>
       <c r="C25" s="15" t="inlineStr">
         <is>
-          <t>Trang LDP Fcitizen</t>
-        </is>
-      </c>
-      <c r="D25" s="14" t="inlineStr">
+          <t>Trang LDP NHA - Lịch thi đấu</t>
+        </is>
+      </c>
+      <c r="D25" s="18" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
       <c r="E25" s="15" t="inlineStr">
         <is>
-          <t>ThuyTT104</t>
-        </is>
-      </c>
-      <c r="F25" s="19" t="inlineStr">
+          <t>SonLN11</t>
+        </is>
+      </c>
+      <c r="F25" s="21" t="inlineStr">
         <is>
           <t>Chưa tiếp nhận</t>
         </is>
@@ -1923,10 +1982,10 @@
       </c>
       <c r="C26" s="15" t="inlineStr">
         <is>
-          <t>Trang LDP Ngoại Hạng Anh (NHA)</t>
-        </is>
-      </c>
-      <c r="D26" s="14" t="inlineStr">
+          <t>Trang LDP NHA - Bảng xếp hạng</t>
+        </is>
+      </c>
+      <c r="D26" s="18" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -1936,7 +1995,7 @@
           <t>SonLN11</t>
         </is>
       </c>
-      <c r="F26" s="19" t="inlineStr">
+      <c r="F26" s="21" t="inlineStr">
         <is>
           <t>Chưa tiếp nhận</t>
         </is>
@@ -1963,10 +2022,10 @@
       </c>
       <c r="C27" s="15" t="inlineStr">
         <is>
-          <t>Trang LDP NHA - Lịch thi đấu</t>
-        </is>
-      </c>
-      <c r="D27" s="14" t="inlineStr">
+          <t>Trang LDP NHA - SA</t>
+        </is>
+      </c>
+      <c r="D27" s="18" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -1976,7 +2035,7 @@
           <t>SonLN11</t>
         </is>
       </c>
-      <c r="F27" s="19" t="inlineStr">
+      <c r="F27" s="21" t="inlineStr">
         <is>
           <t>Chưa tiếp nhận</t>
         </is>
@@ -2003,22 +2062,22 @@
       </c>
       <c r="C28" s="15" t="inlineStr">
         <is>
-          <t>Trang LDP NHA - Bảng xếp hạng</t>
-        </is>
-      </c>
-      <c r="D28" s="14" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>Các link chạy ads team Performance chạy ads - quy hoạch về CMS mới</t>
+        </is>
+      </c>
+      <c r="D28" s="22" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="E28" s="15" t="inlineStr">
         <is>
-          <t>SonLN11</t>
-        </is>
-      </c>
-      <c r="F28" s="19" t="inlineStr">
-        <is>
-          <t>Chưa tiếp nhận</t>
+          <t>ThuyTT104</t>
+        </is>
+      </c>
+      <c r="F28" s="20" t="inlineStr">
+        <is>
+          <t>Đang phân tích/Document</t>
         </is>
       </c>
       <c r="G28" s="14" t="inlineStr">
@@ -2038,25 +2097,25 @@
       </c>
       <c r="B29" s="14" t="inlineStr">
         <is>
-          <t>[Web, CMS]</t>
+          <t>[CMS, Web]</t>
         </is>
       </c>
       <c r="C29" s="15" t="inlineStr">
         <is>
-          <t>Trang LDP NHA - SA</t>
-        </is>
-      </c>
-      <c r="D29" s="14" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>Bổ sung trang Combo Internet Camera</t>
+        </is>
+      </c>
+      <c r="D29" s="23" t="inlineStr">
+        <is>
+          <t>P4</t>
         </is>
       </c>
       <c r="E29" s="15" t="inlineStr">
         <is>
-          <t>SonLN11</t>
-        </is>
-      </c>
-      <c r="F29" s="19" t="inlineStr">
+          <t>ThuyTT104</t>
+        </is>
+      </c>
+      <c r="F29" s="21" t="inlineStr">
         <is>
           <t>Chưa tiếp nhận</t>
         </is>

</xml_diff>

<commit_message>
fix(roadmap): chia chuan tien do 8 phan bang nhau (12.5% moi nac) theo dung 8 trang thai he thong va dong bo excel
</commit_message>
<xml_diff>
--- a/thuyttdoc/Roadmap_Website_CMS_Q4_2026.xlsx
+++ b/thuyttdoc/Roadmap_Website_CMS_Q4_2026.xlsx
@@ -727,7 +727,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Lộ trình thực thi 26 User Stories | Sắp xếp P1 -&gt; P2 -&gt; P3 -&gt; P4 trong cùng 1 mốc thời gian | Chuẩn bảng màu trạng thái</t>
+          <t>Lộ trình thực thi 26 User Stories | Tiến độ chuẩn 8 phần bằng nhau (12.5%/trạng thái) | Ưu tiên P1 -&gt; P4</t>
         </is>
       </c>
     </row>
@@ -1029,23 +1029,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="56" customWidth="1" min="3" max="3"/>
+    <col width="54" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DANH SÁCH CHI TIẾT 26 USER STORIES QUÝ 4/2026 (SẮP XẾP ƯU TIÊN P1 -&gt; P4 THEO MỐC THỜI GIAN)</t>
+          <t>DANH SÁCH CHI TIẾT 26 USER STORIES QUÝ 4/2026 (CHIA ĐỦ 8 PHẦN BẰNG NHAU THEO TRẠNG THÁI)</t>
         </is>
       </c>
     </row>
@@ -1082,10 +1083,15 @@
       </c>
       <c r="G3" s="13" t="inlineStr">
         <is>
+          <t>Tiến độ (8 nấc)</t>
+        </is>
+      </c>
+      <c r="H3" s="13" t="inlineStr">
+        <is>
           <t>Timeline mong muốn</t>
         </is>
       </c>
-      <c r="H3" s="13" t="inlineStr">
+      <c r="I3" s="13" t="inlineStr">
         <is>
           <t>Ghi chú tiến trình</t>
         </is>
@@ -1122,10 +1128,15 @@
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
+          <t>Nấc 5/8 (62.5%)</t>
+        </is>
+      </c>
+      <c r="H4" s="14" t="inlineStr">
+        <is>
           <t>Tháng 10</t>
         </is>
       </c>
-      <c r="H4" s="15" t="inlineStr">
+      <c r="I4" s="15" t="inlineStr">
         <is>
           <t>Hoàn thành trong tháng</t>
         </is>
@@ -1162,10 +1173,15 @@
       </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
+          <t>Nấc 6/8 (75%)</t>
+        </is>
+      </c>
+      <c r="H5" s="14" t="inlineStr">
+        <is>
           <t>Tháng 10</t>
         </is>
       </c>
-      <c r="H5" s="15" t="inlineStr">
+      <c r="I5" s="15" t="inlineStr">
         <is>
           <t>Hoàn thành trong tháng</t>
         </is>
@@ -1202,10 +1218,15 @@
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
+          <t>Nấc 6/8 (75%)</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
           <t>Tháng 10</t>
         </is>
       </c>
-      <c r="H6" s="15" t="inlineStr">
+      <c r="I6" s="15" t="inlineStr">
         <is>
           <t>Hoàn thành trong tháng</t>
         </is>
@@ -1242,10 +1263,15 @@
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
+          <t>Nấc 6/8 (75%)</t>
+        </is>
+      </c>
+      <c r="H7" s="14" t="inlineStr">
+        <is>
           <t>Tháng 10</t>
         </is>
       </c>
-      <c r="H7" s="15" t="inlineStr">
+      <c r="I7" s="15" t="inlineStr">
         <is>
           <t>Hoàn thành trong tháng</t>
         </is>
@@ -1282,10 +1308,15 @@
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
+          <t>Nấc 6/8 (75%)</t>
+        </is>
+      </c>
+      <c r="H8" s="14" t="inlineStr">
+        <is>
           <t>Tháng 10</t>
         </is>
       </c>
-      <c r="H8" s="15" t="inlineStr">
+      <c r="I8" s="15" t="inlineStr">
         <is>
           <t>Hoàn thành trong tháng</t>
         </is>
@@ -1322,10 +1353,15 @@
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
+          <t>Nấc 3/8 (37.5%)</t>
+        </is>
+      </c>
+      <c r="H9" s="14" t="inlineStr">
+        <is>
           <t>Tháng 10 - Tháng 11</t>
         </is>
       </c>
-      <c r="H9" s="15" t="inlineStr">
+      <c r="I9" s="15" t="inlineStr">
         <is>
           <t>Vắt từ T10 sang T11</t>
         </is>
@@ -1362,10 +1398,15 @@
       </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
+          <t>Nấc 5/8 (62.5%)</t>
+        </is>
+      </c>
+      <c r="H10" s="14" t="inlineStr">
+        <is>
           <t>Tháng 10 - Tháng 11</t>
         </is>
       </c>
-      <c r="H10" s="15" t="inlineStr">
+      <c r="I10" s="15" t="inlineStr">
         <is>
           <t>Vắt từ T10 sang T11</t>
         </is>
@@ -1402,10 +1443,15 @@
       </c>
       <c r="G11" s="14" t="inlineStr">
         <is>
+          <t>Nấc 3/8 (37.5%)</t>
+        </is>
+      </c>
+      <c r="H11" s="14" t="inlineStr">
+        <is>
           <t>Tháng 10 - Tháng 11</t>
         </is>
       </c>
-      <c r="H11" s="15" t="inlineStr">
+      <c r="I11" s="15" t="inlineStr">
         <is>
           <t>Vắt từ T10 sang T11</t>
         </is>
@@ -1442,10 +1488,15 @@
       </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
+          <t>Nấc 3/8 (37.5%)</t>
+        </is>
+      </c>
+      <c r="H12" s="14" t="inlineStr">
+        <is>
           <t>Tháng 10 - Tháng 11</t>
         </is>
       </c>
-      <c r="H12" s="15" t="inlineStr">
+      <c r="I12" s="15" t="inlineStr">
         <is>
           <t>Vắt từ T10 sang T11</t>
         </is>
@@ -1482,10 +1533,15 @@
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
+          <t>Nấc 3/8 (37.5%)</t>
+        </is>
+      </c>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
           <t>Tháng 10 - Tháng 11</t>
         </is>
       </c>
-      <c r="H13" s="15" t="inlineStr">
+      <c r="I13" s="15" t="inlineStr">
         <is>
           <t>Vắt từ T10 sang T11</t>
         </is>
@@ -1522,10 +1578,15 @@
       </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
+          <t>Nấc 3/8 (37.5%)</t>
+        </is>
+      </c>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
           <t>Tháng 11</t>
         </is>
       </c>
-      <c r="H14" s="15" t="inlineStr">
+      <c r="I14" s="15" t="inlineStr">
         <is>
           <t>Hoàn thành trong tháng</t>
         </is>
@@ -1562,10 +1623,15 @@
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
+          <t>Nấc 3/8 (37.5%)</t>
+        </is>
+      </c>
+      <c r="H15" s="14" t="inlineStr">
+        <is>
           <t>Tháng 11</t>
         </is>
       </c>
-      <c r="H15" s="15" t="inlineStr">
+      <c r="I15" s="15" t="inlineStr">
         <is>
           <t>Hoàn thành trong tháng</t>
         </is>
@@ -1602,10 +1668,15 @@
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
+          <t>Nấc 1/8 (12.5%)</t>
+        </is>
+      </c>
+      <c r="H16" s="14" t="inlineStr">
+        <is>
           <t>Tháng 11</t>
         </is>
       </c>
-      <c r="H16" s="15" t="inlineStr">
+      <c r="I16" s="15" t="inlineStr">
         <is>
           <t>Hoàn thành trong tháng</t>
         </is>
@@ -1642,10 +1713,15 @@
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
+          <t>Nấc 1/8 (12.5%)</t>
+        </is>
+      </c>
+      <c r="H17" s="14" t="inlineStr">
+        <is>
           <t>Tháng 11</t>
         </is>
       </c>
-      <c r="H17" s="15" t="inlineStr">
+      <c r="I17" s="15" t="inlineStr">
         <is>
           <t>Hoàn thành trong tháng</t>
         </is>
@@ -1682,10 +1758,15 @@
       </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
+          <t>Nấc 1/8 (12.5%)</t>
+        </is>
+      </c>
+      <c r="H18" s="14" t="inlineStr">
+        <is>
           <t>Tháng 11</t>
         </is>
       </c>
-      <c r="H18" s="15" t="inlineStr">
+      <c r="I18" s="15" t="inlineStr">
         <is>
           <t>Hoàn thành trong tháng</t>
         </is>
@@ -1722,10 +1803,15 @@
       </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
+          <t>Nấc 3/8 (37.5%)</t>
+        </is>
+      </c>
+      <c r="H19" s="14" t="inlineStr">
+        <is>
           <t>Tháng 11 - Tháng 12</t>
         </is>
       </c>
-      <c r="H19" s="15" t="inlineStr">
+      <c r="I19" s="15" t="inlineStr">
         <is>
           <t>Vắt từ T11 sang T12</t>
         </is>
@@ -1762,10 +1848,15 @@
       </c>
       <c r="G20" s="14" t="inlineStr">
         <is>
+          <t>Nấc 2/8 (25%)</t>
+        </is>
+      </c>
+      <c r="H20" s="14" t="inlineStr">
+        <is>
           <t>Tháng 11 - Tháng 12</t>
         </is>
       </c>
-      <c r="H20" s="15" t="inlineStr">
+      <c r="I20" s="15" t="inlineStr">
         <is>
           <t>Vắt từ T11 sang T12</t>
         </is>
@@ -1802,10 +1893,15 @@
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
+          <t>Nấc 2/8 (25%)</t>
+        </is>
+      </c>
+      <c r="H21" s="14" t="inlineStr">
+        <is>
           <t>Tháng 11 - Tháng 12</t>
         </is>
       </c>
-      <c r="H21" s="15" t="inlineStr">
+      <c r="I21" s="15" t="inlineStr">
         <is>
           <t>Vắt từ T11 sang T12</t>
         </is>
@@ -1842,10 +1938,15 @@
       </c>
       <c r="G22" s="14" t="inlineStr">
         <is>
+          <t>Nấc 1/8 (12.5%)</t>
+        </is>
+      </c>
+      <c r="H22" s="14" t="inlineStr">
+        <is>
           <t>Tháng 12</t>
         </is>
       </c>
-      <c r="H22" s="15" t="inlineStr">
+      <c r="I22" s="15" t="inlineStr">
         <is>
           <t>Hoàn thành trong tháng</t>
         </is>
@@ -1882,10 +1983,15 @@
       </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
+          <t>Nấc 1/8 (12.5%)</t>
+        </is>
+      </c>
+      <c r="H23" s="14" t="inlineStr">
+        <is>
           <t>Tháng 12</t>
         </is>
       </c>
-      <c r="H23" s="15" t="inlineStr">
+      <c r="I23" s="15" t="inlineStr">
         <is>
           <t>Hoàn thành trong tháng</t>
         </is>
@@ -1922,10 +2028,15 @@
       </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
+          <t>Nấc 1/8 (12.5%)</t>
+        </is>
+      </c>
+      <c r="H24" s="14" t="inlineStr">
+        <is>
           <t>Tháng 12</t>
         </is>
       </c>
-      <c r="H24" s="15" t="inlineStr">
+      <c r="I24" s="15" t="inlineStr">
         <is>
           <t>Hoàn thành trong tháng</t>
         </is>
@@ -1962,10 +2073,15 @@
       </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
+          <t>Nấc 1/8 (12.5%)</t>
+        </is>
+      </c>
+      <c r="H25" s="14" t="inlineStr">
+        <is>
           <t>Tháng 12</t>
         </is>
       </c>
-      <c r="H25" s="15" t="inlineStr">
+      <c r="I25" s="15" t="inlineStr">
         <is>
           <t>Hoàn thành trong tháng</t>
         </is>
@@ -2002,10 +2118,15 @@
       </c>
       <c r="G26" s="14" t="inlineStr">
         <is>
+          <t>Nấc 1/8 (12.5%)</t>
+        </is>
+      </c>
+      <c r="H26" s="14" t="inlineStr">
+        <is>
           <t>Tháng 12</t>
         </is>
       </c>
-      <c r="H26" s="15" t="inlineStr">
+      <c r="I26" s="15" t="inlineStr">
         <is>
           <t>Hoàn thành trong tháng</t>
         </is>
@@ -2042,10 +2163,15 @@
       </c>
       <c r="G27" s="14" t="inlineStr">
         <is>
+          <t>Nấc 1/8 (12.5%)</t>
+        </is>
+      </c>
+      <c r="H27" s="14" t="inlineStr">
+        <is>
           <t>Tháng 12</t>
         </is>
       </c>
-      <c r="H27" s="15" t="inlineStr">
+      <c r="I27" s="15" t="inlineStr">
         <is>
           <t>Hoàn thành trong tháng</t>
         </is>
@@ -2082,10 +2208,15 @@
       </c>
       <c r="G28" s="14" t="inlineStr">
         <is>
+          <t>Nấc 3/8 (37.5%)</t>
+        </is>
+      </c>
+      <c r="H28" s="14" t="inlineStr">
+        <is>
           <t>Tháng 12</t>
         </is>
       </c>
-      <c r="H28" s="15" t="inlineStr">
+      <c r="I28" s="15" t="inlineStr">
         <is>
           <t>Hoàn thành trong tháng</t>
         </is>
@@ -2122,10 +2253,15 @@
       </c>
       <c r="G29" s="14" t="inlineStr">
         <is>
+          <t>Nấc 1/8 (12.5%)</t>
+        </is>
+      </c>
+      <c r="H29" s="14" t="inlineStr">
+        <is>
           <t>Tháng 12</t>
         </is>
       </c>
-      <c r="H29" s="15" t="inlineStr">
+      <c r="I29" s="15" t="inlineStr">
         <is>
           <t>Hoàn thành trong tháng</t>
         </is>

</xml_diff>

<commit_message>
refactor(roadmap): bo sprint, bo subtitle header, cat gon footer theo yeu cau
</commit_message>
<xml_diff>
--- a/thuyttdoc/Roadmap_Website_CMS_Q4_2026.xlsx
+++ b/thuyttdoc/Roadmap_Website_CMS_Q4_2026.xlsx
@@ -750,24 +750,24 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Lộ trình thực thi 26 User Stories | Cập nhật đồng bộ Backlog mới nhất | Tiến độ chuẩn 8 phần bằng nhau | Ưu tiên P1 -&gt; P4</t>
+          <t>Roadmap thực thi Website &amp; CMS FPT.vn (Q4/2026)</t>
         </is>
       </c>
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>THÁNG 10 / 2026 (Sprint 19 - 20)</t>
+          <t>THÁNG 10 / 2026</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>THÁNG 11 / 2026 (Sprint 21 - 22)</t>
+          <t>THÁNG 11 / 2026</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>THÁNG 12 / 2026 (Sprint 23 - 24)</t>
+          <t>THÁNG 12 / 2026</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DANH SÁCH CHI TIẾT 26 USER STORIES QUÝ 4/2026 (ĐỒNG BỘ BACKLOG MỚI NHẤT)</t>
+          <t>DANH SÁCH CHI TIẾT 26 USER STORIES QUÝ 4/2026</t>
         </is>
       </c>
     </row>

</xml_diff>